<commit_message>
related_hadiths data label fixed
</commit_message>
<xml_diff>
--- a/SINGLE HADITH CONTENT/BOOK WISE FINAL UPDATED CONTENT/BN/BN_DHAIF HADIS SIRIJ.xlsx
+++ b/SINGLE HADITH CONTENT/BOOK WISE FINAL UPDATED CONTENT/BN/BN_DHAIF HADIS SIRIJ.xlsx
@@ -60,8 +60,12 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -488,7 +492,7 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | বিবেক নিয়ে বাতিল হাদিসের সতর্কতা","description":"$book_name$ $hadith_number$ - $chapter_name$. দ্বীন হচ্ছে বিবেক—এ কথাটি হাদিস হিসেবে বাতিল; তাই যাচাই ছাড়া রাসূল صلى الله عليه وسلم-এর নামে বলা উচিত নয়।"},"heading":{"title":"বিবেক নিয়ে বাতিল হাদিস: দ্বীন হচ্ছে বিবেক কথার হুকুম","description":"এই বর্ণনায় বলা হয়েছে, “দ্বীন হচ্ছে বিবেক, যার দ্বীন নেই তার কোন বিবেক নেই।” কিন্তু প্রদত্ত আলোচনায় পরিষ্কারভাবে বলা হয়েছে, হাদিসটি বাতিল। এখানে মূল বিষয় হলো জাল ও বাতিল হাদিস থেকে সতর্ক থাকা। মানুষের কাছে কোনো কথা সুন্দর বা গভীর মনে হলেই তা রাসূল صلى الله عليه وسلم-এর কথা হয়ে যায় না। এই বর্ণনার সনদে বিশর ইবনু গালিব নামের একজন অপরিচিত বর্ণনাকারীর সমস্যা উল্লেখ করা হয়েছে। আরও বলা হয়েছে, বিবেকের ফজিলত নিয়ে বর্ণিত অনেক কথাই দুর্বল বা জাল। তাই “বিবেকের ফজিলত হাদিস” বা “দ্বীন হচ্ছে বিবেক” নামে প্রচলিত কথাগুলো যাচাই ছাড়া শেয়ার করা ঠিক নয়। একজন মুসলিমের জন্য নিরাপদ পথ হলো—সহীহ হাদিস গ্রহণ করা এবং দুর্বল, বাতিল বা বানোয়াট বর্ণনাকে নবী صلى الله عليه وسلم-এর নামে না বলা।"},"teachings":["সুন্দর শোনালেই কোনো কথাকে হাদিস বলা ঠিক নয়।","বর্ণনাকারীর অবস্থা হাদিস যাচাইয়ের বড় বিষয়।","বিবেকের ফজিলত বিষয়ে বর্ণিত সব কথাকে সহীহ মনে করা যাবে না।","রাসূল صلى الله عليه وسلم-এর নামে কথা বলার আগে নির্ভরযোগ্য উৎস দেখা জরুরি।"],"related_hadiths":[{"id":"107","book_id":"1","label":"Sahih Bukhari"},{"id":"3","book_id":"2","label":"Sahih Muslim"},{"id":"35","book_id":"6","label":"Sunan Ibn Majah"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | বিবেক নিয়ে বাতিল হাদিসের সতর্কতা","description":"$book_name$ $hadith_number$ - $chapter_name$. দ্বীন হচ্ছে বিবেক—এ কথাটি হাদিস হিসেবে বাতিল; তাই যাচাই ছাড়া রাসূল صلى الله عليه وسلم-এর নামে বলা উচিত নয়।"},"heading":{"title":"বিবেক নিয়ে বাতিল হাদিস: দ্বীন হচ্ছে বিবেক কথার হুকুম","description":"এই বর্ণনায় বলা হয়েছে, “দ্বীন হচ্ছে বিবেক, যার দ্বীন নেই তার কোন বিবেক নেই।” কিন্তু প্রদত্ত আলোচনায় পরিষ্কারভাবে বলা হয়েছে, হাদিসটি বাতিল। এখানে মূল বিষয় হলো জাল ও বাতিল হাদিস থেকে সতর্ক থাকা। মানুষের কাছে কোনো কথা সুন্দর বা গভীর মনে হলেই তা রাসূল صلى الله عليه وسلم-এর কথা হয়ে যায় না। এই বর্ণনার সনদে বিশর ইবনু গালিব নামের একজন অপরিচিত বর্ণনাকারীর সমস্যা উল্লেখ করা হয়েছে। আরও বলা হয়েছে, বিবেকের ফজিলত নিয়ে বর্ণিত অনেক কথাই দুর্বল বা জাল। তাই “বিবেকের ফজিলত হাদিস” বা “দ্বীন হচ্ছে বিবেক” নামে প্রচলিত কথাগুলো যাচাই ছাড়া শেয়ার করা ঠিক নয়। একজন মুসলিমের জন্য নিরাপদ পথ হলো—সহীহ হাদিস গ্রহণ করা এবং দুর্বল, বাতিল বা বানোয়াট বর্ণনাকে নবী صلى الله عليه وسلم-এর নামে না বলা।"},"teachings":["সুন্দর শোনালেই কোনো কথাকে হাদিস বলা ঠিক নয়।","বর্ণনাকারীর অবস্থা হাদিস যাচাইয়ের বড় বিষয়।","বিবেকের ফজিলত বিষয়ে বর্ণিত সব কথাকে সহীহ মনে করা যাবে না।","রাসূল صلى الله عليه وسلم-এর নামে কথা বলার আগে নির্ভরযোগ্য উৎস দেখা জরুরি।"],"related_hadiths":[{"id":"107","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"3","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"35","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
         </is>
       </c>
       <c r="E2" s="4" t="n"/>
@@ -511,7 +515,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | হালাল রুজি নিয়ে জাল হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. হালাল রুজির জন্য পরিশ্রমের কথা ভালো হলেও এই নির্দিষ্ট বর্ণনাটি জাল বলা হয়েছে।"},"heading":{"title":"হালাল রুজির জন্য পরিশ্রম: এই বর্ণনাটি জাল","description":"এই বর্ণনায় বলা হয়েছে, আল্লাহ তাঁর বান্দাকে হালাল রুজি অন্বেষণে পরিশ্রান্ত অবস্থায় দেখতে ভালোবাসেন। কথাটি অর্থের দিক থেকে অনেকের কাছে সুন্দর লাগে। কিন্তু প্রদত্ত আলোচনায় স্পষ্ট বলা হয়েছে, হাদিসটি জাল। এর সনদে মুহাম্মাদ ইবনু সাহাল আল-আত্তার নামে একজন বর্ণনাকারী আছেন, যাকে দারাকুতনী হাদিস জালকারী বলেছেন। তাই “হালাল রুজির জন্য পরিশ্রম হাদিস” নামে এই নির্দিষ্ট বাক্য ছড়ানো ঠিক নয়। হালাল উপার্জন অবশ্যই গুরুত্বপূর্ণ আমল—এ কথা অন্য দলিল থেকে জানা যায়। কিন্তু কোনো জাল বর্ণনা দিয়ে হালাল রুজির মর্যাদা বোঝানো উচিত নয়। দ্বীনের কথা বলার সময় ভালো উদ্দেশ্য যথেষ্ট নয়; সঠিক দলিলও দরকার। এতে হাদিসের সম্মান রক্ষা হয় এবং মানুষ ভুল তথ্য থেকে বাঁচে।"},"teachings":["হালাল রুজির গুরুত্ব বোঝাতে জাল হাদিস ব্যবহার করা ঠিক নয়।","সনদে জালকারী থাকলে বর্ণনা গ্রহণযোগ্য থাকে না।","ভালো অর্থ থাকলেও হাদিসের প্রমাণ আলাদা করে যাচাই করতে হয়।","ধর্মীয় পোস্ট শেয়ার করার আগে উৎস দেখা জরুরি।"],"related_hadiths":[{"id":"2072","book_id":"1","label":"Sahih Bukhari"},{"id":"2137","book_id":"6","label":"Sunan Ibn Majah"},{"id":"2344","book_id":"5","label":"Jami at-Tirmidhi"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | হালাল রুজি নিয়ে জাল হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. হালাল রুজির জন্য পরিশ্রমের কথা ভালো হলেও এই নির্দিষ্ট বর্ণনাটি জাল বলা হয়েছে।"},"heading":{"title":"হালাল রুজির জন্য পরিশ্রম: এই বর্ণনাটি জাল","description":"এই বর্ণনায় বলা হয়েছে, আল্লাহ তাঁর বান্দাকে হালাল রুজি অন্বেষণে পরিশ্রান্ত অবস্থায় দেখতে ভালোবাসেন। কথাটি অর্থের দিক থেকে অনেকের কাছে সুন্দর লাগে। কিন্তু প্রদত্ত আলোচনায় স্পষ্ট বলা হয়েছে, হাদিসটি জাল। এর সনদে মুহাম্মাদ ইবনু সাহাল আল-আত্তার নামে একজন বর্ণনাকারী আছেন, যাকে দারাকুতনী হাদিস জালকারী বলেছেন। তাই “হালাল রুজির জন্য পরিশ্রম হাদিস” নামে এই নির্দিষ্ট বাক্য ছড়ানো ঠিক নয়। হালাল উপার্জন অবশ্যই গুরুত্বপূর্ণ আমল—এ কথা অন্য দলিল থেকে জানা যায়। কিন্তু কোনো জাল বর্ণনা দিয়ে হালাল রুজির মর্যাদা বোঝানো উচিত নয়। দ্বীনের কথা বলার সময় ভালো উদ্দেশ্য যথেষ্ট নয়; সঠিক দলিলও দরকার। এতে হাদিসের সম্মান রক্ষা হয় এবং মানুষ ভুল তথ্য থেকে বাঁচে।"},"teachings":["হালাল রুজির গুরুত্ব বোঝাতে জাল হাদিস ব্যবহার করা ঠিক নয়।","সনদে জালকারী থাকলে বর্ণনা গ্রহণযোগ্য থাকে না।","ভালো অর্থ থাকলেও হাদিসের প্রমাণ আলাদা করে যাচাই করতে হয়।","ধর্মীয় পোস্ট শেয়ার করার আগে উৎস দেখা জরুরি।"],"related_hadiths":[{"id":"2072","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2137","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"},{"id":"2344","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"}]}</t>
         </is>
       </c>
       <c r="E3" s="4" t="n"/>
@@ -534,7 +538,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | উত্তম কর্ম মন্দ কর্ম হয়ে যায় কথার বাতিলতা","description":"$book_name$ $hadith_number$ - $chapter_name$. সদাচরণকারীর উত্তম কাজ নৈকট্যপ্রাপ্তদের মন্দ কাজ—এ কথার কোনো হাদিসি ভিত্তি নেই; অর্থও সঠিক নয় বলা হয়েছে।"},"heading":{"title":"সদাচরণকারীর উত্তম কাজ মন্দ কাজ? বাতিল ও ভিত্তিহীন উক্তির তাহকীক","description":"এই বর্ণনায় বলা হয়েছে, সদাচরণকারীদের উত্তম কর্মগুলো নৈকট্য অর্জনকারীদের মন্দ কর্ম। প্রদত্ত তাহকীক অনুযায়ী এটি বাতিল এবং এর কোনো ভিত্তি নেই। গাযালী আল-ইহইয়া গ্রন্থে এ ভাষায় উল্লেখ করেছেন, কিন্তু আলোচনায় বলা হয়েছে, তিনি বাহ্যিকভাবে এটিকে হাদিস হিসেবে উল্লেখ করেননি। বরং এটি আবূ সাঈদ আল-খাররাজ আস-সূফীর কথা হিসেবে ইঙ্গিত করা হয়েছে। পরে কেউ কেউ এটিকে হাদিস ভেবে নিয়েছেন, কিন্তু তা সঠিক নয়। আলবানী আরও বলেছেন, অর্থের দিক দিয়েও এটি ঠিক নয়; কারণ ভালো কাজ কখনো মন্দ কাজে পরিণত হতে পারে না। এখানে মূল শিক্ষা হলো সুফি উক্তি, নৈতিক বাক্য ও হাদিসের পার্থক্য বোঝা। কোনো গভীর শোনানো বাক্যকে রাসূলের হাদিস বানানো যায় না।"},"teachings":["কোনো আলেম বা সুফির উক্তি হাদিস নয়, যদি সনদে প্রমাণ না থাকে।","গভীর শোনানো কথা হলেও তা রাসূলের নামে বলা যাবে না।","ভালো কাজকে মন্দ কাজ বলা অর্থগতভাবে সতর্কতার দাবি রাখে।","হাদিস, উক্তি ও ব্যাখ্যার পার্থক্য জানা দরকার।"],"related_hadiths":[{"id":"107","book_id":"1","label":"Sahih Bukhari"},{"id":"5","book_id":"2","label":"Sahih Muslim"},{"id":"1907","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | উত্তম কর্ম মন্দ কর্ম হয়ে যায় কথার বাতিলতা","description":"$book_name$ $hadith_number$ - $chapter_name$. সদাচরণকারীর উত্তম কাজ নৈকট্যপ্রাপ্তদের মন্দ কাজ—এ কথার কোনো হাদিসি ভিত্তি নেই; অর্থও সঠিক নয় বলা হয়েছে।"},"heading":{"title":"সদাচরণকারীর উত্তম কাজ মন্দ কাজ? বাতিল ও ভিত্তিহীন উক্তির তাহকীক","description":"এই বর্ণনায় বলা হয়েছে, সদাচরণকারীদের উত্তম কর্মগুলো নৈকট্য অর্জনকারীদের মন্দ কর্ম। প্রদত্ত তাহকীক অনুযায়ী এটি বাতিল এবং এর কোনো ভিত্তি নেই। গাযালী আল-ইহইয়া গ্রন্থে এ ভাষায় উল্লেখ করেছেন, কিন্তু আলোচনায় বলা হয়েছে, তিনি বাহ্যিকভাবে এটিকে হাদিস হিসেবে উল্লেখ করেননি। বরং এটি আবূ সাঈদ আল-খাররাজ আস-সূফীর কথা হিসেবে ইঙ্গিত করা হয়েছে। পরে কেউ কেউ এটিকে হাদিস ভেবে নিয়েছেন, কিন্তু তা সঠিক নয়। আলবানী আরও বলেছেন, অর্থের দিক দিয়েও এটি ঠিক নয়; কারণ ভালো কাজ কখনো মন্দ কাজে পরিণত হতে পারে না। এখানে মূল শিক্ষা হলো সুফি উক্তি, নৈতিক বাক্য ও হাদিসের পার্থক্য বোঝা। কোনো গভীর শোনানো বাক্যকে রাসূলের হাদিস বানানো যায় না।"},"teachings":["কোনো আলেম বা সুফির উক্তি হাদিস নয়, যদি সনদে প্রমাণ না থাকে।","গভীর শোনানো কথা হলেও তা রাসূলের নামে বলা যাবে না।","ভালো কাজকে মন্দ কাজ বলা অর্থগতভাবে সতর্কতার দাবি রাখে।","হাদিস, উক্তি ও ব্যাখ্যার পার্থক্য জানা দরকার।"],"related_hadiths":[{"id":"107","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"5","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"1907","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E4" s="4" t="n"/>
@@ -557,7 +561,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ভুলে যাওয়ার হাদিস যাচাই ও সহিহ বর্ণনা","description":"$book_name$ $hadith_number$ - $chapter_name$. নবীজি ভুলে যান না—এ দাবির ভিত্তিহীনতা ও সহিহ বর্ণনার আলোকে হাদিস যাচাইয়ের শিক্ষা জানুন।"},"heading":{"title":"ভুলে যাওয়ার হাদিস যাচাই: ভিত্তিহীন বর্ণনা ও সহিহ হাদিসের শিক্ষা","description":"এই বর্ণনায় বলা হয়েছে, “আমি ভুলিনা, কিন্তু আমাকে ভুলিয়ে দেয়া হয় যাতে করে আমি বিধান রচনা করতে পারি।” প্রদত্ত তথ্য অনুযায়ী, এটি বাতিল এবং এর কোনো ভিত্তি নেই। তাই এই কথাকে নবী সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লামের হাদিস হিসেবে প্রচার করা ঠিক নয়। এখানে হাদিস যাচাইয়ের বিষয়টি খুব পরিষ্কারভাবে সামনে আসে। শুধু কোনো বিখ্যাত বইয়ে কোনো কথা পাওয়া গেলেই তা সহিহ হাদিস হয়ে যায় না। প্রদত্ত লেখায় দেখা যায়, গাযালী এটি উল্লেখ করেছেন, কিন্তু হাফিয ইরাকী, ইবনু আব্দিল বার, হামযা আল-কিনানী, আবূ তাহের আনমাতী ও হাফিয ইবনু হাজার—তাঁরা এর ভিত্তি নিয়ে কঠোর কথা বলেছেন। একই সঙ্গে সহিহ বুখারী ও সহিহ মুসলিমের বর্ণনায় এসেছে যে, নবীজি মানুষ হিসেবে ভুলে যেতে পারেন এবং ভুল হলে সাহাবীদের স্মরণ করিয়ে দিতে বলেছেন। তাই মূল শিক্ষা হলো, জাল হাদিস বা ভিত্তিহীন বর্ণনা থেকে সতর্ক থাকা এবং সহিহ বর্ণনার আলোকে কথা বলা।"},"teachings":["কোনো বর্ণনাকে হাদিস বলার আগে তার ভিত্তি ও সনদ যাচাই করা দরকার।","ভিত্তিহীন কথা নবীজি সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লামের নামে প্রচার করা উচিত নয়।","সহিহ বর্ণনা অনুযায়ী, সালাতে ভুল হলে স্মরণ করিয়ে দেওয়া ও সাহু সিজদার শিক্ষা রয়েছে।","বিখ্যাত গ্রন্থে উল্লেখ থাকলেও কোনো কথা সহিহ প্রমাণ না হলে সতর্ক থাকা দরকার।"],"related_hadiths":[{"id":"401","book_id":"1","label":"Sahih Bukhari"},{"id":"1161","book_id":"2","label":"Sahih Muslim"},{"id":"1244","book_id":"3","label":"Sunan an-Nasai"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ভুলে যাওয়ার হাদিস যাচাই ও সহিহ বর্ণনা","description":"$book_name$ $hadith_number$ - $chapter_name$. নবীজি ভুলে যান না—এ দাবির ভিত্তিহীনতা ও সহিহ বর্ণনার আলোকে হাদিস যাচাইয়ের শিক্ষা জানুন।"},"heading":{"title":"ভুলে যাওয়ার হাদিস যাচাই: ভিত্তিহীন বর্ণনা ও সহিহ হাদিসের শিক্ষা","description":"এই বর্ণনায় বলা হয়েছে, “আমি ভুলিনা, কিন্তু আমাকে ভুলিয়ে দেয়া হয় যাতে করে আমি বিধান রচনা করতে পারি।” প্রদত্ত তথ্য অনুযায়ী, এটি বাতিল এবং এর কোনো ভিত্তি নেই। তাই এই কথাকে নবী সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লামের হাদিস হিসেবে প্রচার করা ঠিক নয়। এখানে হাদিস যাচাইয়ের বিষয়টি খুব পরিষ্কারভাবে সামনে আসে। শুধু কোনো বিখ্যাত বইয়ে কোনো কথা পাওয়া গেলেই তা সহিহ হাদিস হয়ে যায় না। প্রদত্ত লেখায় দেখা যায়, গাযালী এটি উল্লেখ করেছেন, কিন্তু হাফিয ইরাকী, ইবনু আব্দিল বার, হামযা আল-কিনানী, আবূ তাহের আনমাতী ও হাফিয ইবনু হাজার—তাঁরা এর ভিত্তি নিয়ে কঠোর কথা বলেছেন। একই সঙ্গে সহিহ বুখারী ও সহিহ মুসলিমের বর্ণনায় এসেছে যে, নবীজি মানুষ হিসেবে ভুলে যেতে পারেন এবং ভুল হলে সাহাবীদের স্মরণ করিয়ে দিতে বলেছেন। তাই মূল শিক্ষা হলো, জাল হাদিস বা ভিত্তিহীন বর্ণনা থেকে সতর্ক থাকা এবং সহিহ বর্ণনার আলোকে কথা বলা।"},"teachings":["কোনো বর্ণনাকে হাদিস বলার আগে তার ভিত্তি ও সনদ যাচাই করা দরকার।","ভিত্তিহীন কথা নবীজি সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লামের নামে প্রচার করা উচিত নয়।","সহিহ বর্ণনা অনুযায়ী, সালাতে ভুল হলে স্মরণ করিয়ে দেওয়া ও সাহু সিজদার শিক্ষা রয়েছে।","বিখ্যাত গ্রন্থে উল্লেখ থাকলেও কোনো কথা সহিহ প্রমাণ না হলে সতর্ক থাকা দরকার।"],"related_hadiths":[{"id":"401","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"1161","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"1244","book_id":"3","slug":"nasai","label":"সুনান আন-নাসায়ী"}]}</t>
         </is>
       </c>
       <c r="E5" s="4" t="n"/>
@@ -580,7 +584,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | শিক্ষাদান নিয়ে দুর্বল হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. আমাকে শিক্ষক হিসেবে পাঠানো হয়েছে—এই বর্ণনাটি অর্থে পরিচিত হলেও সনদের দিক থেকে দুর্বল।"},"heading":{"title":"শিক্ষাদান নিয়ে দুর্বল হাদিস: আমাকে শিক্ষক হিসেবে পাঠানো হয়েছে","description":"এই বর্ণনায় বলা হয়েছে, “আমাকে প্রেরণ করা হয়েছে শিক্ষাদানকারী হিসেবে।” প্রদত্ত আলোচনায় হাদিসটি দুর্বল বলা হয়েছে। এর সনদে আব্দুর রহমান ইবনু যিয়াদ এবং আব্দুর রহমান ইবনু রাফে’—উভয়কে দুর্বল বলা হয়েছে। আরও একটি সনদ এসেছে, সেটি প্রথমটির চেয়ে বেশি দুর্বল বলে আলোচনা করা হয়েছে। তাই এই নির্দিষ্ট বর্ণনাকে শক্ত সহীহ হাদিস হিসেবে ব্যবহার করা ঠিক নয়। তবে রাসূল صلى الله عليه وسلم মানুষকে শিক্ষা দিয়েছেন—এটি ইসলামের বহু সহীহ দলিলে জানা যায়। কিন্তু এই বাক্যটি উদ্ধৃত করার সময় তার দুর্বলতা উল্লেখ করা উচিত। “শিক্ষাদান সম্পর্কে হাদিস” বা “রাসূল صلى الله عليه وسلم শিক্ষক” বিষয়ে লেখার সময় সহীহ বর্ণনা আগে ব্যবহার করা নিরাপদ। এতে জ্ঞানচর্চা ও হাদিসের সততা—দুটিই রক্ষা পায়।"},"teachings":["দুর্বল হাদিসকে সহীহ বলে প্রচার করা উচিত নয়।","রাসূল صلى الله عليه وسلم-এর শিক্ষা দেওয়ার ভূমিকা সত্য, তবে নির্দিষ্ট বর্ণনার সনদ দেখা দরকার।","একাধিক দুর্বল বর্ণনাকারী থাকলে হাদিসের মান কমে যায়।","ইলমের কথা বলার সময় দলিলের মান উল্লেখ করা ভালো।"],"related_hadiths":[{"id":"69","book_id":"1","label":"Sahih Bukhari"},{"id":"2699","book_id":"2","label":"Sahih Muslim"},{"id":"224","book_id":"6","label":"Sunan Ibn Majah"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | শিক্ষাদান নিয়ে দুর্বল হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. আমাকে শিক্ষক হিসেবে পাঠানো হয়েছে—এই বর্ণনাটি অর্থে পরিচিত হলেও সনদের দিক থেকে দুর্বল।"},"heading":{"title":"শিক্ষাদান নিয়ে দুর্বল হাদিস: আমাকে শিক্ষক হিসেবে পাঠানো হয়েছে","description":"এই বর্ণনায় বলা হয়েছে, “আমাকে প্রেরণ করা হয়েছে শিক্ষাদানকারী হিসেবে।” প্রদত্ত আলোচনায় হাদিসটি দুর্বল বলা হয়েছে। এর সনদে আব্দুর রহমান ইবনু যিয়াদ এবং আব্দুর রহমান ইবনু রাফে’—উভয়কে দুর্বল বলা হয়েছে। আরও একটি সনদ এসেছে, সেটি প্রথমটির চেয়ে বেশি দুর্বল বলে আলোচনা করা হয়েছে। তাই এই নির্দিষ্ট বর্ণনাকে শক্ত সহীহ হাদিস হিসেবে ব্যবহার করা ঠিক নয়। তবে রাসূল صلى الله عليه وسلم মানুষকে শিক্ষা দিয়েছেন—এটি ইসলামের বহু সহীহ দলিলে জানা যায়। কিন্তু এই বাক্যটি উদ্ধৃত করার সময় তার দুর্বলতা উল্লেখ করা উচিত। “শিক্ষাদান সম্পর্কে হাদিস” বা “রাসূল صلى الله عليه وسلم শিক্ষক” বিষয়ে লেখার সময় সহীহ বর্ণনা আগে ব্যবহার করা নিরাপদ। এতে জ্ঞানচর্চা ও হাদিসের সততা—দুটিই রক্ষা পায়।"},"teachings":["দুর্বল হাদিসকে সহীহ বলে প্রচার করা উচিত নয়।","রাসূল صلى الله عليه وسلم-এর শিক্ষা দেওয়ার ভূমিকা সত্য, তবে নির্দিষ্ট বর্ণনার সনদ দেখা দরকার।","একাধিক দুর্বল বর্ণনাকারী থাকলে হাদিসের মান কমে যায়।","ইলমের কথা বলার সময় দলিলের মান উল্লেখ করা ভালো।"],"related_hadiths":[{"id":"69","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2699","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"224","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
@@ -603,7 +607,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | দুনিয়া নিয়ে জাল হাদিসের সতর্কতা","description":"$book_name$ $hadith_number$ - $chapter_name$. দুনিয়া আল্লাহর খেদমতকারীকে খেদমত করে—এই বর্ণনাটি জাল বলে উল্লেখ করা হয়েছে।"},"heading":{"title":"দুনিয়া নিয়ে জাল হাদিস: খেদমত কথার যাচাই","description":"এই বর্ণনায় বলা হয়েছে, আল্লাহ দুনিয়াকে ওহীর মাধ্যমে বলেছেন—যে আমার খেদমত করে তুমি তার খেদমত কর, আর যে তোমার খেদমত করে তাকে কষ্ট দাও। প্রদত্ত আলোচনায় হাদিসটি জাল বলা হয়েছে। খতীব বাগদাদীও এটি বানোয়াট বলেছেন বলে উল্লেখ এসেছে। এর সনদে হুসাইন ইবনু দাউদের সমস্যা বলা হয়েছে, যিনি এমন একটি কপি বর্ণনা করেছেন যার অধিকাংশই বানোয়াট। তাই “দুনিয়া তার খেদমত করে” বা “দুনিয়া সম্পর্কিত হাদিস” নামে এই কথাটি রাসূল صلى الله عليه وسلم-এর বাণী হিসেবে বলা যাবে না। দুনিয়ার মোহ থেকে বাঁচা অবশ্যই ইসলামের বড় শিক্ষা, কিন্তু তার জন্য সহীহ আয়াত ও হাদিস রয়েছে। জাল বর্ণনা ব্যবহার করলে মানুষ ভুলকে দ্বীন মনে করতে পারে। তাই দুনিয়া বিষয়ে নসিহত করলেও যাচাই করা সূত্র ব্যবহার করা উচিত।"},"teachings":["দুনিয়া সম্পর্কে নসিহত করতে জাল হাদিস ব্যবহার করা উচিত নয়।","বানোয়াট কপি বা দুর্বল সনদ থেকে সতর্ক থাকতে হবে।","ভালো উপদেশ হলেও রাসূল صلى الله عليه وسلم-এর নামে বলার আগে প্রমাণ দরকার।","দুনিয়ার মোহ থেকে বাঁচার শিক্ষা সহীহ দলিল থেকেই নেওয়া উচিত।"],"related_hadiths":[{"id":"2956","book_id":"2","label":"Sahih Muslim"},{"id":"2322","book_id":"5","label":"Jami at-Tirmidhi"},{"id":"4109","book_id":"6","label":"Sunan Ibn Majah"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | দুনিয়া নিয়ে জাল হাদিসের সতর্কতা","description":"$book_name$ $hadith_number$ - $chapter_name$. দুনিয়া আল্লাহর খেদমতকারীকে খেদমত করে—এই বর্ণনাটি জাল বলে উল্লেখ করা হয়েছে।"},"heading":{"title":"দুনিয়া নিয়ে জাল হাদিস: খেদমত কথার যাচাই","description":"এই বর্ণনায় বলা হয়েছে, আল্লাহ দুনিয়াকে ওহীর মাধ্যমে বলেছেন—যে আমার খেদমত করে তুমি তার খেদমত কর, আর যে তোমার খেদমত করে তাকে কষ্ট দাও। প্রদত্ত আলোচনায় হাদিসটি জাল বলা হয়েছে। খতীব বাগদাদীও এটি বানোয়াট বলেছেন বলে উল্লেখ এসেছে। এর সনদে হুসাইন ইবনু দাউদের সমস্যা বলা হয়েছে, যিনি এমন একটি কপি বর্ণনা করেছেন যার অধিকাংশই বানোয়াট। তাই “দুনিয়া তার খেদমত করে” বা “দুনিয়া সম্পর্কিত হাদিস” নামে এই কথাটি রাসূল صلى الله عليه وسلم-এর বাণী হিসেবে বলা যাবে না। দুনিয়ার মোহ থেকে বাঁচা অবশ্যই ইসলামের বড় শিক্ষা, কিন্তু তার জন্য সহীহ আয়াত ও হাদিস রয়েছে। জাল বর্ণনা ব্যবহার করলে মানুষ ভুলকে দ্বীন মনে করতে পারে। তাই দুনিয়া বিষয়ে নসিহত করলেও যাচাই করা সূত্র ব্যবহার করা উচিত।"},"teachings":["দুনিয়া সম্পর্কে নসিহত করতে জাল হাদিস ব্যবহার করা উচিত নয়।","বানোয়াট কপি বা দুর্বল সনদ থেকে সতর্ক থাকতে হবে।","ভালো উপদেশ হলেও রাসূল صلى الله عليه وسلم-এর নামে বলার আগে প্রমাণ দরকার।","দুনিয়ার মোহ থেকে বাঁচার শিক্ষা সহীহ দলিল থেকেই নেওয়া উচিত।"],"related_hadiths":[{"id":"2956","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"2322","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"4109","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
         </is>
       </c>
       <c r="E7" s="4" t="n"/>
@@ -626,7 +630,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | শাম সম্পর্কে দুর্বল বর্ণনা","description":"$book_name$ $hadith_number$ - $chapter_name$. শামের অধিবাসীদের নিয়ে এই বর্ণনাটি মারফূ হিসেবে দুর্বল; মওকূফ হিসেবেই বেশি সঠিক বলা হয়েছে।"},"heading":{"title":"শাম সম্পর্কে দুর্বল হাদিস: মারফূ না মওকূফ?","description":"এই বর্ণনায় শামের অধিবাসীদের আল্লাহর পৃথিবীতে তাঁর চাবুক বলা হয়েছে। প্রদত্ত আলোচনায় হাদিসটি দুর্বল বলা হয়েছে। কারণ হিসেবে ওয়ালীদ ইবনু মুসলিমের আনআন করে বর্ণনা এবং তাঁর তাদলীসের সমস্যা উল্লেখ করা হয়েছে। আরও বলা হয়েছে, মওকূফ অর্থাৎ সাহাবীর কথা হিসেবে এর সনদ সহীহ। তাই এই নির্দিষ্ট বর্ণনাকে সরাসরি রাসূল صلى الله عليه وسلم-এর হাদিস হিসেবে বলা ঠিক নয়। শাম সম্পর্কে কিছু ফজিলতের বর্ণনা অন্য জায়গায় থাকতে পারে, কিন্তু এই বর্ণনার মান আলাদা করে বুঝতে হবে। “শাম সম্পর্কে হাদিস” খোঁজার সময় মারফূ ও মওকূফ পার্থক্য জানা দরকার। এতে দলিল ব্যবহারে সতর্কতা আসে। মুসলিমের জন্য নিরাপদ হলো—যে কথাটি সাহাবীর কথা হিসেবে সঠিক, তাকে নবী صلى الله عليه وسلم-এর কথা বানিয়ে না বলা।"},"teachings":["মারফূ ও মওকূফ বর্ণনার পার্থক্য জানা জরুরি।","তাদলীস থাকা সনদে অতিরিক্ত সতর্কতা দরকার।","শাম সম্পর্কে বর্ণনা ব্যবহার করলে তার মান দেখা উচিত।","সাহাবীর কথা রাসূল صلى الله عليه وسلم-এর হাদিস হিসেবে প্রচার করা যাবে না।"],"related_hadiths":[{"id":"3511","book_id":"1","label":"Sahih Bukhari"},{"id":"3954","book_id":"5","label":"Jami at-Tirmidhi"},{"id":"2483","book_id":"4","label":"Sunan Abu Dawud"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | শাম সম্পর্কে দুর্বল বর্ণনা","description":"$book_name$ $hadith_number$ - $chapter_name$. শামের অধিবাসীদের নিয়ে এই বর্ণনাটি মারফূ হিসেবে দুর্বল; মওকূফ হিসেবেই বেশি সঠিক বলা হয়েছে।"},"heading":{"title":"শাম সম্পর্কে দুর্বল হাদিস: মারফূ না মওকূফ?","description":"এই বর্ণনায় শামের অধিবাসীদের আল্লাহর পৃথিবীতে তাঁর চাবুক বলা হয়েছে। প্রদত্ত আলোচনায় হাদিসটি দুর্বল বলা হয়েছে। কারণ হিসেবে ওয়ালীদ ইবনু মুসলিমের আনআন করে বর্ণনা এবং তাঁর তাদলীসের সমস্যা উল্লেখ করা হয়েছে। আরও বলা হয়েছে, মওকূফ অর্থাৎ সাহাবীর কথা হিসেবে এর সনদ সহীহ। তাই এই নির্দিষ্ট বর্ণনাকে সরাসরি রাসূল صلى الله عليه وسلم-এর হাদিস হিসেবে বলা ঠিক নয়। শাম সম্পর্কে কিছু ফজিলতের বর্ণনা অন্য জায়গায় থাকতে পারে, কিন্তু এই বর্ণনার মান আলাদা করে বুঝতে হবে। “শাম সম্পর্কে হাদিস” খোঁজার সময় মারফূ ও মওকূফ পার্থক্য জানা দরকার। এতে দলিল ব্যবহারে সতর্কতা আসে। মুসলিমের জন্য নিরাপদ হলো—যে কথাটি সাহাবীর কথা হিসেবে সঠিক, তাকে নবী صلى الله عليه وسلم-এর কথা বানিয়ে না বলা।"},"teachings":["মারফূ ও মওকূফ বর্ণনার পার্থক্য জানা জরুরি।","তাদলীস থাকা সনদে অতিরিক্ত সতর্কতা দরকার।","শাম সম্পর্কে বর্ণনা ব্যবহার করলে তার মান দেখা উচিত।","সাহাবীর কথা রাসূল صلى الله عليه وسلم-এর হাদিস হিসেবে প্রচার করা যাবে না।"],"related_hadiths":[{"id":"3511","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"3954","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"2483","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"}]}</t>
         </is>
       </c>
       <c r="E8" s="4" t="n"/>
@@ -649,7 +653,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | বিয়ের পছন্দ নিয়ে দুর্বল বর্ণনা","description":"$book_name$ $hadith_number$ - $chapter_name$. সুন্দরী নারী ও বংশ নিয়ে প্রচলিত এই বর্ণনাটি নিতান্তই দুর্বল বলা হয়েছে।"},"heading":{"title":"বিয়ের পছন্দ নিয়ে দুর্বল হাদিস: সুন্দরী নারী প্রসঙ্গ","description":"এই বর্ণনায় সার দেওয়া ভূমির সবুজের মতো নিকৃষ্ট উৎপত্তি থেকে জন্ম নেওয়া সুন্দরী নারী থেকে সতর্ক করার কথা এসেছে। প্রদত্ত আলোচনায় হাদিসটি নিতান্তই দুর্বল বলা হয়েছে। এর সনদে ওয়াকেদী এককভাবে বর্ণনা করেছেন, আর তাকে দুর্বল, এমনকি অনেক মুহাদ্দিস মিথ্যুক বলেছেন বলে উল্লেখ আছে। তাই এই বর্ণনাকে সহীহ হাদিস হিসেবে ব্যবহার করা উচিত নয়। বিয়ের পছন্দ নিয়ে ইসলামি শিক্ষা গুরুত্বপূর্ণ, কিন্তু এই নির্দিষ্ট কথাকে নবী صلى الله عليه وسلم-এর নামে বলা নিরাপদ নয়। “বিয়ের জন্য নারী নির্বাচন হাদিস” বা “সুন্দরী নারী সম্পর্কে হাদিস” খোঁজার সময় সহীহ দলিল দেখা দরকার। কোনো ব্যক্তি বা পরিবারকে অপমান করার জন্য দুর্বল বর্ণনা ব্যবহার করা আরও ক্ষতিকর হতে পারে। তাই হাদিস যাচাই এবং কথার শালীনতা—দুটিই জরুরি।"},"teachings":["বিয়ের বিষয়ে দুর্বল বর্ণনা দিয়ে সিদ্ধান্ত বা অপমান করা উচিত নয়।","একক দুর্বল বর্ণনাকারীর বর্ণনা সতর্কতার সঙ্গে দেখতে হয়।","সুন্দর কথাকে হাদিস বলার আগে সনদ যাচাই জরুরি।","মানুষের বংশ বা পরিবার নিয়ে কথা বলায় শালীনতা দরকার।"],"related_hadiths":[{"id":"5090","book_id":"1","label":"Sahih Bukhari"},{"id":"1466","book_id":"2","label":"Sahih Muslim"},{"id":"2047","book_id":"4","label":"Sunan Abu Dawud"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | বিয়ের পছন্দ নিয়ে দুর্বল বর্ণনা","description":"$book_name$ $hadith_number$ - $chapter_name$. সুন্দরী নারী ও বংশ নিয়ে প্রচলিত এই বর্ণনাটি নিতান্তই দুর্বল বলা হয়েছে।"},"heading":{"title":"বিয়ের পছন্দ নিয়ে দুর্বল হাদিস: সুন্দরী নারী প্রসঙ্গ","description":"এই বর্ণনায় সার দেওয়া ভূমির সবুজের মতো নিকৃষ্ট উৎপত্তি থেকে জন্ম নেওয়া সুন্দরী নারী থেকে সতর্ক করার কথা এসেছে। প্রদত্ত আলোচনায় হাদিসটি নিতান্তই দুর্বল বলা হয়েছে। এর সনদে ওয়াকেদী এককভাবে বর্ণনা করেছেন, আর তাকে দুর্বল, এমনকি অনেক মুহাদ্দিস মিথ্যুক বলেছেন বলে উল্লেখ আছে। তাই এই বর্ণনাকে সহীহ হাদিস হিসেবে ব্যবহার করা উচিত নয়। বিয়ের পছন্দ নিয়ে ইসলামি শিক্ষা গুরুত্বপূর্ণ, কিন্তু এই নির্দিষ্ট কথাকে নবী صلى الله عليه وسلم-এর নামে বলা নিরাপদ নয়। “বিয়ের জন্য নারী নির্বাচন হাদিস” বা “সুন্দরী নারী সম্পর্কে হাদিস” খোঁজার সময় সহীহ দলিল দেখা দরকার। কোনো ব্যক্তি বা পরিবারকে অপমান করার জন্য দুর্বল বর্ণনা ব্যবহার করা আরও ক্ষতিকর হতে পারে। তাই হাদিস যাচাই এবং কথার শালীনতা—দুটিই জরুরি।"},"teachings":["বিয়ের বিষয়ে দুর্বল বর্ণনা দিয়ে সিদ্ধান্ত বা অপমান করা উচিত নয়।","একক দুর্বল বর্ণনাকারীর বর্ণনা সতর্কতার সঙ্গে দেখতে হয়।","সুন্দর কথাকে হাদিস বলার আগে সনদ যাচাই জরুরি।","মানুষের বংশ বা পরিবার নিয়ে কথা বলায় শালীনতা দরকার।"],"related_hadiths":[{"id":"5090","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"1466","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"2047","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"}]}</t>
         </is>
       </c>
       <c r="E9" s="4" t="n"/>
@@ -672,7 +676,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | শাম নিয়ে ভিত্তিহীন মারফূ বর্ণনা","description":"$book_name$ $hadith_number$ - $chapter_name$. শাম আমার তীর রাখার স্থল—এই কথাটি মারফূ হাদিস হিসেবে ভিত্তিহীন বলা হয়েছে।"},"heading":{"title":"শাম আমার তীর রাখার স্থল—মারফূ হিসেবে ভিত্তিহীন","description":"এই বর্ণনায় বলা হয়েছে, “শাম দেশ আমার তীর রাখার স্থল। যে তার ক্ষতি করতে চাইবে, আমি তাকে সেখানকার তীর দ্বারা আঘাত করব।” প্রদত্ত আলোচনায় বলা হয়েছে, মারফূ হিসেবে হাদিসটির কোনো ভিত্তি নেই। এমনও বলা হয়েছে, সম্ভবত এটি ইসরাইলী বর্ণনার অন্তর্ভুক্ত। সনদে মাসউদী নামের একজন বর্ণনাকারীর দুর্বলতার কথা এসেছে, কারণ তাঁর স্মৃতিতে পরিবর্তন ঘটেছিল। আরও কিছু বর্ণনাকারীর পরিচয় পাওয়া যায়নি বলে উল্লেখ আছে। তাই “শাম সম্পর্কে হাদিস” হিসেবে এই কথাটি ব্যবহার করা ঠিক নয়। শামের ফজিলত নিয়ে কোনো কথা বলতে হলে নির্ভরযোগ্য বর্ণনা বেছে নিতে হবে। শুধু আবেগ বা অঞ্চলভিত্তিক ভালোবাসা দিয়ে হাদিস প্রমাণ হয় না। নবী صلى الله عليه وسلم-এর নামে কোনো কথা বলার আগে তার সনদ ও মান জানা জরুরি।"},"teachings":["অঞ্চল সম্পর্কিত বর্ণনাও যাচাই করা দরকার।","ইসরাইলী বর্ণনা ও মারফূ হাদিস এক নয়।","অপরিচিত বা দুর্বল বর্ণনাকারী থাকলে সতর্কতা দরকার।","শামের ফজিলত বলতে সহীহ সূত্র ব্যবহার করা উচিত।"],"related_hadiths":[{"id":"3511","book_id":"1","label":"Sahih Bukhari"},{"id":"3954","book_id":"5","label":"Jami at-Tirmidhi"},{"id":"2483","book_id":"4","label":"Sunan Abu Dawud"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | শাম নিয়ে ভিত্তিহীন মারফূ বর্ণনা","description":"$book_name$ $hadith_number$ - $chapter_name$. শাম আমার তীর রাখার স্থল—এই কথাটি মারফূ হাদিস হিসেবে ভিত্তিহীন বলা হয়েছে।"},"heading":{"title":"শাম আমার তীর রাখার স্থল—মারফূ হিসেবে ভিত্তিহীন","description":"এই বর্ণনায় বলা হয়েছে, “শাম দেশ আমার তীর রাখার স্থল। যে তার ক্ষতি করতে চাইবে, আমি তাকে সেখানকার তীর দ্বারা আঘাত করব।” প্রদত্ত আলোচনায় বলা হয়েছে, মারফূ হিসেবে হাদিসটির কোনো ভিত্তি নেই। এমনও বলা হয়েছে, সম্ভবত এটি ইসরাইলী বর্ণনার অন্তর্ভুক্ত। সনদে মাসউদী নামের একজন বর্ণনাকারীর দুর্বলতার কথা এসেছে, কারণ তাঁর স্মৃতিতে পরিবর্তন ঘটেছিল। আরও কিছু বর্ণনাকারীর পরিচয় পাওয়া যায়নি বলে উল্লেখ আছে। তাই “শাম সম্পর্কে হাদিস” হিসেবে এই কথাটি ব্যবহার করা ঠিক নয়। শামের ফজিলত নিয়ে কোনো কথা বলতে হলে নির্ভরযোগ্য বর্ণনা বেছে নিতে হবে। শুধু আবেগ বা অঞ্চলভিত্তিক ভালোবাসা দিয়ে হাদিস প্রমাণ হয় না। নবী صلى الله عليه وسلم-এর নামে কোনো কথা বলার আগে তার সনদ ও মান জানা জরুরি।"},"teachings":["অঞ্চল সম্পর্কিত বর্ণনাও যাচাই করা দরকার।","ইসরাইলী বর্ণনা ও মারফূ হাদিস এক নয়।","অপরিচিত বা দুর্বল বর্ণনাকারী থাকলে সতর্কতা দরকার।","শামের ফজিলত বলতে সহীহ সূত্র ব্যবহার করা উচিত।"],"related_hadiths":[{"id":"3511","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"3954","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"2483","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"}]}</t>
         </is>
       </c>
       <c r="E10" s="4" t="n"/>
@@ -695,7 +699,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | নেতা ও আলেম নিয়ে জাল হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. উম্মতের নেতা ও আলেম ঠিক হলে মানুষ ভালো হবে—এই বর্ণনাটি জাল বলা হয়েছে।"},"heading":{"title":"নেতা ও আলেম ঠিক হলে মানুষ ভালো হবে—জাল হাদিস","description":"এই বর্ণনায় বলা হয়েছে, উম্মতের দুই শ্রেণী—নেতাগণ ও ফাকীহ বা আলেমগণ—ঠিক হলে মানুষ ভালো হবে। প্রদত্ত আলোচনায় হাদিসটি জাল বলা হয়েছে। এর সনদে মুহাম্মাদ ইবনু যিয়াদ ইয়াশকুরী নামের একজন বর্ণনাকারী আছেন, যাকে ইমাম আহমাদ, ইবনু মাঈন, দারাকুতনীসহ অনেকে মিথ্যুক ও হাদিস জালকারী বলেছেন। তাই এই নির্দিষ্ট বাক্যকে রাসূল صلى الله عليه وسلم-এর হাদিস বলা যাবে না। অবশ্য সমাজে নেতা ও আলেমের প্রভাব বড়—এ কথা সাধারণভাবে বোঝা যায়; কিন্তু এই বর্ণনা দিয়ে তা প্রমাণ করা ঠিক নয়। “নেতা ও আলেম সম্পর্কে হাদিস” খোঁজার সময় বিশেষ সতর্কতা দরকার। কারণ নেতৃত্ব ও ইলমের বিষয় মানুষ দ্রুত শেয়ার করে, কিন্তু জাল হাদিস ছড়ালে দ্বীনের নামে ভুল কথা ছড়ায়।"},"teachings":["নেতা ও আলেম নিয়ে কথাও সহীহ দলিল দিয়ে বলতে হবে।","সনদে মিথ্যুক বর্ণনাকারী থাকলে বর্ণনা গ্রহণযোগ্য নয়।","জাল হাদিসকে শুধু দুর্বল বলে হালকা করে দেখা উচিত নয়।","সামাজিক শিক্ষা দিতে গিয়ে রাসূল صلى الله عليه وسلم-এর নামে ভুল কথা বলা যাবে না।"],"related_hadiths":[{"id":"7138","book_id":"1","label":"Sahih Bukhari"},{"id":"1829","book_id":"2","label":"Sahih Muslim"},{"id":"3641","book_id":"4","label":"Sunan Abu Dawud"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | নেতা ও আলেম নিয়ে জাল হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. উম্মতের নেতা ও আলেম ঠিক হলে মানুষ ভালো হবে—এই বর্ণনাটি জাল বলা হয়েছে।"},"heading":{"title":"নেতা ও আলেম ঠিক হলে মানুষ ভালো হবে—জাল হাদিস","description":"এই বর্ণনায় বলা হয়েছে, উম্মতের দুই শ্রেণী—নেতাগণ ও ফাকীহ বা আলেমগণ—ঠিক হলে মানুষ ভালো হবে। প্রদত্ত আলোচনায় হাদিসটি জাল বলা হয়েছে। এর সনদে মুহাম্মাদ ইবনু যিয়াদ ইয়াশকুরী নামের একজন বর্ণনাকারী আছেন, যাকে ইমাম আহমাদ, ইবনু মাঈন, দারাকুতনীসহ অনেকে মিথ্যুক ও হাদিস জালকারী বলেছেন। তাই এই নির্দিষ্ট বাক্যকে রাসূল صلى الله عليه وسلم-এর হাদিস বলা যাবে না। অবশ্য সমাজে নেতা ও আলেমের প্রভাব বড়—এ কথা সাধারণভাবে বোঝা যায়; কিন্তু এই বর্ণনা দিয়ে তা প্রমাণ করা ঠিক নয়। “নেতা ও আলেম সম্পর্কে হাদিস” খোঁজার সময় বিশেষ সতর্কতা দরকার। কারণ নেতৃত্ব ও ইলমের বিষয় মানুষ দ্রুত শেয়ার করে, কিন্তু জাল হাদিস ছড়ালে দ্বীনের নামে ভুল কথা ছড়ায়।"},"teachings":["নেতা ও আলেম নিয়ে কথাও সহীহ দলিল দিয়ে বলতে হবে।","সনদে মিথ্যুক বর্ণনাকারী থাকলে বর্ণনা গ্রহণযোগ্য নয়।","জাল হাদিসকে শুধু দুর্বল বলে হালকা করে দেখা উচিত নয়।","সামাজিক শিক্ষা দিতে গিয়ে রাসূল صلى الله عليه وسلم-এর নামে ভুল কথা বলা যাবে না।"],"related_hadiths":[{"id":"7138","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"1829","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"3641","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"}]}</t>
         </is>
       </c>
       <c r="E11" s="4" t="n"/>
@@ -718,7 +722,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | গুনাহ নিয়ে জাল হাদিসের সতর্কতা","description":"$book_name$ $hadith_number$ - $chapter_name$. হাসতে হাসতে গুনাহ করলে কাঁদতে কাঁদতে জাহান্নামে যাবে—এই বর্ণনাটি জাল।"},"heading":{"title":"হাসতে হাসতে গুনাহ করলে—জাল হাদিসের সতর্কতা","description":"এই বর্ণনায় বলা হয়েছে, যে ব্যক্তি হাসতে হাসতে গুনাহ করবে, সে কাঁদতে কাঁদতে জাহান্নামে প্রবেশ করবে। প্রদত্ত আলোচনায় হাদিসটি জাল বলা হয়েছে। এর সনদে উমার ইবনু আইউব এবং মুহাম্মাদ ইবনু যিয়াদ ইয়াশকুরীর সমস্যা উল্লেখ করা হয়েছে। বিশেষ করে ইয়াশকুরীকে মুহাদ্দিসগণ মিথ্যুক ও হাদিস জালকারী বলেছেন। তাই এই নির্দিষ্ট বাক্যকে হাদিস হিসেবে ব্যবহার করা ঠিক নয়। গুনাহকে হালকা করে দেখা অবশ্যই ভয়ংকর বিষয়—এ কথা ইসলামের সাধারণ শিক্ষা। কিন্তু মানুষকে গুনাহ থেকে বাঁচাতে জাল হাদিস দিয়ে ভয় দেখানো যাবে না। “গুনাহ নিয়ে হাদিস” বা “হাসতে হাসতে গুনাহ” নামে প্রচলিত পোস্ট দেখলে উৎস যাচাই করা দরকার। সহীহ দলিল দিয়েই তাওবা, ভয় ও আশা—সব শেখানো যায়।"},"teachings":["গুনাহকে হালকা করা ভালো নয়, তবে জাল হাদিস দিয়ে ভয় দেখানো ঠিক নয়।","সনদে জালকারী থাকলে বর্ণনা গ্রহণযোগ্য নয়।","ধর্মীয় সতর্কতা দিতে সহীহ দলিল ব্যবহার করা উচিত।","প্রচলিত ভয় দেখানো বাক্য যাচাই ছাড়া শেয়ার করা যাবে না।"],"related_hadiths":[{"id":"6308","book_id":"1","label":"Sahih Bukhari"},{"id":"2749","book_id":"2","label":"Sahih Muslim"},{"id":"2497","book_id":"5","label":"Jami at-Tirmidhi"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | গুনাহ নিয়ে জাল হাদিসের সতর্কতা","description":"$book_name$ $hadith_number$ - $chapter_name$. হাসতে হাসতে গুনাহ করলে কাঁদতে কাঁদতে জাহান্নামে যাবে—এই বর্ণনাটি জাল।"},"heading":{"title":"হাসতে হাসতে গুনাহ করলে—জাল হাদিসের সতর্কতা","description":"এই বর্ণনায় বলা হয়েছে, যে ব্যক্তি হাসতে হাসতে গুনাহ করবে, সে কাঁদতে কাঁদতে জাহান্নামে প্রবেশ করবে। প্রদত্ত আলোচনায় হাদিসটি জাল বলা হয়েছে। এর সনদে উমার ইবনু আইউব এবং মুহাম্মাদ ইবনু যিয়াদ ইয়াশকুরীর সমস্যা উল্লেখ করা হয়েছে। বিশেষ করে ইয়াশকুরীকে মুহাদ্দিসগণ মিথ্যুক ও হাদিস জালকারী বলেছেন। তাই এই নির্দিষ্ট বাক্যকে হাদিস হিসেবে ব্যবহার করা ঠিক নয়। গুনাহকে হালকা করে দেখা অবশ্যই ভয়ংকর বিষয়—এ কথা ইসলামের সাধারণ শিক্ষা। কিন্তু মানুষকে গুনাহ থেকে বাঁচাতে জাল হাদিস দিয়ে ভয় দেখানো যাবে না। “গুনাহ নিয়ে হাদিস” বা “হাসতে হাসতে গুনাহ” নামে প্রচলিত পোস্ট দেখলে উৎস যাচাই করা দরকার। সহীহ দলিল দিয়েই তাওবা, ভয় ও আশা—সব শেখানো যায়।"},"teachings":["গুনাহকে হালকা করা ভালো নয়, তবে জাল হাদিস দিয়ে ভয় দেখানো ঠিক নয়।","সনদে জালকারী থাকলে বর্ণনা গ্রহণযোগ্য নয়।","ধর্মীয় সতর্কতা দিতে সহীহ দলিল ব্যবহার করা উচিত।","প্রচলিত ভয় দেখানো বাক্য যাচাই ছাড়া শেয়ার করা যাবে না।"],"related_hadiths":[{"id":"6308","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2749","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"2497","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"}]}</t>
         </is>
       </c>
       <c r="E12" s="4" t="n"/>
@@ -741,7 +745,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কবুতর ও জিন নিয়ে জাল হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. পরকাটা কবুতর সন্তানদের থেকে জিন দূর করে—এই বর্ণনাটি জাল বলে উল্লেখ করা হয়েছে।"},"heading":{"title":"কবুতর ও জিন নিয়ে জাল হাদিস: সন্তান প্রসঙ্গে সতর্কতা","description":"এই বর্ণনায় বলা হয়েছে, পরকাটা কবুতর গ্রহণ করো, কারণ তা সন্তানদের থেকে জিনকে বিমুখ করে দেয়। প্রদত্ত আলোচনায় হাদিসটি জাল বলা হয়েছে। এটি পূর্বের সনদে মুহাম্মাদ ইবনু যিয়াদ ইয়াশকুরীর সূত্রে এসেছে, আর তাঁর সম্পর্কে ইমাম আহমাদ, ইবনু মাঈনসহ বহু মুহাদ্দিস বলেছেন—তিনি মিথ্যুক ও হাদিস জালকারী। তাই “কবুতর জিন দূর করে” বা “সন্তানদের জিন থেকে বাঁচানোর হাদিস” নামে এই কথাটি প্রচার করা ঠিক নয়। জিনের ক্ষতি থেকে বাঁচার জন্য ইসলামে সহীহ দোয়া, যিকির ও আশ্রয় প্রার্থনার শিক্ষা আছে। কিন্তু পশু-পাখি নিয়ে ভিত্তিহীন বিশ্বাস তৈরি করা উচিত নয়। হাদিস যাচাই না করলে কুসংস্কার দ্বীনের নামে ছড়িয়ে যেতে পারে।"},"teachings":["জিন থেকে বাঁচার বিষয়ে জাল বর্ণনা বিশ্বাস করা ঠিক নয়।","সন্তান রক্ষার জন্য সহীহ দোয়া ও যিকিরে ভরসা করা উচিত।","কুসংস্কারকে হাদিসের নামে ছড়ানো বিপজ্জনক।","মিথ্যুক বর্ণনাকারীর বর্ণনা গ্রহণযোগ্য নয়।"],"related_hadiths":[{"id":"3275","book_id":"1","label":"Sahih Bukhari"},{"id":"2181","book_id":"2","label":"Sahih Muslim"},{"id":"5088","book_id":"4","label":"Sunan Abu Dawud"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কবুতর ও জিন নিয়ে জাল হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. পরকাটা কবুতর সন্তানদের থেকে জিন দূর করে—এই বর্ণনাটি জাল বলে উল্লেখ করা হয়েছে।"},"heading":{"title":"কবুতর ও জিন নিয়ে জাল হাদিস: সন্তান প্রসঙ্গে সতর্কতা","description":"এই বর্ণনায় বলা হয়েছে, পরকাটা কবুতর গ্রহণ করো, কারণ তা সন্তানদের থেকে জিনকে বিমুখ করে দেয়। প্রদত্ত আলোচনায় হাদিসটি জাল বলা হয়েছে। এটি পূর্বের সনদে মুহাম্মাদ ইবনু যিয়াদ ইয়াশকুরীর সূত্রে এসেছে, আর তাঁর সম্পর্কে ইমাম আহমাদ, ইবনু মাঈনসহ বহু মুহাদ্দিস বলেছেন—তিনি মিথ্যুক ও হাদিস জালকারী। তাই “কবুতর জিন দূর করে” বা “সন্তানদের জিন থেকে বাঁচানোর হাদিস” নামে এই কথাটি প্রচার করা ঠিক নয়। জিনের ক্ষতি থেকে বাঁচার জন্য ইসলামে সহীহ দোয়া, যিকির ও আশ্রয় প্রার্থনার শিক্ষা আছে। কিন্তু পশু-পাখি নিয়ে ভিত্তিহীন বিশ্বাস তৈরি করা উচিত নয়। হাদিস যাচাই না করলে কুসংস্কার দ্বীনের নামে ছড়িয়ে যেতে পারে।"},"teachings":["জিন থেকে বাঁচার বিষয়ে জাল বর্ণনা বিশ্বাস করা ঠিক নয়।","সন্তান রক্ষার জন্য সহীহ দোয়া ও যিকিরে ভরসা করা উচিত।","কুসংস্কারকে হাদিসের নামে ছড়ানো বিপজ্জনক।","মিথ্যুক বর্ণনাকারীর বর্ণনা গ্রহণযোগ্য নয়।"],"related_hadiths":[{"id":"3275","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2181","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"5088","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"}]}</t>
         </is>
       </c>
       <c r="E13" s="4" t="n"/>
@@ -764,7 +768,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | নারীদের মজলিস নিয়ে বানোয়াট হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. নারীদের মজলিস প্রেমালাপ দিয়ে সাজাও—এই বর্ণনাটি বানোয়াট বলা হয়েছে।"},"heading":{"title":"নারীদের মজলিস নিয়ে বানোয়াট হাদিসের সতর্কতা","description":"এই বর্ণনায় বলা হয়েছে, “তোমরা তোমাদের নারীদের মজলিসগুলো প্রেমালাপের দ্বারা সৌন্দর্যমণ্ডিত কর।” প্রদত্ত আলোচনায় হাদিসটি বানোয়াট বলা হয়েছে। এটি ইয়াশকুরী সূত্রে বর্ণিত হয়েছে, আর তাঁর সম্পর্কে বলা হয়েছে তিনি দুর্বলদের অন্তর্ভুক্ত এবং এমন মুনকার বর্ণনা করেছেন যা অন্য নির্ভরযোগ্য বর্ণনাকারীরা বর্ণনা করেননি। ইবনুল জাওযী এটিকে মাওযূআত গ্রন্থে উল্লেখ করেছেন এবং সুয়ূতীও সমর্থন করেছেন বলে লেখা আছে। তাই এই বাক্যকে হাদিস বলা ঠিক নয়। “নারীদের মজলিস সম্পর্কে হাদিস” বা পারিবারিক সম্পর্ক নিয়ে কথা বলার সময় সহীহ দলিল ব্যবহার করতে হবে। কোনো অশালীন বা অস্পষ্ট অর্থের কথাকে নবী صلى الله عليه وسلم-এর নামে চালানো আরও বেশি ক্ষতিকর। মুসলিমের কথা হওয়া উচিত যাচাই করা, শালীন এবং সত্যভিত্তিক।"},"teachings":["নারী ও পরিবার বিষয়ে বানোয়াট বর্ণনা ব্যবহার করা উচিত নয়।","মুনকার বর্ণনা থেকে সতর্ক থাকতে হবে।","শালীনতা রক্ষা করে সহীহ দলিলের ভিত্তিতে কথা বলা জরুরি।","যাচাই ছাড়া প্রচলিত কথাকে হাদিস বলা যায় না।"],"related_hadiths":[{"id":"5185","book_id":"1","label":"Sahih Bukhari"},{"id":"1468","book_id":"2","label":"Sahih Muslim"},{"id":"2142","book_id":"4","label":"Sunan Abu Dawud"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | নারীদের মজলিস নিয়ে বানোয়াট হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. নারীদের মজলিস প্রেমালাপ দিয়ে সাজাও—এই বর্ণনাটি বানোয়াট বলা হয়েছে।"},"heading":{"title":"নারীদের মজলিস নিয়ে বানোয়াট হাদিসের সতর্কতা","description":"এই বর্ণনায় বলা হয়েছে, “তোমরা তোমাদের নারীদের মজলিসগুলো প্রেমালাপের দ্বারা সৌন্দর্যমণ্ডিত কর।” প্রদত্ত আলোচনায় হাদিসটি বানোয়াট বলা হয়েছে। এটি ইয়াশকুরী সূত্রে বর্ণিত হয়েছে, আর তাঁর সম্পর্কে বলা হয়েছে তিনি দুর্বলদের অন্তর্ভুক্ত এবং এমন মুনকার বর্ণনা করেছেন যা অন্য নির্ভরযোগ্য বর্ণনাকারীরা বর্ণনা করেননি। ইবনুল জাওযী এটিকে মাওযূআত গ্রন্থে উল্লেখ করেছেন এবং সুয়ূতীও সমর্থন করেছেন বলে লেখা আছে। তাই এই বাক্যকে হাদিস বলা ঠিক নয়। “নারীদের মজলিস সম্পর্কে হাদিস” বা পারিবারিক সম্পর্ক নিয়ে কথা বলার সময় সহীহ দলিল ব্যবহার করতে হবে। কোনো অশালীন বা অস্পষ্ট অর্থের কথাকে নবী صلى الله عليه وسلم-এর নামে চালানো আরও বেশি ক্ষতিকর। মুসলিমের কথা হওয়া উচিত যাচাই করা, শালীন এবং সত্যভিত্তিক।"},"teachings":["নারী ও পরিবার বিষয়ে বানোয়াট বর্ণনা ব্যবহার করা উচিত নয়।","মুনকার বর্ণনা থেকে সতর্ক থাকতে হবে।","শালীনতা রক্ষা করে সহীহ দলিলের ভিত্তিতে কথা বলা জরুরি।","যাচাই ছাড়া প্রচলিত কথাকে হাদিস বলা যায় না।"],"related_hadiths":[{"id":"5185","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"1468","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"2142","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"}]}</t>
         </is>
       </c>
       <c r="E14" s="4" t="n"/>
@@ -787,7 +791,7 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সলাত নিয়ে বাতিল বর্ণনার বিশ্লেষণ","description":"$book_name$ $hadith_number$ - $chapter_name$. সলাত গুনাহ থেকে বিরত রাখে—এ শিক্ষা সত্য, তবে এই নির্দিষ্ট বর্ণনাটি মারফূ হিসেবে সহীহ নয়।"},"heading":{"title":"সলাত নিয়ে বাতিল হাদিস: সলাত দূরত্ব বাড়ায় কি?","description":"এই বর্ণনায় বলা হয়েছে, যে ব্যক্তির সলাত তাকে অশ্লীল ও মন্দ কাজ থেকে বিরত করে না, আল্লাহর কাছ থেকে তার দূরত্বই বাড়ে। কিন্তু প্রদত্ত লেখায় স্পষ্ট বলা হয়েছে, হাদিসটি বাতিল; সনদ ও ভাষা উভয় দিক থেকেই এটি সহীহ নয়। এখানে মূল শিক্ষা হলো—সলাতের গুরুত্ব ঠিক রাখতে হবে, কিন্তু দুর্বল বা বাতিল বর্ণনা দিয়ে ভয় দেখানো ঠিক নয়। লেখায় বলা হয়েছে, বর্ণনাটির কিছু কথা সাহাবী বা হাসান বসরীর কথা হিসেবে এসেছে, কিন্তু রাসূল صلى الله عليه وسلم-এর বাণী হিসেবে সাব্যস্ত নয়। একই সঙ্গে কুরআনের আয়াত উল্লেখ করা হয়েছে যে সলাত নির্লজ্জ ও মন্দ কাজ থেকে বিরত রাখে। তাই সলাতের প্রভাব অস্বীকার করা যাবে না, আবার এই নির্দিষ্ট বাক্যকে সহীহ হাদিসও বলা যাবে না। “সলাত গুনাহ থেকে বিরত রাখে” বিষয়টি বুঝতে হলে সহীহ দলিলের ওপর নির্ভর করা জরুরি।"},"teachings":["সলাতের মর্যাদা বুঝাতে সহীহ দলিল ব্যবহার করা উচিত।","প্রচলিত কোনো কথা হাদিস হিসেবে বিখ্যাত হলেও তা সহীহ নাও হতে পারে।","সলাত মানুষকে মন্দ কাজ থেকে ফিরাতে সাহায্য করে—এটি কুরআনের শিক্ষা।","সাহাবীর কথা ও রাসূল صلى الله عليه وسلم-এর হাদিস—দুটির মর্যাদা এক নয়।"],"related_hadiths":[{"id":"526","book_id":"1","label":"Sahih Bukhari"},{"id":"667","book_id":"2","label":"Sahih Muslim"},{"id":"864","book_id":"4","label":"Sunan Abu Dawud"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সলাত নিয়ে বাতিল বর্ণনার বিশ্লেষণ","description":"$book_name$ $hadith_number$ - $chapter_name$. সলাত গুনাহ থেকে বিরত রাখে—এ শিক্ষা সত্য, তবে এই নির্দিষ্ট বর্ণনাটি মারফূ হিসেবে সহীহ নয়।"},"heading":{"title":"সলাত নিয়ে বাতিল হাদিস: সলাত দূরত্ব বাড়ায় কি?","description":"এই বর্ণনায় বলা হয়েছে, যে ব্যক্তির সলাত তাকে অশ্লীল ও মন্দ কাজ থেকে বিরত করে না, আল্লাহর কাছ থেকে তার দূরত্বই বাড়ে। কিন্তু প্রদত্ত লেখায় স্পষ্ট বলা হয়েছে, হাদিসটি বাতিল; সনদ ও ভাষা উভয় দিক থেকেই এটি সহীহ নয়। এখানে মূল শিক্ষা হলো—সলাতের গুরুত্ব ঠিক রাখতে হবে, কিন্তু দুর্বল বা বাতিল বর্ণনা দিয়ে ভয় দেখানো ঠিক নয়। লেখায় বলা হয়েছে, বর্ণনাটির কিছু কথা সাহাবী বা হাসান বসরীর কথা হিসেবে এসেছে, কিন্তু রাসূল صلى الله عليه وسلم-এর বাণী হিসেবে সাব্যস্ত নয়। একই সঙ্গে কুরআনের আয়াত উল্লেখ করা হয়েছে যে সলাত নির্লজ্জ ও মন্দ কাজ থেকে বিরত রাখে। তাই সলাতের প্রভাব অস্বীকার করা যাবে না, আবার এই নির্দিষ্ট বাক্যকে সহীহ হাদিসও বলা যাবে না। “সলাত গুনাহ থেকে বিরত রাখে” বিষয়টি বুঝতে হলে সহীহ দলিলের ওপর নির্ভর করা জরুরি।"},"teachings":["সলাতের মর্যাদা বুঝাতে সহীহ দলিল ব্যবহার করা উচিত।","প্রচলিত কোনো কথা হাদিস হিসেবে বিখ্যাত হলেও তা সহীহ নাও হতে পারে।","সলাত মানুষকে মন্দ কাজ থেকে ফিরাতে সাহায্য করে—এটি কুরআনের শিক্ষা।","সাহাবীর কথা ও রাসূল صلى الله عليه وسلم-এর হাদিস—দুটির মর্যাদা এক নয়।"],"related_hadiths":[{"id":"526","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"667","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"864","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"}]}</t>
         </is>
       </c>
       <c r="E15" s="4" t="n"/>
@@ -810,7 +814,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | দস্তরখানা ও সবজি নিয়ে জাল হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. দস্তরখানায় সবজি রেখে বিসমিল্লাহ বললে শয়তান দূর হয়—এই বর্ণনাটি বানোয়াট।"},"heading":{"title":"দস্তরখানা ও সবজি নিয়ে জাল হাদিস: বিসমিল্লাহ প্রসঙ্গ","description":"এই বর্ণনায় বলা হয়েছে, দস্তরখানাগুলো সবজি দিয়ে সাজাও, কারণ বিসমিল্লাহ বলে আহার করলে তা শয়তান বিতাড়নকারী যন্ত্র। প্রদত্ত আলোচনায় হাদিসটি বানোয়াট বলা হয়েছে। এর সনদে আলা ইবনু মাসলামা নামের একজন বর্ণনাকারীর সমস্যা উল্লেখ করা হয়েছে। ইবনু হিব্বান বলেছেন, তিনি নির্ভরযোগ্যদের নামে হাদিস জাল করতেন এবং তার দ্বারা দলিল গ্রহণ করা হালাল নয়। আরেক সূত্রেও হাসান ইবনু শাবীবুল মাকতাবের সমস্যা বলা হয়েছে। তাই “দস্তরখানায় সবজি হাদিস” বা “সবজি শয়তান তাড়ায়” এই কথাটি হাদিস হিসেবে শেয়ার করা ঠিক নয়। খাবারের আগে বিসমিল্লাহ বলা অবশ্যই ইসলামের শিক্ষা, কিন্তু সবজি দিয়ে দস্তরখানা সাজানোর এই নির্দিষ্ট দাবি সহীহ নয়।"},"teachings":["খাবারের আগে বিসমিল্লাহ বলা গুরুত্বপূর্ণ, তবে জাল দাবি যোগ করা যাবে না।","দস্তরখানা ও খাবার বিষয়ে প্রচলিত কথাও যাচাই করা দরকার।","জালকারী বর্ণনাকারীর বর্ণনা দলিল নয়।","সুন্নাহ মানতে হলে সহীহ বর্ণনা অনুসরণ করতে হবে।"],"related_hadiths":[{"id":"5376","book_id":"1","label":"Sahih Bukhari"},{"id":"2017","book_id":"2","label":"Sahih Muslim"},{"id":"3767","book_id":"4","label":"Sunan Abu Dawud"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | দস্তরখানা ও সবজি নিয়ে জাল হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. দস্তরখানায় সবজি রেখে বিসমিল্লাহ বললে শয়তান দূর হয়—এই বর্ণনাটি বানোয়াট।"},"heading":{"title":"দস্তরখানা ও সবজি নিয়ে জাল হাদিস: বিসমিল্লাহ প্রসঙ্গ","description":"এই বর্ণনায় বলা হয়েছে, দস্তরখানাগুলো সবজি দিয়ে সাজাও, কারণ বিসমিল্লাহ বলে আহার করলে তা শয়তান বিতাড়নকারী যন্ত্র। প্রদত্ত আলোচনায় হাদিসটি বানোয়াট বলা হয়েছে। এর সনদে আলা ইবনু মাসলামা নামের একজন বর্ণনাকারীর সমস্যা উল্লেখ করা হয়েছে। ইবনু হিব্বান বলেছেন, তিনি নির্ভরযোগ্যদের নামে হাদিস জাল করতেন এবং তার দ্বারা দলিল গ্রহণ করা হালাল নয়। আরেক সূত্রেও হাসান ইবনু শাবীবুল মাকতাবের সমস্যা বলা হয়েছে। তাই “দস্তরখানায় সবজি হাদিস” বা “সবজি শয়তান তাড়ায়” এই কথাটি হাদিস হিসেবে শেয়ার করা ঠিক নয়। খাবারের আগে বিসমিল্লাহ বলা অবশ্যই ইসলামের শিক্ষা, কিন্তু সবজি দিয়ে দস্তরখানা সাজানোর এই নির্দিষ্ট দাবি সহীহ নয়।"},"teachings":["খাবারের আগে বিসমিল্লাহ বলা গুরুত্বপূর্ণ, তবে জাল দাবি যোগ করা যাবে না।","দস্তরখানা ও খাবার বিষয়ে প্রচলিত কথাও যাচাই করা দরকার।","জালকারী বর্ণনাকারীর বর্ণনা দলিল নয়।","সুন্নাহ মানতে হলে সহীহ বর্ণনা অনুসরণ করতে হবে।"],"related_hadiths":[{"id":"5376","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2017","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"3767","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"}]}</t>
         </is>
       </c>
       <c r="E16" s="4" t="n"/>
@@ -833,7 +837,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মনোবল নিয়ে হাদিস নয়","description":"$book_name$ $hadith_number$ - $chapter_name$. পুরুষদের মনোবল পর্বত সরায়—কথাটি সুন্দর শোনালেও হাদিস হিসেবে এর কোনো ভিত্তি পাওয়া যায় না।"},"heading":{"title":"মনোবল নিয়ে প্রচলিত কথা: এটি হাদিস নয়","description":"এই বর্ণনায় বলা হয়েছে, “পুরুষদের ইচ্ছা বা মনোবল পর্বতমালাকে স্থানচ্যুত করতে পারে।” প্রদত্ত আলোচনায় পরিষ্কার বলা হয়েছে, এটি হাদিস নয়। সুন্নাহর গ্রন্থগুলোতে এই কথার কোনো অস্তিত্ব পাওয়া যায়নি বলে উল্লেখ করা হয়েছে। এখানে মূল বিষয় হলো—উৎসহীন কথা হাদিস হিসেবে প্রচার করা থেকে বাঁচা। কোনো কথায় উৎসাহ, সাহস বা মনোবলের বার্তা থাকলেও সেটি রাসূল صلى الله عليه وسلم-এর নামে বলা যাবে না, যদি সহীহ সনদ না থাকে। লেখায় শাইখ আহমাদ গাযালীর উদ্ধৃতির কথা এসেছে, কিন্তু সেটি হাদিস প্রমাণের জন্য যথেষ্ট নয় বলে বলা হয়েছে। তাই “মনোবল সম্পর্কে হাদিস” খোঁজার সময় এই বর্ণনাকে গ্রহণযোগ্য হাদিস বলা ঠিক হবে না। ইসলাম সত্য কথা বলতে শেখায়, বিশেষ করে নবী صلى الله عليه وسلم-এর নামে কথা বলার ক্ষেত্রে আরও বেশি সাবধান হতে বলে।"},"teachings":["উৎস না থাকলে কোনো কথাকে হাদিস বলা যাবে না।","উৎসাহমূলক বাক্য হলেও তা রাসূল صلى الله عليه وسلم-এর নামে চালানো ঠিক নয়।","হাদিস প্রমাণের জন্য নির্ভরযোগ্য সনদ দরকার।","প্রচলিত বাণী আর সহীহ হাদিস এক জিনিস নয়।"],"related_hadiths":[{"id":"6463","book_id":"1","label":"Sahih Bukhari"},{"id":"2664","book_id":"2","label":"Sahih Muslim"},{"id":"2517","book_id":"5","label":"Jami at-Tirmidhi"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মনোবল নিয়ে হাদিস নয়","description":"$book_name$ $hadith_number$ - $chapter_name$. পুরুষদের মনোবল পর্বত সরায়—কথাটি সুন্দর শোনালেও হাদিস হিসেবে এর কোনো ভিত্তি পাওয়া যায় না।"},"heading":{"title":"মনোবল নিয়ে প্রচলিত কথা: এটি হাদিস নয়","description":"এই বর্ণনায় বলা হয়েছে, “পুরুষদের ইচ্ছা বা মনোবল পর্বতমালাকে স্থানচ্যুত করতে পারে।” প্রদত্ত আলোচনায় পরিষ্কার বলা হয়েছে, এটি হাদিস নয়। সুন্নাহর গ্রন্থগুলোতে এই কথার কোনো অস্তিত্ব পাওয়া যায়নি বলে উল্লেখ করা হয়েছে। এখানে মূল বিষয় হলো—উৎসহীন কথা হাদিস হিসেবে প্রচার করা থেকে বাঁচা। কোনো কথায় উৎসাহ, সাহস বা মনোবলের বার্তা থাকলেও সেটি রাসূল صلى الله عليه وسلم-এর নামে বলা যাবে না, যদি সহীহ সনদ না থাকে। লেখায় শাইখ আহমাদ গাযালীর উদ্ধৃতির কথা এসেছে, কিন্তু সেটি হাদিস প্রমাণের জন্য যথেষ্ট নয় বলে বলা হয়েছে। তাই “মনোবল সম্পর্কে হাদিস” খোঁজার সময় এই বর্ণনাকে গ্রহণযোগ্য হাদিস বলা ঠিক হবে না। ইসলাম সত্য কথা বলতে শেখায়, বিশেষ করে নবী صلى الله عليه وسلم-এর নামে কথা বলার ক্ষেত্রে আরও বেশি সাবধান হতে বলে।"},"teachings":["উৎস না থাকলে কোনো কথাকে হাদিস বলা যাবে না।","উৎসাহমূলক বাক্য হলেও তা রাসূল صلى الله عليه وسلم-এর নামে চালানো ঠিক নয়।","হাদিস প্রমাণের জন্য নির্ভরযোগ্য সনদ দরকার।","প্রচলিত বাণী আর সহীহ হাদিস এক জিনিস নয়।"],"related_hadiths":[{"id":"6463","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2664","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"2517","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"}]}</t>
         </is>
       </c>
       <c r="E17" s="4" t="n"/>
@@ -856,7 +860,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মসজিদে কথা বলা নিয়ে ভিত্তিহীন হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. মসজিদে কথাবার্তা নেকি খেয়ে ফেলে—এই প্রচলিত কথাটির কোনো নির্ভরযোগ্য ভিত্তি নেই।"},"heading":{"title":"মসজিদে কথা বলা নিয়ে ভিত্তিহীন হাদিসের সতর্কতা","description":"এই বর্ণনায় বলা হয়েছে, মসজিদের মধ্যে কথোপকথন সৎ কাজগুলোকে খেয়ে ফেলে, যেমন পশু ঘাস খায়। প্রদত্ত লেখায় স্পষ্ট বলা হয়েছে, হাদিসটির কোনো ভিত্তি নেই। গাযালী এটি “আল-ইহইয়া” গ্রন্থে উল্লেখ করলেও হাফিয ইরাকী, ইবনু হাজার এবং সুবকী এর কোনো সনদ পাননি বলে আলোচনা এসেছে। তাই “মসজিদে কথা বলা নেকি খায়” কথাটি হাদিস হিসেবে বলা নিরাপদ নয়। অবশ্য মসজিদের আদব রক্ষা করা জরুরি—এটি সাধারণ ইসলামী শিক্ষা। কিন্তু এই নির্দিষ্ট বাক্যকে রাসূল صلى الله عليه وسلم-এর নামে বলা যাবে না। মসজিদে অপ্রয়োজনীয় কথা, বাজারের মতো হৈচৈ বা অন্যের ইবাদতে বাধা দেওয়া ভালো নয়—এ কথা বোঝানো যায়; তবে ভিত্তিহীন হাদিস দিয়ে নয়। একজন সচেতন মুসলিমের কাজ হলো মসজিদের সম্মান রাখা এবং একই সঙ্গে হাদিস যাচাই করা।"},"teachings":["মসজিদের আদব রক্ষা করতে হবে, তবে ভিত্তিহীন হাদিস দিয়ে নয়।","কোনো গ্রন্থে থাকা মানেই বর্ণনাটি সহীহ—এমন নয়।","সনদ না থাকলে হাদিস হিসেবে প্রচার করা উচিত নয়।","মসজিদে কথা বলার বিষয়ে ভারসাম্য রাখা দরকার।"],"related_hadiths":[{"id":"568","book_id":"2","label":"Sahih Muslim"},{"id":"1079","book_id":"4","label":"Sunan Abu Dawud"},{"id":"771","book_id":"6","label":"Sunan Ibn Majah"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মসজিদে কথা বলা নিয়ে ভিত্তিহীন হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. মসজিদে কথাবার্তা নেকি খেয়ে ফেলে—এই প্রচলিত কথাটির কোনো নির্ভরযোগ্য ভিত্তি নেই।"},"heading":{"title":"মসজিদে কথা বলা নিয়ে ভিত্তিহীন হাদিসের সতর্কতা","description":"এই বর্ণনায় বলা হয়েছে, মসজিদের মধ্যে কথোপকথন সৎ কাজগুলোকে খেয়ে ফেলে, যেমন পশু ঘাস খায়। প্রদত্ত লেখায় স্পষ্ট বলা হয়েছে, হাদিসটির কোনো ভিত্তি নেই। গাযালী এটি “আল-ইহইয়া” গ্রন্থে উল্লেখ করলেও হাফিয ইরাকী, ইবনু হাজার এবং সুবকী এর কোনো সনদ পাননি বলে আলোচনা এসেছে। তাই “মসজিদে কথা বলা নেকি খায়” কথাটি হাদিস হিসেবে বলা নিরাপদ নয়। অবশ্য মসজিদের আদব রক্ষা করা জরুরি—এটি সাধারণ ইসলামী শিক্ষা। কিন্তু এই নির্দিষ্ট বাক্যকে রাসূল صلى الله عليه وسلم-এর নামে বলা যাবে না। মসজিদে অপ্রয়োজনীয় কথা, বাজারের মতো হৈচৈ বা অন্যের ইবাদতে বাধা দেওয়া ভালো নয়—এ কথা বোঝানো যায়; তবে ভিত্তিহীন হাদিস দিয়ে নয়। একজন সচেতন মুসলিমের কাজ হলো মসজিদের সম্মান রাখা এবং একই সঙ্গে হাদিস যাচাই করা।"},"teachings":["মসজিদের আদব রক্ষা করতে হবে, তবে ভিত্তিহীন হাদিস দিয়ে নয়।","কোনো গ্রন্থে থাকা মানেই বর্ণনাটি সহীহ—এমন নয়।","সনদ না থাকলে হাদিস হিসেবে প্রচার করা উচিত নয়।","মসজিদে কথা বলার বিষয়ে ভারসাম্য রাখা দরকার।"],"related_hadiths":[{"id":"568","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"1079","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"771","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
         </is>
       </c>
       <c r="E18" s="4" t="n"/>
@@ -879,7 +883,7 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আল্লাহর জন্য ত্যাগের বর্ণনা","description":"$book_name$ $hadith_number$ - $chapter_name$. এই ভাষার বর্ণনাটি বানোয়াট, তবে আল্লাহর জন্য কিছু ত্যাগের অর্থ সহীহ সূত্রে অন্য ভাষায় এসেছে।"},"heading":{"title":"আল্লাহর জন্য কিছু ত্যাগ করলে—কোন ভাষা সহীহ?","description":"এই বর্ণনায় বলা হয়েছে, কোনো বান্দা আল্লাহর সন্তুষ্টির জন্য কিছু ত্যাগ করলে আল্লাহ তাকে দ্বীন ও দুনিয়ায় তার চেয়ে উত্তম প্রতিদান দেন। প্রদত্ত আলোচনায় বলা হয়েছে, এই ভাষায় হাদিসটি বানোয়াট। অর্থাৎ বাক্যটি যেভাবে প্রচলিত, সেই নির্দিষ্ট ভাষায় এটি গ্রহণযোগ্য নয়। তবে লেখায় আরও বলা হয়েছে, “তুমি আল্লাহর উদ্দেশ্যে কিছু ত্যাগ করলে আল্লাহ তোমাকে তার চেয়ে উত্তম কিছু দান করবেন”—এই অর্থের একটি বর্ণনার সনদ সহীহ। তাই এখানে খুব সূক্ষ্ম একটি শিক্ষা আছে: ভালো অর্থ থাকলেও নির্দিষ্ট শব্দকে সহীহ হাদিস বলা যাবে কি না, তা যাচাই করতে হয়। “আল্লাহর জন্য ত্যাগ” একটি গুরুত্বপূর্ণ আমল, কিন্তু জাল ভাষা ব্যবহার না করে সহীহ ভাষা ব্যবহার করা ভালো। মুসলিমের সতর্কতা হলো—অর্থ ভালো হলেও উৎস ঠিক আছে কি না দেখা।"},"teachings":["হাদিসের অর্থ ভালো হলেও নির্দিষ্ট ভাষা যাচাই করা জরুরি।","আল্লাহর জন্য কিছু ত্যাগ করা প্রশংসনীয় আমল।","বানোয়াট ভাষা বাদ দিয়ে সহীহ বর্ণনা ব্যবহার করা উচিত।","ধর্মীয় কথা বলার সময় শব্দ ও সূত্র দুটোই গুরুত্বপূর্ণ।"],"related_hadiths":[{"id":"588","book_id":"8","label":"Riyadus Salihin"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আল্লাহর জন্য ত্যাগের বর্ণনা","description":"$book_name$ $hadith_number$ - $chapter_name$. এই ভাষার বর্ণনাটি বানোয়াট, তবে আল্লাহর জন্য কিছু ত্যাগের অর্থ সহীহ সূত্রে অন্য ভাষায় এসেছে।"},"heading":{"title":"আল্লাহর জন্য কিছু ত্যাগ করলে—কোন ভাষা সহীহ?","description":"এই বর্ণনায় বলা হয়েছে, কোনো বান্দা আল্লাহর সন্তুষ্টির জন্য কিছু ত্যাগ করলে আল্লাহ তাকে দ্বীন ও দুনিয়ায় তার চেয়ে উত্তম প্রতিদান দেন। প্রদত্ত আলোচনায় বলা হয়েছে, এই ভাষায় হাদিসটি বানোয়াট। অর্থাৎ বাক্যটি যেভাবে প্রচলিত, সেই নির্দিষ্ট ভাষায় এটি গ্রহণযোগ্য নয়। তবে লেখায় আরও বলা হয়েছে, “তুমি আল্লাহর উদ্দেশ্যে কিছু ত্যাগ করলে আল্লাহ তোমাকে তার চেয়ে উত্তম কিছু দান করবেন”—এই অর্থের একটি বর্ণনার সনদ সহীহ। তাই এখানে খুব সূক্ষ্ম একটি শিক্ষা আছে: ভালো অর্থ থাকলেও নির্দিষ্ট শব্দকে সহীহ হাদিস বলা যাবে কি না, তা যাচাই করতে হয়। “আল্লাহর জন্য ত্যাগ” একটি গুরুত্বপূর্ণ আমল, কিন্তু জাল ভাষা ব্যবহার না করে সহীহ ভাষা ব্যবহার করা ভালো। মুসলিমের সতর্কতা হলো—অর্থ ভালো হলেও উৎস ঠিক আছে কি না দেখা।"},"teachings":["হাদিসের অর্থ ভালো হলেও নির্দিষ্ট ভাষা যাচাই করা জরুরি।","আল্লাহর জন্য কিছু ত্যাগ করা প্রশংসনীয় আমল।","বানোয়াট ভাষা বাদ দিয়ে সহীহ বর্ণনা ব্যবহার করা উচিত।","ধর্মীয় কথা বলার সময় শব্দ ও সূত্র দুটোই গুরুত্বপূর্ণ।"],"related_hadiths":[{"id":"588","book_id":"8","slug":"riyadus-salihin","label":"রিয়াদুস সালেহীন"}]}</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
@@ -906,7 +910,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ধূলিকণা নিয়ে ভিত্তিহীন বর্ণনা","description":"$book_name$ $hadith_number$ - $chapter_name$. ধূলিকণা থেকে জীবাণু সৃষ্টি হয়—এই কথাটি মারফূ হাদিস হিসেবে ভিত্তিহীন বলা হয়েছে।"},"heading":{"title":"ধূলিকণা নিয়ে ভিত্তিহীন হাদিস: জীবাণু প্রসঙ্গে সতর্কতা","description":"এই বর্ণনায় বলা হয়েছে, “ধূলিকণা হতে বেঁচে চল, কারণ ধূলিকণা হতেই জীবাণু সৃষ্টি হয়।” প্রদত্ত আলোচনায় বলা হয়েছে, হাদিসটির কোনো ভিত্তি নেই। ইবনুল আসীর এটি উল্লেখ করলেও মারফূ হিসেবে এর ভিত্তি জানা নেই বলে আলোচনা এসেছে। আমর ইবনুল আস রা. থেকে মাওকূফভাবে একটি বর্ণনার কথা বলা হয়েছে, কিন্তু সেটিও সনদের দিক থেকে সহীহ নয় বলে কয়েকটি কারণ উল্লেখ করা হয়েছে। এখানে মূল শিক্ষা হলো—স্বাস্থ্য বা পরিচ্ছন্নতা বিষয়ে কোনো কথা শুনলেই সেটিকে নবী صلى الله عليه وسلم-এর হাদিস বলা যাবে না। ইসলাম পরিচ্ছন্নতা পছন্দ করে—এটি আলাদা বিষয়; কিন্তু এই নির্দিষ্ট বাক্যকে সহীহ হাদিস হিসেবে প্রচার করা ঠিক নয়। “ধূলিকণা সম্পর্কে হাদিস” খোঁজার সময় বর্ণনার মান বোঝা জরুরি।"},"teachings":["স্বাস্থ্যবিষয়ক কথাও হাদিস হিসেবে বলার আগে যাচাই দরকার।","মারফূ হাদিস ও সাহাবীর কথা আলাদা বিষয়।","মাওকূফ বর্ণনাও সনদে দুর্বল হতে পারে।","পরিচ্ছন্নতার শিক্ষা দিতে ভিত্তিহীন বর্ণনা ব্যবহার করা উচিত নয়।"],"related_hadiths":[{"id":"223","book_id":"2","label":"Sahih Muslim"},{"id":"2799","book_id":"5","label":"Jami at-Tirmidhi"},{"id":"4012","book_id":"4","label":"Sunan Abu Dawud"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ধূলিকণা নিয়ে ভিত্তিহীন বর্ণনা","description":"$book_name$ $hadith_number$ - $chapter_name$. ধূলিকণা থেকে জীবাণু সৃষ্টি হয়—এই কথাটি মারফূ হাদিস হিসেবে ভিত্তিহীন বলা হয়েছে।"},"heading":{"title":"ধূলিকণা নিয়ে ভিত্তিহীন হাদিস: জীবাণু প্রসঙ্গে সতর্কতা","description":"এই বর্ণনায় বলা হয়েছে, “ধূলিকণা হতে বেঁচে চল, কারণ ধূলিকণা হতেই জীবাণু সৃষ্টি হয়।” প্রদত্ত আলোচনায় বলা হয়েছে, হাদিসটির কোনো ভিত্তি নেই। ইবনুল আসীর এটি উল্লেখ করলেও মারফূ হিসেবে এর ভিত্তি জানা নেই বলে আলোচনা এসেছে। আমর ইবনুল আস রা. থেকে মাওকূফভাবে একটি বর্ণনার কথা বলা হয়েছে, কিন্তু সেটিও সনদের দিক থেকে সহীহ নয় বলে কয়েকটি কারণ উল্লেখ করা হয়েছে। এখানে মূল শিক্ষা হলো—স্বাস্থ্য বা পরিচ্ছন্নতা বিষয়ে কোনো কথা শুনলেই সেটিকে নবী صلى الله عليه وسلم-এর হাদিস বলা যাবে না। ইসলাম পরিচ্ছন্নতা পছন্দ করে—এটি আলাদা বিষয়; কিন্তু এই নির্দিষ্ট বাক্যকে সহীহ হাদিস হিসেবে প্রচার করা ঠিক নয়। “ধূলিকণা সম্পর্কে হাদিস” খোঁজার সময় বর্ণনার মান বোঝা জরুরি।"},"teachings":["স্বাস্থ্যবিষয়ক কথাও হাদিস হিসেবে বলার আগে যাচাই দরকার।","মারফূ হাদিস ও সাহাবীর কথা আলাদা বিষয়।","মাওকূফ বর্ণনাও সনদে দুর্বল হতে পারে।","পরিচ্ছন্নতার শিক্ষা দিতে ভিত্তিহীন বর্ণনা ব্যবহার করা উচিত নয়।"],"related_hadiths":[{"id":"223","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"2799","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"4012","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"}]}</t>
         </is>
       </c>
       <c r="E20" s="4" t="n"/>
@@ -929,7 +933,7 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সাহাবীদের নক্ষত্রতুল্য বলা—জাল হাদিসের সতর্কতা","description":"$book_name$ $hadith_number$ - $chapter_name$. সাহাবীদের নক্ষত্রতুল্য বলে যে বর্ণনা প্রচলিত, এখানে সেটিকে জাল বলা হয়েছে; তাই সম্মান থাকবে, কিন্তু দলীল হবে সহীহ হাদিস।"},"heading":{"title":"সাহাবীদের মর্যাদা ও জাল হাদিস যাচাই","description":"এই বর্ণনায় বলা হয়েছে, সাহাবীগণ নক্ষত্রের মতো; তাঁদের যে কারো কথা নিলে হিদায়াত পাওয়া যাবে। কিন্তু প্রদত্ত তাহকীক অনুযায়ী হাদিসটি জাল। আলোচনায় হামযা যাযারীসহ কয়েকজন বর্ণনাকারীর দুর্বলতা, জাল বর্ণনার অভিযোগ এবং ইবনু আব্দিল বার ও ইবনু হাযমের আপত্তি উল্লেখ করা হয়েছে। মূল শিক্ষা হলো, সাহাবীদের প্রতি সম্মান রাখা জরুরি, কিন্তু শরীয়তের দলীল বানাতে হলে কুরআন ও রাসূল সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম থেকে সহীহভাবে প্রমাণিত সুন্নাহকে সামনে রাখতে হবে। কারো প্রতি ভালোবাসা দেখাতে গিয়ে “জাল হাদিস” প্রচার করা দ্বীনের খেদমত নয়। মতভেদকে অন্ধভাবে অনুসরণ করার বদলে যাচাই করা জরুরি।"},"teachings":["সাহাবীদের মর্যাদা মানতে হবে, তবে জাল বর্ণনা দিয়ে নয়।","শরীয়তের দলীল কুরআন ও সহীহ সুন্নাহ থেকে নিতে হবে।","কোনো বর্ণনা জনপ্রিয় হলেই তা সহীহ হয় না।","মতভেদের ক্ষেত্রে যাচাই ছাড়া অন্ধ অনুসরণ নিরাপদ নয়।"],"related_hadiths":[{"id":"3861","book_id":"5","label":"Jami at-Tirmidhi"},{"id":"4658","book_id":"4","label":"Sunan Abu Dawud"},{"id":"2659","book_id":"5","label":"Jami at-Tirmidhi"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সাহাবীদের নক্ষত্রতুল্য বলা—জাল হাদিসের সতর্কতা","description":"$book_name$ $hadith_number$ - $chapter_name$. সাহাবীদের নক্ষত্রতুল্য বলে যে বর্ণনা প্রচলিত, এখানে সেটিকে জাল বলা হয়েছে; তাই সম্মান থাকবে, কিন্তু দলীল হবে সহীহ হাদিস।"},"heading":{"title":"সাহাবীদের মর্যাদা ও জাল হাদিস যাচাই","description":"এই বর্ণনায় বলা হয়েছে, সাহাবীগণ নক্ষত্রের মতো; তাঁদের যে কারো কথা নিলে হিদায়াত পাওয়া যাবে। কিন্তু প্রদত্ত তাহকীক অনুযায়ী হাদিসটি জাল। আলোচনায় হামযা যাযারীসহ কয়েকজন বর্ণনাকারীর দুর্বলতা, জাল বর্ণনার অভিযোগ এবং ইবনু আব্দিল বার ও ইবনু হাযমের আপত্তি উল্লেখ করা হয়েছে। মূল শিক্ষা হলো, সাহাবীদের প্রতি সম্মান রাখা জরুরি, কিন্তু শরীয়তের দলীল বানাতে হলে কুরআন ও রাসূল সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম থেকে সহীহভাবে প্রমাণিত সুন্নাহকে সামনে রাখতে হবে। কারো প্রতি ভালোবাসা দেখাতে গিয়ে “জাল হাদিস” প্রচার করা দ্বীনের খেদমত নয়। মতভেদকে অন্ধভাবে অনুসরণ করার বদলে যাচাই করা জরুরি।"},"teachings":["সাহাবীদের মর্যাদা মানতে হবে, তবে জাল বর্ণনা দিয়ে নয়।","শরীয়তের দলীল কুরআন ও সহীহ সুন্নাহ থেকে নিতে হবে।","কোনো বর্ণনা জনপ্রিয় হলেই তা সহীহ হয় না।","মতভেদের ক্ষেত্রে যাচাই ছাড়া অন্ধ অনুসরণ নিরাপদ নয়।"],"related_hadiths":[{"id":"3861","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"4658","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"2659","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"}]}</t>
         </is>
       </c>
       <c r="E21" s="4" t="n"/>
@@ -952,7 +956,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | পরিবারকে নক্ষত্র বলা—জাল বর্ণনার তাহকীক","description":"$book_name$ $hadith_number$ - $chapter_name$. আহলে বাইতকে নক্ষত্রতুল্য বলে অনুসরণের বর্ণনাটি জাল; ভালোবাসা থাকবে, কিন্তু ভিত্তিহীন কথা রাসূলের নামে বলা যাবে না।"},"heading":{"title":"আহলে বাইতের মর্যাদা ও জাল হাদিস যাচাই","description":"এই বর্ণনায় বলা হয়েছে, নবী পরিবারের সদস্যরা নক্ষত্রের মতো, তাঁদের যে কাউকে অনুসরণ করলে সঠিক পথ পাওয়া যাবে। কিন্তু প্রদত্ত পাঠে স্পষ্টভাবে বলা হয়েছে—হাদিসটি জাল। এর সনদে আহমাদ ইবনু ইসহাককে মিথ্যুক বলা হয়েছে এবং আহমাদ ইবনু কাসেম আল-লোকাঈকে দুর্বল বলা হয়েছে। তাই আহলে বাইতের প্রতি ভালোবাসা ও সম্মান থাকা সত্ত্বেও এমন বর্ণনাকে রাসূল সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম-এর কথা বলা ঠিক নয়। মূল বিষয় হলো, আকীদা বা আমলের ক্ষেত্রে আবেগ নয়, প্রমাণ দরকার। যে কথা প্রমাণিত নয়, তা দিয়ে ফজিলত বা অনুসরণের নিয়ম তৈরি করা দ্বীনের ব্যাপারে অসতর্কতা।"},"teachings":["আহলে বাইতের মর্যাদা মানা হবে, কিন্তু জাল হাদিস দিয়ে নয়।","মিথ্যুক বা দুর্বল বর্ণনাকারীর সূত্রে আসা কথা যাচাই করতে হয়।","রাসূলের নামে কথা বলার আগে সনদ ও হুকুম জানা জরুরি।","ভালোবাসা ও অনুসরণ—দুটিই সহীহ দলীলের আলোকে হওয়া উচিত।"],"related_hadiths":[{"id":"3861","book_id":"5","label":"Jami at-Tirmidhi"},{"id":"2659","book_id":"5","label":"Jami at-Tirmidhi"},{"id":"7400","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | পরিবারকে নক্ষত্র বলা—জাল বর্ণনার তাহকীক","description":"$book_name$ $hadith_number$ - $chapter_name$. আহলে বাইতকে নক্ষত্রতুল্য বলে অনুসরণের বর্ণনাটি জাল; ভালোবাসা থাকবে, কিন্তু ভিত্তিহীন কথা রাসূলের নামে বলা যাবে না।"},"heading":{"title":"আহলে বাইতের মর্যাদা ও জাল হাদিস যাচাই","description":"এই বর্ণনায় বলা হয়েছে, নবী পরিবারের সদস্যরা নক্ষত্রের মতো, তাঁদের যে কাউকে অনুসরণ করলে সঠিক পথ পাওয়া যাবে। কিন্তু প্রদত্ত পাঠে স্পষ্টভাবে বলা হয়েছে—হাদিসটি জাল। এর সনদে আহমাদ ইবনু ইসহাককে মিথ্যুক বলা হয়েছে এবং আহমাদ ইবনু কাসেম আল-লোকাঈকে দুর্বল বলা হয়েছে। তাই আহলে বাইতের প্রতি ভালোবাসা ও সম্মান থাকা সত্ত্বেও এমন বর্ণনাকে রাসূল সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম-এর কথা বলা ঠিক নয়। মূল বিষয় হলো, আকীদা বা আমলের ক্ষেত্রে আবেগ নয়, প্রমাণ দরকার। যে কথা প্রমাণিত নয়, তা দিয়ে ফজিলত বা অনুসরণের নিয়ম তৈরি করা দ্বীনের ব্যাপারে অসতর্কতা।"},"teachings":["আহলে বাইতের মর্যাদা মানা হবে, কিন্তু জাল হাদিস দিয়ে নয়।","মিথ্যুক বা দুর্বল বর্ণনাকারীর সূত্রে আসা কথা যাচাই করতে হয়।","রাসূলের নামে কথা বলার আগে সনদ ও হুকুম জানা জরুরি।","ভালোবাসা ও অনুসরণ—দুটিই সহীহ দলীলের আলোকে হওয়া উচিত।"],"related_hadiths":[{"id":"3861","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"2659","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"7400","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E22" s="4" t="n"/>
@@ -975,7 +979,7 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | শীলা খাওয়ার বর্ণনা—মুনকার হাদিসের সতর্কতা","description":"$book_name$ $hadith_number$ - $chapter_name$. শীলাকে খাদ্য-পানীয় নয় বলা মারফূ হাদিস হিসেবে মুনকার; রোজার বিষয়ে ব্যক্তিগত মতকে নববী হাদিস বানানো ঠিক নয়।"},"heading":{"title":"রোজা অবস্থায় শীলা খাওয়া: মুনকার বর্ণনার শিক্ষা","description":"এই বর্ণনায় বলা হয়েছে, শীলা খাদ্যও নয়, পানীয়ও নয়। কিন্তু প্রদত্ত তাহকীক অনুযায়ী মারফূ হিসেবে এটি মুনকার। কারণ আলী ইবনু যায়েদ ইবনু যাদআন দুর্বল এবং তিনি মওকূফ কথাকে মারফূ করে ফেলতেন বলে আলোচনা এসেছে। পাঠে আরও বলা হয়েছে, আনাস রা. থেকে মওকূফভাবে আবূ তালহার ঘটনা সহীহ হলেও সেটি তাঁর ব্যক্তিগত মত; অন্যরা সেই মতের বিরোধিতা করেছেন। তাই রোজা বা সওমের মাসআলা নির্ধারণে ব্যক্তিগত অভিমতকে রাসূলের কথা বানানো যাবে না। এখানে মূল শিক্ষা হলো, রোজা সম্পর্কিত আমলে সহীহ দলীল দরকার, আর মুনকার বর্ণনা দিয়ে সাধারণ বিধান দেওয়া নিরাপদ নয়।"},"teachings":["মওকূফ কথা ও মারফূ হাদিস এক জিনিস নয়।","রোজার বিধান ব্যক্তিগত মতের উপর দাঁড় করানো ঠিক নয়।","দুর্বল বর্ণনাকারীর কারণে হাদিসের হুকুম বদলে যেতে পারে।","সহীহ হিসেবে কোনো ঘটনা থাকলেও তা সবার জন্য বিধান নাও হতে পারে।"],"related_hadiths":[{"id":"2659","book_id":"5","label":"Jami at-Tirmidhi"},{"id":"7400","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | শীলা খাওয়ার বর্ণনা—মুনকার হাদিসের সতর্কতা","description":"$book_name$ $hadith_number$ - $chapter_name$. শীলাকে খাদ্য-পানীয় নয় বলা মারফূ হাদিস হিসেবে মুনকার; রোজার বিষয়ে ব্যক্তিগত মতকে নববী হাদিস বানানো ঠিক নয়।"},"heading":{"title":"রোজা অবস্থায় শীলা খাওয়া: মুনকার বর্ণনার শিক্ষা","description":"এই বর্ণনায় বলা হয়েছে, শীলা খাদ্যও নয়, পানীয়ও নয়। কিন্তু প্রদত্ত তাহকীক অনুযায়ী মারফূ হিসেবে এটি মুনকার। কারণ আলী ইবনু যায়েদ ইবনু যাদআন দুর্বল এবং তিনি মওকূফ কথাকে মারফূ করে ফেলতেন বলে আলোচনা এসেছে। পাঠে আরও বলা হয়েছে, আনাস রা. থেকে মওকূফভাবে আবূ তালহার ঘটনা সহীহ হলেও সেটি তাঁর ব্যক্তিগত মত; অন্যরা সেই মতের বিরোধিতা করেছেন। তাই রোজা বা সওমের মাসআলা নির্ধারণে ব্যক্তিগত অভিমতকে রাসূলের কথা বানানো যাবে না। এখানে মূল শিক্ষা হলো, রোজা সম্পর্কিত আমলে সহীহ দলীল দরকার, আর মুনকার বর্ণনা দিয়ে সাধারণ বিধান দেওয়া নিরাপদ নয়।"},"teachings":["মওকূফ কথা ও মারফূ হাদিস এক জিনিস নয়।","রোজার বিধান ব্যক্তিগত মতের উপর দাঁড় করানো ঠিক নয়।","দুর্বল বর্ণনাকারীর কারণে হাদিসের হুকুম বদলে যেতে পারে।","সহীহ হিসেবে কোনো ঘটনা থাকলেও তা সবার জন্য বিধান নাও হতে পারে।"],"related_hadiths":[{"id":"2659","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"7400","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E23" s="4" t="n"/>
@@ -998,7 +1002,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মেষ শাবক দিয়ে কুরবানী—দুর্বল সনদ ও ব্যাখ্যা","description":"$book_name$ $hadith_number$ - $chapter_name$. মেষ শাবক দিয়ে কুরবানীর বর্ণনার সনদ দুর্বল, তবে পাঠে সহায়ক বর্ণনা ও ছাগলছানা থেকে ভেড়ার পার্থক্য আলোচিত হয়েছে।"},"heading":{"title":"মেষ শাবক দিয়ে কুরবানী: দুর্বল সনদ ও সতর্ক ব্যাখ্যা","description":"এই বর্ণনায় বলা হয়েছে, মেষ শাবক দ্বারা কুরবানী দেওয়া জায়েয। প্রদত্ত তাহকীক অনুযায়ী মূল সনদ দুর্বল, কারণ উম্মু মুহাম্মাদ ইবনু আবী ইয়াহইয়া ও উম্মু বিলাল সম্পর্কে অজ্ঞতার আলোচনা এসেছে। তবে পাঠের শেষে আলবানী বলেন, সনদের দিক দিয়ে বর্ণনাটি সহীহ নয়, কিন্তু অর্থের দিক থেকে উকবা ও মুশাজে’র বর্ণনার সাক্ষ্য আছে। একই সাথে ছাগলছানা দিয়ে কুরবানী সাধারণভাবে যথেষ্ট নয়—এ কথাও বারাআ রা.-এর ঘটনার আলোকে উল্লেখ করা হয়েছে। তাই “এক বছরের ভেড়া” ও “ছাগলছানা” এক করে দেখা যাবে না। কুরবানীর মাসআলায় শব্দের অর্থ, পশুর বয়স এবং সনদ—সবই গুরুত্বপূর্ণ।"},"teachings":["দুর্বল সনদ থাকলেও অর্থ নিয়ে আলেমদের ব্যাখ্যা আলাদা হতে পারে।","মেষ শাবক ও ছাগলছানার বিধান এক নয়।","কুরবানীর পশুর বয়স বুঝতে ভাষা ও দলীল দুটোই জরুরি।","একটি বর্ণনা দুর্বল হলে সহায়ক বর্ণনা আছে কি না দেখা হয়।"],"related_hadiths":[{"id":"1493","book_id":"5","label":"Jami at-Tirmidhi"},{"id":"2659","book_id":"5","label":"Jami at-Tirmidhi"},{"id":"7400","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মেষ শাবক দিয়ে কুরবানী—দুর্বল সনদ ও ব্যাখ্যা","description":"$book_name$ $hadith_number$ - $chapter_name$. মেষ শাবক দিয়ে কুরবানীর বর্ণনার সনদ দুর্বল, তবে পাঠে সহায়ক বর্ণনা ও ছাগলছানা থেকে ভেড়ার পার্থক্য আলোচিত হয়েছে।"},"heading":{"title":"মেষ শাবক দিয়ে কুরবানী: দুর্বল সনদ ও সতর্ক ব্যাখ্যা","description":"এই বর্ণনায় বলা হয়েছে, মেষ শাবক দ্বারা কুরবানী দেওয়া জায়েয। প্রদত্ত তাহকীক অনুযায়ী মূল সনদ দুর্বল, কারণ উম্মু মুহাম্মাদ ইবনু আবী ইয়াহইয়া ও উম্মু বিলাল সম্পর্কে অজ্ঞতার আলোচনা এসেছে। তবে পাঠের শেষে আলবানী বলেন, সনদের দিক দিয়ে বর্ণনাটি সহীহ নয়, কিন্তু অর্থের দিক থেকে উকবা ও মুশাজে’র বর্ণনার সাক্ষ্য আছে। একই সাথে ছাগলছানা দিয়ে কুরবানী সাধারণভাবে যথেষ্ট নয়—এ কথাও বারাআ রা.-এর ঘটনার আলোকে উল্লেখ করা হয়েছে। তাই “এক বছরের ভেড়া” ও “ছাগলছানা” এক করে দেখা যাবে না। কুরবানীর মাসআলায় শব্দের অর্থ, পশুর বয়স এবং সনদ—সবই গুরুত্বপূর্ণ।"},"teachings":["দুর্বল সনদ থাকলেও অর্থ নিয়ে আলেমদের ব্যাখ্যা আলাদা হতে পারে।","মেষ শাবক ও ছাগলছানার বিধান এক নয়।","কুরবানীর পশুর বয়স বুঝতে ভাষা ও দলীল দুটোই জরুরি।","একটি বর্ণনা দুর্বল হলে সহায়ক বর্ণনা আছে কি না দেখা হয়।"],"related_hadiths":[{"id":"1493","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"2659","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"7400","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E24" s="4" t="n"/>
@@ -1021,7 +1025,7 @@
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | নিজেকে চিনলে প্রভুকে চেনা—ভিত্তিহীন কথা","description":"$book_name$ $hadith_number$ - $chapter_name$. নিজেকে চিনলে প্রভুকে চেনা যায়—এ কথাটি জনপ্রিয় হলেও এখানে হাদিস হিসেবে ভিত্তিহীন বলা হয়েছে; তাই এটিকে নববী বাণী বলা যাবে না।"},"heading":{"title":"নিজেকে চিনলে আল্লাহকে চেনা—হাদিস নয়, সতর্কতা","description":"এই বর্ণনায় বলা হয়েছে, যে নিজেকে চিনেছে, সে তার প্রভুকে চিনতে সক্ষম হয়েছে। কিন্তু প্রদত্ত তাহকীক অনুযায়ী এর কোনো ভিত্তি নেই। সাখাবী, নাবাবী, সুয়ূতী, আলী আল-কারী, ইবনু তাইমিয়্যা এবং ফিরোযাবাদীর বক্তব্যে দেখা যায়—এটি রাসূল সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম-এর হাদিস হিসেবে প্রমাণিত নয়। কেউ কেউ এটিকে ইয়াহইয়া ইবনু মুয়ায আর-রাযীর কথা বলেছেন, কেউ ইসরাইলী বর্ণনার দিকে ইঙ্গিত করেছেন। তাই সুন্দর অর্থ মনে হলেই কোনো বাক্যকে হাদিস বলা যাবে না। আত্মশুদ্ধি গুরুত্বপূর্ণ, কিন্তু “হাদিস” শব্দটি ব্যবহার করতে হলে প্রমাণ থাকা দরকার।"},"teachings":["জনপ্রিয় উক্তি সবসময় হাদিস নয়।","ভালো অর্থ থাকলেও রাসূলের নামে প্রমাণ ছাড়া বলা যাবে না।","আত্মশুদ্ধির কথা বলতে হলে উৎস পরিষ্কার করা জরুরি।","হাদিস যাচাই না করলে ভুল কথা দ্বীনের নামে ছড়িয়ে পড়ে।"],"related_hadiths":[{"id":"2659","book_id":"5","label":"Jami at-Tirmidhi"},{"id":"7400","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | নিজেকে চিনলে প্রভুকে চেনা—ভিত্তিহীন কথা","description":"$book_name$ $hadith_number$ - $chapter_name$. নিজেকে চিনলে প্রভুকে চেনা যায়—এ কথাটি জনপ্রিয় হলেও এখানে হাদিস হিসেবে ভিত্তিহীন বলা হয়েছে; তাই এটিকে নববী বাণী বলা যাবে না।"},"heading":{"title":"নিজেকে চিনলে আল্লাহকে চেনা—হাদিস নয়, সতর্কতা","description":"এই বর্ণনায় বলা হয়েছে, যে নিজেকে চিনেছে, সে তার প্রভুকে চিনতে সক্ষম হয়েছে। কিন্তু প্রদত্ত তাহকীক অনুযায়ী এর কোনো ভিত্তি নেই। সাখাবী, নাবাবী, সুয়ূতী, আলী আল-কারী, ইবনু তাইমিয়্যা এবং ফিরোযাবাদীর বক্তব্যে দেখা যায়—এটি রাসূল সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম-এর হাদিস হিসেবে প্রমাণিত নয়। কেউ কেউ এটিকে ইয়াহইয়া ইবনু মুয়ায আর-রাযীর কথা বলেছেন, কেউ ইসরাইলী বর্ণনার দিকে ইঙ্গিত করেছেন। তাই সুন্দর অর্থ মনে হলেই কোনো বাক্যকে হাদিস বলা যাবে না। আত্মশুদ্ধি গুরুত্বপূর্ণ, কিন্তু “হাদিস” শব্দটি ব্যবহার করতে হলে প্রমাণ থাকা দরকার।"},"teachings":["জনপ্রিয় উক্তি সবসময় হাদিস নয়।","ভালো অর্থ থাকলেও রাসূলের নামে প্রমাণ ছাড়া বলা যাবে না।","আত্মশুদ্ধির কথা বলতে হলে উৎস পরিষ্কার করা জরুরি।","হাদিস যাচাই না করলে ভুল কথা দ্বীনের নামে ছড়িয়ে পড়ে।"],"related_hadiths":[{"id":"2659","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"7400","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E25" s="4" t="n"/>
@@ -1044,7 +1048,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ফজরে নির্দিষ্ট সূরা পড়ে চোখ ভালো থাকা—ভিত্তিহীন","description":"$book_name$ $hadith_number$ - $chapter_name$. ফজরে আলাম নাশরাহ ও আলাম তারা পাঠে চোখে ঝাপসা না দেখার বর্ণনার ভিত্তি নেই; কিরাআতে সহীহ সুন্নাহ মানতে হবে।"},"heading":{"title":"ফজরের সলাতে সূরা পাঠ: ভিত্তিহীন ফজিলত থেকে সতর্কতা","description":"এই বর্ণনায় দাবি করা হয়েছে, ফজরের সলাতে সূরা আলাম নাশরাহ ও সূরা আলাম তারা কাইফা পড়লে চোখে ঝাপসা দেখা হবে না। প্রদত্ত তাহকীক অনুযায়ী হাদিসটির কোনো ভিত্তি নেই। সাখাবী বলেছেন, ফজর বলতে সুন্নাত বা ফরয—যেটাই ধরা হোক, এই দাবি প্রমাণিত নয়। বরং পাঠে বলা হয়েছে, ফজরের সুন্নাতে কুল ইয়াআইয়ুহাল কাফিরুন ও কুল হুয়াল্লাহু আহাদ পড়ার সুন্নাহ আছে, আর ফজরের ফরযে দীর্ঘ কিরাআতের কথা এসেছে। তাই চিকিৎসা বা দৃষ্টিশক্তির বিশেষ ফল দাবি করে ভিত্তিহীন আমল প্রচার করা উচিত নয়। নামাজে কিরাআত সহীহ সুন্নাহ অনুযায়ী শেখাই নিরাপদ।"},"teachings":["কোনো সূরা পাঠের বিশেষ ফল দাবি করতে সহীহ দলীল দরকার।","ফজরের সুন্নাত ও ফরযের কিরাআত এক নয়।","চোখের রোগের জন্য ভিত্তিহীন ফজিলত প্রচার করা ঠিক নয়।","ইবাদতে সহীহ সুন্নাহকে আগে জানতে হয়।"],"related_hadiths":[{"id":"2659","book_id":"5","label":"Jami at-Tirmidhi"},{"id":"7400","book_id":"2","label":"Sahih Muslim"},{"id":"599","book_id":"1","label":"Sahih Bukhari"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ফজরে নির্দিষ্ট সূরা পড়ে চোখ ভালো থাকা—ভিত্তিহীন","description":"$book_name$ $hadith_number$ - $chapter_name$. ফজরে আলাম নাশরাহ ও আলাম তারা পাঠে চোখে ঝাপসা না দেখার বর্ণনার ভিত্তি নেই; কিরাআতে সহীহ সুন্নাহ মানতে হবে।"},"heading":{"title":"ফজরের সলাতে সূরা পাঠ: ভিত্তিহীন ফজিলত থেকে সতর্কতা","description":"এই বর্ণনায় দাবি করা হয়েছে, ফজরের সলাতে সূরা আলাম নাশরাহ ও সূরা আলাম তারা কাইফা পড়লে চোখে ঝাপসা দেখা হবে না। প্রদত্ত তাহকীক অনুযায়ী হাদিসটির কোনো ভিত্তি নেই। সাখাবী বলেছেন, ফজর বলতে সুন্নাত বা ফরয—যেটাই ধরা হোক, এই দাবি প্রমাণিত নয়। বরং পাঠে বলা হয়েছে, ফজরের সুন্নাতে কুল ইয়াআইয়ুহাল কাফিরুন ও কুল হুয়াল্লাহু আহাদ পড়ার সুন্নাহ আছে, আর ফজরের ফরযে দীর্ঘ কিরাআতের কথা এসেছে। তাই চিকিৎসা বা দৃষ্টিশক্তির বিশেষ ফল দাবি করে ভিত্তিহীন আমল প্রচার করা উচিত নয়। নামাজে কিরাআত সহীহ সুন্নাহ অনুযায়ী শেখাই নিরাপদ।"},"teachings":["কোনো সূরা পাঠের বিশেষ ফল দাবি করতে সহীহ দলীল দরকার।","ফজরের সুন্নাত ও ফরযের কিরাআত এক নয়।","চোখের রোগের জন্য ভিত্তিহীন ফজিলত প্রচার করা ঠিক নয়।","ইবাদতে সহীহ সুন্নাহকে আগে জানতে হয়।"],"related_hadiths":[{"id":"2659","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"7400","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"599","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
         </is>
       </c>
       <c r="E26" s="4" t="n"/>
@@ -1067,7 +1071,7 @@
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ওযুর পরে সূরা কদর পাঠ—ভিত্তিহীন আমল","description":"$book_name$ $hadith_number$ - $chapter_name$. ওযুর পরে ইন্না আনযালনাহু পড়ার বর্ণনার ভিত্তি নেই; ওযুর পর প্রমাণিত দোয়া পাঠ করাই সুন্নাহর কাছাকাছি।"},"heading":{"title":"ওযুর পর সূরা কদর নয়—সহীহ দোয়ার শিক্ষা","description":"এই বর্ণনায় বলা হয়েছে, ওযূর পরে ইন্না আনযালনাহু সূরা পাঠ করতে হয়। কিন্তু প্রদত্ত তাহকীক অনুযায়ী এর কোনো ভিত্তি নেই। সাখাবী বলেছেন, এটি সহীহ সুন্নাহকে সরিয়ে দেয়। পাঠে আলবানী ব্যাখ্যা করেছেন, ওযুর পরের সুন্নাহ হলো নির্দিষ্ট দোয়া পড়া, যা মুসলিম ও তিরমিযীতে এসেছে; আর আরেকটি দোয়ার কথাও সহীহ সনদে উল্লেখ করা হয়েছে। তাই ওযুর পর আমল শেখার সময় “ওযুর দোয়া” ও “ভিত্তিহীন আমল” আলাদা করা দরকার। কোনো বইয়ে পাওয়া গেলেই সেটি নববী সুন্নাহ হয়ে যায় না। পবিত্রতা অর্জনের ইবাদতকে সহীহ প্রমাণের উপর রাখা উত্তম।"},"teachings":["ওযুর পর কোন দোয়া পড়তে হবে তা সহীহ সূত্রে জানা উচিত।","সূরা কদর পাঠকে ওযুর পরের সুন্নাহ বলা প্রমাণিত নয়।","একটি আমল প্রচলিত হলেই তা হাদিস নয়।","সহীহ সুন্নাহ বাদ দিয়ে ভিত্তিহীন আমল ধরার ঝুঁকি আছে।"],"related_hadiths":[{"id":"234b","book_id":"2","label":"Sahih Muslim"},{"id":"2659","book_id":"5","label":"Jami at-Tirmidhi"},{"id":"7400","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ওযুর পরে সূরা কদর পাঠ—ভিত্তিহীন আমল","description":"$book_name$ $hadith_number$ - $chapter_name$. ওযুর পরে ইন্না আনযালনাহু পড়ার বর্ণনার ভিত্তি নেই; ওযুর পর প্রমাণিত দোয়া পাঠ করাই সুন্নাহর কাছাকাছি।"},"heading":{"title":"ওযুর পর সূরা কদর নয়—সহীহ দোয়ার শিক্ষা","description":"এই বর্ণনায় বলা হয়েছে, ওযূর পরে ইন্না আনযালনাহু সূরা পাঠ করতে হয়। কিন্তু প্রদত্ত তাহকীক অনুযায়ী এর কোনো ভিত্তি নেই। সাখাবী বলেছেন, এটি সহীহ সুন্নাহকে সরিয়ে দেয়। পাঠে আলবানী ব্যাখ্যা করেছেন, ওযুর পরের সুন্নাহ হলো নির্দিষ্ট দোয়া পড়া, যা মুসলিম ও তিরমিযীতে এসেছে; আর আরেকটি দোয়ার কথাও সহীহ সনদে উল্লেখ করা হয়েছে। তাই ওযুর পর আমল শেখার সময় “ওযুর দোয়া” ও “ভিত্তিহীন আমল” আলাদা করা দরকার। কোনো বইয়ে পাওয়া গেলেই সেটি নববী সুন্নাহ হয়ে যায় না। পবিত্রতা অর্জনের ইবাদতকে সহীহ প্রমাণের উপর রাখা উত্তম।"},"teachings":["ওযুর পর কোন দোয়া পড়তে হবে তা সহীহ সূত্রে জানা উচিত।","সূরা কদর পাঠকে ওযুর পরের সুন্নাহ বলা প্রমাণিত নয়।","একটি আমল প্রচলিত হলেই তা হাদিস নয়।","সহীহ সুন্নাহ বাদ দিয়ে ভিত্তিহীন আমল ধরার ঝুঁকি আছে।"],"related_hadiths":[{"id":"234b","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"2659","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"7400","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E27" s="4" t="n"/>
@@ -1090,7 +1094,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | গর্দান মাসাহ ও বন্দি থেকে নিরাপত্তা—জাল হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. গর্দান মাসাহ করলে বন্দি হওয়া থেকে নিরাপত্তা মেলে—এ বর্ণনা জাল; ওযুর পদ্ধতি সহীহ হাদিস অনুযায়ী জানা দরকার।"},"heading":{"title":"গর্দান মাসাহ: ওযুর নামে জাল বর্ণনা থেকে সতর্কতা","description":"এই বর্ণনায় বলা হয়েছে, গর্দান মাসাহ করা বন্দি হওয়া থেকে নিরাপত্তা দেয়। প্রদত্ত তাহকীক অনুযায়ী হাদিসটি জাল; নাবাবী স্পষ্ট বলেছেন, এটি নবী সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম-এর কথা নয়। আলোচনায় বিভিন্ন সনদের দুর্বলতা, মাসউদীর স্মৃতির সমস্যা, মুহাম্মাদ ইবনু আমর আল-আনসারী ও অন্য বর্ণনাকারীর দুর্বলতার কথা এসেছে। আরও গুরুত্বপূর্ণ হলো, সহীহ হাদিসগুলোতে বর্ণিত ওযুর পদ্ধতিতে গর্দান মাসাহ করার কথা নেই। তাই “গর্দান মাসাহের ফজিলত” নামে কোনো নিরাপত্তার প্রতিশ্রুতি প্রচার করা ঠিক নয়। ওযু একটি ইবাদত; এতে নবীজির প্রমাণিত পদ্ধতি অনুসরণ করাই মূল।"},"teachings":["ওযুর পদ্ধতি সহীহ হাদিস থেকে নিতে হবে।","গর্দান মাসাহের বিশেষ ফজিলত জাল বর্ণনা দিয়ে প্রমাণিত নয়।","ইবাদতে বাড়তি কাজ যোগ করার আগে দলীল দেখা জরুরি।","নবীজির নামে জাল প্রতিশ্রুতি প্রচার করা বিপজ্জনক।"],"related_hadiths":[{"id":"234b","book_id":"2","label":"Sahih Muslim"},{"id":"2659","book_id":"5","label":"Jami at-Tirmidhi"},{"id":"7400","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | গর্দান মাসাহ ও বন্দি থেকে নিরাপত্তা—জাল হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. গর্দান মাসাহ করলে বন্দি হওয়া থেকে নিরাপত্তা মেলে—এ বর্ণনা জাল; ওযুর পদ্ধতি সহীহ হাদিস অনুযায়ী জানা দরকার।"},"heading":{"title":"গর্দান মাসাহ: ওযুর নামে জাল বর্ণনা থেকে সতর্কতা","description":"এই বর্ণনায় বলা হয়েছে, গর্দান মাসাহ করা বন্দি হওয়া থেকে নিরাপত্তা দেয়। প্রদত্ত তাহকীক অনুযায়ী হাদিসটি জাল; নাবাবী স্পষ্ট বলেছেন, এটি নবী সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম-এর কথা নয়। আলোচনায় বিভিন্ন সনদের দুর্বলতা, মাসউদীর স্মৃতির সমস্যা, মুহাম্মাদ ইবনু আমর আল-আনসারী ও অন্য বর্ণনাকারীর দুর্বলতার কথা এসেছে। আরও গুরুত্বপূর্ণ হলো, সহীহ হাদিসগুলোতে বর্ণিত ওযুর পদ্ধতিতে গর্দান মাসাহ করার কথা নেই। তাই “গর্দান মাসাহের ফজিলত” নামে কোনো নিরাপত্তার প্রতিশ্রুতি প্রচার করা ঠিক নয়। ওযু একটি ইবাদত; এতে নবীজির প্রমাণিত পদ্ধতি অনুসরণ করাই মূল।"},"teachings":["ওযুর পদ্ধতি সহীহ হাদিস থেকে নিতে হবে।","গর্দান মাসাহের বিশেষ ফজিলত জাল বর্ণনা দিয়ে প্রমাণিত নয়।","ইবাদতে বাড়তি কাজ যোগ করার আগে দলীল দেখা জরুরি।","নবীজির নামে জাল প্রতিশ্রুতি প্রচার করা বিপজ্জনক।"],"related_hadiths":[{"id":"234b","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"2659","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"7400","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E28" s="4" t="n"/>
@@ -1113,7 +1117,7 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | শিরক ও ক্ষতি নিয়ে ভিত্তিহীন হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. শিরক ও মানুষের ক্ষতি থেকে বাঁচার কথা সত্য, তবে এই নির্দিষ্ট বাক্যের কোনো ভিত্তি নেই।"},"heading":{"title":"শিরক ও মানুষের ক্ষতি নিয়ে ভিত্তিহীন বর্ণনার হুকুম","description":"এই বর্ণনায় বলা হয়েছে, “দু’টি বস্তুর নিকটবর্তী হয়ো না—আল্লাহর সাথে শরীক করা এবং মানুষের ক্ষতি করা।” কথাটির অর্থ ভালো মনে হলেও প্রদত্ত আলোচনায় বলা হয়েছে, হাদিসটির কোনো ভিত্তি নেই। সুন্নাহর গ্রন্থে এর ভিত্তি পাওয়া যায়নি বলে উল্লেখ করা হয়েছে। সম্ভবত এটি কিছু গ্রন্থে প্রচলিত কথিত বর্ণনা থেকে এসেছে, কিন্তু সনদ পাওয়া যায়নি। এখানে মূল বিষয় হলো—শিরক থেকে বাঁচা এবং মানুষের ক্ষতি না করা অবশ্যই বড় ইসলামী শিক্ষা; কিন্তু এই নির্দিষ্ট বাক্যকে হাদিস বলা ঠিক নয়। “শিরক ও মানুষের ক্ষতি হাদিস” নামে কোনো পোস্ট বা লেখা শেয়ার করার আগে উৎস দেখা দরকার। ভালো কথা হলেও রাসূল صلى الله عليه وسلم-এর নামে বলার জন্য দলিল দরকার। এতে হাদিসের মর্যাদা রক্ষা হয়।"},"teachings":["শিরক থেকে দূরে থাকা ইসলামের বড় শিক্ষা।","মানুষের ক্ষতি করা থেকে বাঁচা জরুরি।","ভালো অর্থ থাকলেই কোনো কথা হাদিস হয় না।","সনদহীন বর্ণনা রাসূল صلى الله عليه وسلم-এর নামে বলা উচিত নয়।"],"related_hadiths":[{"id":"6018","book_id":"1","label":"Sahih Bukhari"},{"id":"2577","book_id":"2","label":"Sahih Muslim"},{"id":"2340","book_id":"6","label":"Sunan Ibn Majah"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | শিরক ও ক্ষতি নিয়ে ভিত্তিহীন হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. শিরক ও মানুষের ক্ষতি থেকে বাঁচার কথা সত্য, তবে এই নির্দিষ্ট বাক্যের কোনো ভিত্তি নেই।"},"heading":{"title":"শিরক ও মানুষের ক্ষতি নিয়ে ভিত্তিহীন বর্ণনার হুকুম","description":"এই বর্ণনায় বলা হয়েছে, “দু’টি বস্তুর নিকটবর্তী হয়ো না—আল্লাহর সাথে শরীক করা এবং মানুষের ক্ষতি করা।” কথাটির অর্থ ভালো মনে হলেও প্রদত্ত আলোচনায় বলা হয়েছে, হাদিসটির কোনো ভিত্তি নেই। সুন্নাহর গ্রন্থে এর ভিত্তি পাওয়া যায়নি বলে উল্লেখ করা হয়েছে। সম্ভবত এটি কিছু গ্রন্থে প্রচলিত কথিত বর্ণনা থেকে এসেছে, কিন্তু সনদ পাওয়া যায়নি। এখানে মূল বিষয় হলো—শিরক থেকে বাঁচা এবং মানুষের ক্ষতি না করা অবশ্যই বড় ইসলামী শিক্ষা; কিন্তু এই নির্দিষ্ট বাক্যকে হাদিস বলা ঠিক নয়। “শিরক ও মানুষের ক্ষতি হাদিস” নামে কোনো পোস্ট বা লেখা শেয়ার করার আগে উৎস দেখা দরকার। ভালো কথা হলেও রাসূল صلى الله عليه وسلم-এর নামে বলার জন্য দলিল দরকার। এতে হাদিসের মর্যাদা রক্ষা হয়।"},"teachings":["শিরক থেকে দূরে থাকা ইসলামের বড় শিক্ষা।","মানুষের ক্ষতি করা থেকে বাঁচা জরুরি।","ভালো অর্থ থাকলেই কোনো কথা হাদিস হয় না।","সনদহীন বর্ণনা রাসূল صلى الله عليه وسلم-এর নামে বলা উচিত নয়।"],"related_hadiths":[{"id":"6018","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2577","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"2340","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
         </is>
       </c>
       <c r="E29" s="4" t="n"/>
@@ -1136,7 +1140,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | খাওয়ানো-পান করানোর অতিরঞ্জিত ফজিলত—জাল","description":"$book_name$ $hadith_number$ - $chapter_name$. ভাইকে রুটি-পানি খাওয়ালে সাত খন্দক দূরে জাহান্নাম—এ বর্ণনা জাল; দান ও খাদ্যদান নিয়ে প্রমাণিত কথা আলাদা।"},"heading":{"title":"খাদ্যদান ফজিলত: জাল বর্ণনা ও সতর্ক দৃষ্টিভঙ্গি","description":"এই বর্ণনায় বলা হয়েছে, কোনো ভাইকে পরিতৃপ্ত না হওয়া পর্যন্ত রুটি এবং তৃষ্ণা না মেটা পর্যন্ত পানি দিলে আল্লাহ তাকে সাত খন্দক দূর জাহান্নাম থেকে সরিয়ে দেবেন। কিন্তু প্রদত্ত তাহকীক অনুযায়ী হাদিসটি জাল। সনদে রাজা ইবনু আবী আতা নামে এক বর্ণনাকারী আছে, যাকে জাল হাদিসের হোতা বলা হয়েছে। হাকিমের সহীহ বলা এখানে ভুল হিসেবে সমালোচিত হয়েছে। তাই খাদ্যদান ভালো কাজ হলেও এই নির্দিষ্ট পরিমাণ, সাত খন্দক, পাঁচশত বছরের দূরত্ব—এসব দাবি প্রমাণ ছাড়া বলা যাবে না। দ্বীনের ফজিলত বলতে হলে ভাষা মেপে বলা দরকার, যেন মানুষ জাল হাদিসকে সত্য মনে না করে।"},"teachings":["দান-খাদ্যদান ভালো কাজ, তবে জাল ফজিলত বানানো যাবে না।","অতিরঞ্জিত সংখ্যা দেখলেই হাদিস যাচাই করা দরকার।","বর্ণনাকারীর অবস্থা হাদিসের হুকুমে বড় প্রভাব ফেলে।","সহীহ না হলে ফজিলতের দাবি সতর্কভাবে বাদ দিতে হয়।"],"related_hadiths":[{"id":"2659","book_id":"5","label":"Jami at-Tirmidhi"},{"id":"7400","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | খাওয়ানো-পান করানোর অতিরঞ্জিত ফজিলত—জাল","description":"$book_name$ $hadith_number$ - $chapter_name$. ভাইকে রুটি-পানি খাওয়ালে সাত খন্দক দূরে জাহান্নাম—এ বর্ণনা জাল; দান ও খাদ্যদান নিয়ে প্রমাণিত কথা আলাদা।"},"heading":{"title":"খাদ্যদান ফজিলত: জাল বর্ণনা ও সতর্ক দৃষ্টিভঙ্গি","description":"এই বর্ণনায় বলা হয়েছে, কোনো ভাইকে পরিতৃপ্ত না হওয়া পর্যন্ত রুটি এবং তৃষ্ণা না মেটা পর্যন্ত পানি দিলে আল্লাহ তাকে সাত খন্দক দূর জাহান্নাম থেকে সরিয়ে দেবেন। কিন্তু প্রদত্ত তাহকীক অনুযায়ী হাদিসটি জাল। সনদে রাজা ইবনু আবী আতা নামে এক বর্ণনাকারী আছে, যাকে জাল হাদিসের হোতা বলা হয়েছে। হাকিমের সহীহ বলা এখানে ভুল হিসেবে সমালোচিত হয়েছে। তাই খাদ্যদান ভালো কাজ হলেও এই নির্দিষ্ট পরিমাণ, সাত খন্দক, পাঁচশত বছরের দূরত্ব—এসব দাবি প্রমাণ ছাড়া বলা যাবে না। দ্বীনের ফজিলত বলতে হলে ভাষা মেপে বলা দরকার, যেন মানুষ জাল হাদিসকে সত্য মনে না করে।"},"teachings":["দান-খাদ্যদান ভালো কাজ, তবে জাল ফজিলত বানানো যাবে না।","অতিরঞ্জিত সংখ্যা দেখলেই হাদিস যাচাই করা দরকার।","বর্ণনাকারীর অবস্থা হাদিসের হুকুমে বড় প্রভাব ফেলে।","সহীহ না হলে ফজিলতের দাবি সতর্কভাবে বাদ দিতে হয়।"],"related_hadiths":[{"id":"2659","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"7400","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E30" s="4" t="n"/>
@@ -1159,7 +1163,7 @@
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আযানের তাকবীর আলাদা আলাদা বলা—ভিত্তিহীন","description":"$book_name$ $hadith_number$ - $chapter_name$. আযানের তাকবীর পৃথকভাবে বলার বর্ণনার ভিত্তি নেই; সহীহ সুন্নাহতে আযানের তাকবীর জোড়া করে বলার ইঙ্গিত এসেছে।"},"heading":{"title":"আযানের তাকবীর: ভিত্তিহীন পদ্ধতি নয়, সহীহ সুন্নাহ","description":"এই বর্ণনায় বলা হয়েছে, তাকবীর পৃথক পৃথকভাবে হবে—এটি আযানের তাকবীর হিসেবে প্রচলিত করা হয়েছে। কিন্তু প্রদত্ত তাহকীক অনুযায়ী এর কোনো ভিত্তি নেই। হাফিয ইবনু হাজার, সাখাবী ও সুয়ূতী এ কথা বলেছেন। সুয়ূতী এটিকে ইবরাহীম নাখঈর কথা হিসেবে উল্লেখ করেছেন, আর সেখানে সলাতের তাকবীর বোঝানো হয়েছে, আযানের সাথে নয়। পাঠে আরও বলা হয়েছে, মিসরের কিছু লোক এই ধারণায় আযান আলাদাভাবে দেয়, অথচ সুন্নাহতে আযানের তাকবীর জোড়া করে বলার ইঙ্গিত এসেছে। তাই আযানের পদ্ধতি নিয়ে প্রচলন নয়, প্রমাণ দেখা দরকার। আযান মুসলিম সমাজের প্রকাশ্য ইবাদত; এতে ভিত্তিহীন পরিবর্তন ভালো নয়।"},"teachings":["আযানের পদ্ধতি সহীহ সুন্নাহ থেকে নিতে হবে।","সলাতের তাকবীর ও আযানের তাকবীর এক বিষয় নয়।","কোনো অঞ্চলের প্রচলন সুন্নাহর দলীল হতে পারে না।","ইবাদতের প্রকাশ্য রূপে ভিত্তিহীন পরিবর্তন এড়ানো উচিত।"],"related_hadiths":[{"id":"611","book_id":"1","label":"Sahih Bukhari"},{"id":"614","book_id":"1","label":"Sahih Bukhari"},{"id":"2659","book_id":"5","label":"Jami at-Tirmidhi"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আযানের তাকবীর আলাদা আলাদা বলা—ভিত্তিহীন","description":"$book_name$ $hadith_number$ - $chapter_name$. আযানের তাকবীর পৃথকভাবে বলার বর্ণনার ভিত্তি নেই; সহীহ সুন্নাহতে আযানের তাকবীর জোড়া করে বলার ইঙ্গিত এসেছে।"},"heading":{"title":"আযানের তাকবীর: ভিত্তিহীন পদ্ধতি নয়, সহীহ সুন্নাহ","description":"এই বর্ণনায় বলা হয়েছে, তাকবীর পৃথক পৃথকভাবে হবে—এটি আযানের তাকবীর হিসেবে প্রচলিত করা হয়েছে। কিন্তু প্রদত্ত তাহকীক অনুযায়ী এর কোনো ভিত্তি নেই। হাফিয ইবনু হাজার, সাখাবী ও সুয়ূতী এ কথা বলেছেন। সুয়ূতী এটিকে ইবরাহীম নাখঈর কথা হিসেবে উল্লেখ করেছেন, আর সেখানে সলাতের তাকবীর বোঝানো হয়েছে, আযানের সাথে নয়। পাঠে আরও বলা হয়েছে, মিসরের কিছু লোক এই ধারণায় আযান আলাদাভাবে দেয়, অথচ সুন্নাহতে আযানের তাকবীর জোড়া করে বলার ইঙ্গিত এসেছে। তাই আযানের পদ্ধতি নিয়ে প্রচলন নয়, প্রমাণ দেখা দরকার। আযান মুসলিম সমাজের প্রকাশ্য ইবাদত; এতে ভিত্তিহীন পরিবর্তন ভালো নয়।"},"teachings":["আযানের পদ্ধতি সহীহ সুন্নাহ থেকে নিতে হবে।","সলাতের তাকবীর ও আযানের তাকবীর এক বিষয় নয়।","কোনো অঞ্চলের প্রচলন সুন্নাহর দলীল হতে পারে না।","ইবাদতের প্রকাশ্য রূপে ভিত্তিহীন পরিবর্তন এড়ানো উচিত।"],"related_hadiths":[{"id":"611","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"614","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2659","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"}]}</t>
         </is>
       </c>
       <c r="E31" s="4" t="n"/>
@@ -1182,7 +1186,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আল্লাহ আমাকে শিষ্টাচার শিখিয়েছেন—দুর্বল বর্ণনা","description":"$book_name$ $hadith_number$ - $chapter_name$. আল্লাহ আমাকে আদব শিখিয়েছেন—এ বর্ণনার অর্থ ভালো বলা হলেও সনদ জানা যায় না; তাই হাদিস হিসেবে সতর্কতা দরকার।"},"heading":{"title":"নববী আদব ও দুর্বল হাদিসের সীমা","description":"এই বর্ণনায় বলা হয়েছে, আল্লাহ তা’আলা আমাকে শিষ্টাচার শিক্ষা দিয়েছেন, এরপর আমার শিষ্টাচার সুন্দর করেছেন। প্রদত্ত তাহকীক অনুযায়ী হাদিসটি দুর্বল। ইবনু তাইমিয়্যা বলেছেন, এর অর্থ সহীহ, কিন্তু সনদ সম্পর্কে জানা যায় না। সাখাবী ও সুয়ূতী তাঁর কথাকে সমর্থন করেছেন। তাই এখানে ভারসাম্য জরুরি: নবী সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম-এর চরিত্র সর্বোত্তম—এটি ইসলামের প্রতিষ্ঠিত সত্য; কিন্তু এই নির্দিষ্ট বাক্যকে সহীহ হাদিস হিসেবে উদ্ধৃত করা যাবে না। “আদব” ও “আখলাক” শেখানোর সময় দুর্বল বর্ণনাকে স্পষ্টভাবে দুর্বল বলে উল্লেখ করা উচিত। ভালো অর্থ থাকলেই সনদহীন কথাকে নববী বাণী বানানো ঠিক নয়।"},"teachings":["ভালো অর্থ থাকা আর সহীহ সনদ থাকা এক কথা নয়।","নবীজির আদব শেখাতে প্রমাণিত বর্ণনা ব্যবহার করা উত্তম।","দুর্বল হাদিস উদ্ধৃত করলে তার হুকুম বলা উচিত।","চরিত্র গঠনের আলোচনায়ও হাদিস যাচাই জরুরি।"],"related_hadiths":[{"id":"813","book_id":"14","label":"Mishkat al-Masabih"},{"id":"2659","book_id":"5","label":"Jami at-Tirmidhi"},{"id":"7400","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আল্লাহ আমাকে শিষ্টাচার শিখিয়েছেন—দুর্বল বর্ণনা","description":"$book_name$ $hadith_number$ - $chapter_name$. আল্লাহ আমাকে আদব শিখিয়েছেন—এ বর্ণনার অর্থ ভালো বলা হলেও সনদ জানা যায় না; তাই হাদিস হিসেবে সতর্কতা দরকার।"},"heading":{"title":"নববী আদব ও দুর্বল হাদিসের সীমা","description":"এই বর্ণনায় বলা হয়েছে, আল্লাহ তা’আলা আমাকে শিষ্টাচার শিক্ষা দিয়েছেন, এরপর আমার শিষ্টাচার সুন্দর করেছেন। প্রদত্ত তাহকীক অনুযায়ী হাদিসটি দুর্বল। ইবনু তাইমিয়্যা বলেছেন, এর অর্থ সহীহ, কিন্তু সনদ সম্পর্কে জানা যায় না। সাখাবী ও সুয়ূতী তাঁর কথাকে সমর্থন করেছেন। তাই এখানে ভারসাম্য জরুরি: নবী সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম-এর চরিত্র সর্বোত্তম—এটি ইসলামের প্রতিষ্ঠিত সত্য; কিন্তু এই নির্দিষ্ট বাক্যকে সহীহ হাদিস হিসেবে উদ্ধৃত করা যাবে না। “আদব” ও “আখলাক” শেখানোর সময় দুর্বল বর্ণনাকে স্পষ্টভাবে দুর্বল বলে উল্লেখ করা উচিত। ভালো অর্থ থাকলেই সনদহীন কথাকে নববী বাণী বানানো ঠিক নয়।"},"teachings":["ভালো অর্থ থাকা আর সহীহ সনদ থাকা এক কথা নয়।","নবীজির আদব শেখাতে প্রমাণিত বর্ণনা ব্যবহার করা উত্তম।","দুর্বল হাদিস উদ্ধৃত করলে তার হুকুম বলা উচিত।","চরিত্র গঠনের আলোচনায়ও হাদিস যাচাই জরুরি।"],"related_hadiths":[{"id":"813","book_id":"14","slug":"mishkatul-masabih","label":"মিশকাতুল মাসাবীহ"},{"id":"2659","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"7400","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E32" s="4" t="n"/>
@@ -1205,7 +1209,7 @@
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আযানের সময় চোখ মাসাহ—সহীহ নয়","description":"$book_name$ $hadith_number$ - $chapter_name$. আযানে শাহাদাতের সময় আঙুল দিয়ে চোখ মাসাহ করলে শাফাআত অপরিহার্য—এই বর্ণনা সহীহ নয়; প্রমাণিত আযানের জবাবই যথেষ্ট।"},"heading":{"title":"আযানে চোখ মাসাহ: সহীহ নয় এমন ফজিলত","description":"এই বর্ণনায় বলা হয়েছে, মুয়াজ্জিন যখন আশহাদু আন্না মুহাম্মাদার রাসূলুল্লাহ বলে, তখন তর্জনী দিয়ে দুই চোখ মাসাহ করলে রাসূল সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম-এর সুপারিশ অপরিহার্য হবে। কিন্তু প্রদত্ত তাহকীক অনুযায়ী হাদিসটি সহীহ নয়। দাইলামী এটি আবূ বকর রা. থেকে মারফূ হিসেবে উল্লেখ করেছেন, আর ইবনু তাহির, শাওকানী ও সাখাবী একে সহীহ নয় বলেছেন। তাই আযানের সময় চোখে আঙুল লাগানোকে নিশ্চিত শাফাআতের আমল বলা যাবে না। আযানের জবাবের ক্ষেত্রে প্রমাণিত সুন্নাহ হলো মুয়াজ্জিন যা বলে তা বলা। ফজিলত পেতে হলে নবীজির নামে প্রমাণিত আমলই অনুসরণ করা দরকার।"},"teachings":["আযানের জবাবে প্রমাণিত আমলকে গুরুত্ব দিতে হবে।","চোখ মাসাহের সাথে নিশ্চিত শাফাআত যুক্ত করা সহীহ নয়।","দাইলামীতে থাকা মানেই কোনো বর্ণনা সহীহ নয়।","শাফাআতের মতো বড় বিষয়ে জোর দাবি করতে শক্ত দলীল দরকার।"],"related_hadiths":[{"id":"611","book_id":"1","label":"Sahih Bukhari"},{"id":"614","book_id":"1","label":"Sahih Bukhari"},{"id":"2659","book_id":"5","label":"Jami at-Tirmidhi"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আযানের সময় চোখ মাসাহ—সহীহ নয়","description":"$book_name$ $hadith_number$ - $chapter_name$. আযানে শাহাদাতের সময় আঙুল দিয়ে চোখ মাসাহ করলে শাফাআত অপরিহার্য—এই বর্ণনা সহীহ নয়; প্রমাণিত আযানের জবাবই যথেষ্ট।"},"heading":{"title":"আযানে চোখ মাসাহ: সহীহ নয় এমন ফজিলত","description":"এই বর্ণনায় বলা হয়েছে, মুয়াজ্জিন যখন আশহাদু আন্না মুহাম্মাদার রাসূলুল্লাহ বলে, তখন তর্জনী দিয়ে দুই চোখ মাসাহ করলে রাসূল সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম-এর সুপারিশ অপরিহার্য হবে। কিন্তু প্রদত্ত তাহকীক অনুযায়ী হাদিসটি সহীহ নয়। দাইলামী এটি আবূ বকর রা. থেকে মারফূ হিসেবে উল্লেখ করেছেন, আর ইবনু তাহির, শাওকানী ও সাখাবী একে সহীহ নয় বলেছেন। তাই আযানের সময় চোখে আঙুল লাগানোকে নিশ্চিত শাফাআতের আমল বলা যাবে না। আযানের জবাবের ক্ষেত্রে প্রমাণিত সুন্নাহ হলো মুয়াজ্জিন যা বলে তা বলা। ফজিলত পেতে হলে নবীজির নামে প্রমাণিত আমলই অনুসরণ করা দরকার।"},"teachings":["আযানের জবাবে প্রমাণিত আমলকে গুরুত্ব দিতে হবে।","চোখ মাসাহের সাথে নিশ্চিত শাফাআত যুক্ত করা সহীহ নয়।","দাইলামীতে থাকা মানেই কোনো বর্ণনা সহীহ নয়।","শাফাআতের মতো বড় বিষয়ে জোর দাবি করতে শক্ত দলীল দরকার।"],"related_hadiths":[{"id":"611","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"614","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2659","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"}]}</t>
         </is>
       </c>
       <c r="E33" s="4" t="n"/>
@@ -1228,7 +1232,7 @@
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সলাত ও তওবায় দ্রুততা—জাল বর্ণনা, অর্থ সঠিক","description":"$book_name$ $hadith_number$ - $chapter_name$. সলাত ছুটে যাওয়ার আগে আদায় ও মৃত্যুর আগে তওবার বর্ণনাটি জাল, তবে সতর্কতার অর্থ আলাদাভাবে সঠিক বলা হয়েছে।"},"heading":{"title":"সলাত ও তওবা: জাল হাদিস নয়, সতর্ক অর্থ","description":"এই বর্ণনায় বলা হয়েছে, সলাত ছুটে যাওয়ার আগে দ্রুত আদায় কর এবং মৃত্যু আসার আগে দ্রুত তওবা কর। প্রদত্ত তাহকীক অনুযায়ী হাদিসটি জাল; সাগানী একে মাওযূআহ গ্রন্থে উল্লেখ করেছেন। তবে পাঠে বলা হয়েছে, এর অর্থটি সঠিক। তাই এখানে গুরুত্বপূর্ণ পার্থক্য আছে: কথা ভালো হতে পারে, কিন্তু সেটি রাসূল সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম-এর হাদিস কিনা—তা আলাদা প্রশ্ন। সলাত সময়মতো আদায় ও তওবায় দেরি না করা ইসলামী শিক্ষার সাথে মেলে, কিন্তু এই নির্দিষ্ট বাক্যকে নববী হাদিস বলা যাবে না। দাওয়াহ বা লেখা তৈরির সময় “অর্থ ভালো” আর “হাদিস সহীহ”—এই দুইকে গুলিয়ে ফেললে পাঠক ভুল বুঝতে পারে।"},"teachings":["অর্থ ভালো হলেও জাল হাদিস বলা যাবে না।","সলাত ও তওবার গুরুত্ব সহীহ দলীল থেকে শেখানো উচিত।","মৃত্যুর আগে তওবার সুযোগ নিয়ে অবহেলা করা ঠিক নয়।","হাদিসের নামে উদ্ধৃতি দেওয়ার আগে হুকুম জানা দরকার।"],"related_hadiths":[{"id":"2479","book_id":"4","label":"Sunan Abu Dawud"},{"id":"3535","book_id":"5","label":"Jami at-Tirmidhi"},{"id":"2659","book_id":"5","label":"Jami at-Tirmidhi"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সলাত ও তওবায় দ্রুততা—জাল বর্ণনা, অর্থ সঠিক","description":"$book_name$ $hadith_number$ - $chapter_name$. সলাত ছুটে যাওয়ার আগে আদায় ও মৃত্যুর আগে তওবার বর্ণনাটি জাল, তবে সতর্কতার অর্থ আলাদাভাবে সঠিক বলা হয়েছে।"},"heading":{"title":"সলাত ও তওবা: জাল হাদিস নয়, সতর্ক অর্থ","description":"এই বর্ণনায় বলা হয়েছে, সলাত ছুটে যাওয়ার আগে দ্রুত আদায় কর এবং মৃত্যু আসার আগে দ্রুত তওবা কর। প্রদত্ত তাহকীক অনুযায়ী হাদিসটি জাল; সাগানী একে মাওযূআহ গ্রন্থে উল্লেখ করেছেন। তবে পাঠে বলা হয়েছে, এর অর্থটি সঠিক। তাই এখানে গুরুত্বপূর্ণ পার্থক্য আছে: কথা ভালো হতে পারে, কিন্তু সেটি রাসূল সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম-এর হাদিস কিনা—তা আলাদা প্রশ্ন। সলাত সময়মতো আদায় ও তওবায় দেরি না করা ইসলামী শিক্ষার সাথে মেলে, কিন্তু এই নির্দিষ্ট বাক্যকে নববী হাদিস বলা যাবে না। দাওয়াহ বা লেখা তৈরির সময় “অর্থ ভালো” আর “হাদিস সহীহ”—এই দুইকে গুলিয়ে ফেললে পাঠক ভুল বুঝতে পারে।"},"teachings":["অর্থ ভালো হলেও জাল হাদিস বলা যাবে না।","সলাত ও তওবার গুরুত্ব সহীহ দলীল থেকে শেখানো উচিত।","মৃত্যুর আগে তওবার সুযোগ নিয়ে অবহেলা করা ঠিক নয়।","হাদিসের নামে উদ্ধৃতি দেওয়ার আগে হুকুম জানা দরকার।"],"related_hadiths":[{"id":"2479","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"3535","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"2659","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"}]}</t>
         </is>
       </c>
       <c r="E34" s="4" t="n"/>
@@ -1251,7 +1255,7 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আলেম-আমলকারী-মুখলেস—জাল বর্ণনা","description":"$book_name$ $hadith_number$ - $chapter_name$. আলেম ছাড়া সবাই মৃত, মুখলেসরা বিপদে—এই বর্ণনা জাল; ইলম, আমল ও ইখলাস নিয়ে সহীহ দলীল প্রয়োজন।"},"heading":{"title":"ইলম, আমল ও ইখলাস: জাল বর্ণনার সীমা","description":"এই বর্ণনায় বলা হয়েছে, আলেম ছাড়া সবাই মৃত; আমলকারী ছাড়া সব আলেম ধ্বংসপ্রাপ্ত; মুখলেস ছাড়া সব আমলকারী ডুবে আছে; আর মুখলেসরা মহা বিপদে। প্রদত্ত তাহকীক অনুযায়ী হাদিসটি জাল। সাগানী একে মিথ্যারোপ বলেছেন এবং আলবানী বলেছেন, কথাটির সাথে সূফীদের ভাষার সাদৃশ্য আছে। এখানে শিক্ষা হলো, ইলম, আমল ও ইখলাস—তিনটিই দ্বীনের বড় বিষয়; কিন্তু এগুলো বোঝাতে রাসূলের নামে অতিরঞ্জিত বা প্রমাণহীন বাক্য প্রচার করা যাবে না। “ইখলাস” নিয়ে ভয় ও সচেতনতা ভালো, তবে জাল হাদিস দিয়ে মানুষকে শেখালে উল্টো দ্বীনের প্রতি আস্থা কমে। সহীহ দলীল দিয়ে আন্তরিকতা শেখানোই নিরাপদ।"},"teachings":["ইলম, আমল ও ইখলাসের গুরুত্ব আছে, কিন্তু জাল বর্ণনা দিয়ে নয়।","অতিরঞ্জিত আধ্যাত্মিক বাক্য হাদিস কিনা যাচাই করা দরকার।","রাসূলের নামে মিথ্যা কথা বলা বড় সতর্কতার বিষয়।","শিক্ষামূলক কথা উদ্ধৃত করলে উৎস পরিষ্কার করা উচিত।"],"related_hadiths":[{"id":"1","book_id":"1","label":"Sahih Bukhari"},{"id":"100","book_id":"2","label":"Sahih Muslim"},{"id":"2659","book_id":"5","label":"Jami at-Tirmidhi"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আলেম-আমলকারী-মুখলেস—জাল বর্ণনা","description":"$book_name$ $hadith_number$ - $chapter_name$. আলেম ছাড়া সবাই মৃত, মুখলেসরা বিপদে—এই বর্ণনা জাল; ইলম, আমল ও ইখলাস নিয়ে সহীহ দলীল প্রয়োজন।"},"heading":{"title":"ইলম, আমল ও ইখলাস: জাল বর্ণনার সীমা","description":"এই বর্ণনায় বলা হয়েছে, আলেম ছাড়া সবাই মৃত; আমলকারী ছাড়া সব আলেম ধ্বংসপ্রাপ্ত; মুখলেস ছাড়া সব আমলকারী ডুবে আছে; আর মুখলেসরা মহা বিপদে। প্রদত্ত তাহকীক অনুযায়ী হাদিসটি জাল। সাগানী একে মিথ্যারোপ বলেছেন এবং আলবানী বলেছেন, কথাটির সাথে সূফীদের ভাষার সাদৃশ্য আছে। এখানে শিক্ষা হলো, ইলম, আমল ও ইখলাস—তিনটিই দ্বীনের বড় বিষয়; কিন্তু এগুলো বোঝাতে রাসূলের নামে অতিরঞ্জিত বা প্রমাণহীন বাক্য প্রচার করা যাবে না। “ইখলাস” নিয়ে ভয় ও সচেতনতা ভালো, তবে জাল হাদিস দিয়ে মানুষকে শেখালে উল্টো দ্বীনের প্রতি আস্থা কমে। সহীহ দলীল দিয়ে আন্তরিকতা শেখানোই নিরাপদ।"},"teachings":["ইলম, আমল ও ইখলাসের গুরুত্ব আছে, কিন্তু জাল বর্ণনা দিয়ে নয়।","অতিরঞ্জিত আধ্যাত্মিক বাক্য হাদিস কিনা যাচাই করা দরকার।","রাসূলের নামে মিথ্যা কথা বলা বড় সতর্কতার বিষয়।","শিক্ষামূলক কথা উদ্ধৃত করলে উৎস পরিষ্কার করা উচিত।"],"related_hadiths":[{"id":"1","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"100","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"2659","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"}]}</t>
         </is>
       </c>
       <c r="E35" s="4" t="n"/>
@@ -1274,7 +1278,7 @@
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ঈসা ছাড়া মাহদী নেই—মুনকার বর্ণনা","description":"$book_name$ $hadith_number$ - $chapter_name$. এক মাত্র ঈসা আ.-ই মাহদী—এই বর্ণনা মুনকার; মাহদী বিষয়ে দুর্বল ও জাল বর্ণনা থেকে সতর্ক থাকা জরুরি।"},"heading":{"title":"মাহদী ও ঈসা আ.: মুনকার বর্ণনা থেকে সতর্কতা","description":"এই বর্ণনায় বলা হয়েছে, একমাত্র ঈসা আলাইহিস সালামই মাহদী। প্রদত্ত তাহকীক অনুযায়ী হাদিসটি মুনকার। সনদে হাসান বাসরীর আনআনাহ, মুহাম্মাদ ইবনু খালিদ আল-জানাদীর অজ্ঞতা এবং সনদের বিভিন্নতার কথা এসেছে। বাইহাকী একে মুনকাতি বলেছেন, যাহাবী মুনকার বলেছেন, আর ইবনু হাজার মাহদী সংক্রান্ত অন্য বর্ণনার বিরোধিতার কারণে একে পরিত্যাজ্য বলে ইঙ্গিত করেছেন। তাই শেষ যুগ, মাহদী ও ঈসা আ. বিষয়ে আবেগী বক্তব্য নয়, যাচাইকৃত বর্ণনা দরকার। এই বিষয়ে বহু দুর্বল ও জাল কথা প্রচলিত হতে পারে, তাই নির্দিষ্ট দাবি করার আগে হাদিসের হুকুম দেখা জরুরি।"},"teachings":["মাহদী বিষয়ে দুর্বল ও জাল বর্ণনা অনেক আছে—যাচাই জরুরি।","সনদে তাদলীস, অজ্ঞ বর্ণনাকারী ও বিচ্ছিন্নতা হাদিস দুর্বল করে।","ঈসা আ. ও মাহদী বিষয়ে আলাদা আলাদা বর্ণনা গুলিয়ে ফেলা ঠিক নয়।","শেষ যুগের আলোচনায় সাবধান ভাষা ব্যবহার করা দরকার।"],"related_hadiths":[{"id":"2230","book_id":"5","label":"Jami at-Tirmidhi"},{"id":"2659","book_id":"5","label":"Jami at-Tirmidhi"},{"id":"7400","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ঈসা ছাড়া মাহদী নেই—মুনকার বর্ণনা","description":"$book_name$ $hadith_number$ - $chapter_name$. এক মাত্র ঈসা আ.-ই মাহদী—এই বর্ণনা মুনকার; মাহদী বিষয়ে দুর্বল ও জাল বর্ণনা থেকে সতর্ক থাকা জরুরি।"},"heading":{"title":"মাহদী ও ঈসা আ.: মুনকার বর্ণনা থেকে সতর্কতা","description":"এই বর্ণনায় বলা হয়েছে, একমাত্র ঈসা আলাইহিস সালামই মাহদী। প্রদত্ত তাহকীক অনুযায়ী হাদিসটি মুনকার। সনদে হাসান বাসরীর আনআনাহ, মুহাম্মাদ ইবনু খালিদ আল-জানাদীর অজ্ঞতা এবং সনদের বিভিন্নতার কথা এসেছে। বাইহাকী একে মুনকাতি বলেছেন, যাহাবী মুনকার বলেছেন, আর ইবনু হাজার মাহদী সংক্রান্ত অন্য বর্ণনার বিরোধিতার কারণে একে পরিত্যাজ্য বলে ইঙ্গিত করেছেন। তাই শেষ যুগ, মাহদী ও ঈসা আ. বিষয়ে আবেগী বক্তব্য নয়, যাচাইকৃত বর্ণনা দরকার। এই বিষয়ে বহু দুর্বল ও জাল কথা প্রচলিত হতে পারে, তাই নির্দিষ্ট দাবি করার আগে হাদিসের হুকুম দেখা জরুরি।"},"teachings":["মাহদী বিষয়ে দুর্বল ও জাল বর্ণনা অনেক আছে—যাচাই জরুরি।","সনদে তাদলীস, অজ্ঞ বর্ণনাকারী ও বিচ্ছিন্নতা হাদিস দুর্বল করে।","ঈসা আ. ও মাহদী বিষয়ে আলাদা আলাদা বর্ণনা গুলিয়ে ফেলা ঠিক নয়।","শেষ যুগের আলোচনায় সাবধান ভাষা ব্যবহার করা দরকার।"],"related_hadiths":[{"id":"2230","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"2659","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"7400","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E36" s="4" t="n"/>
@@ -1297,7 +1301,7 @@
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মুমিনের উচ্ছিষ্টে আরোগ্য—ভিত্তিহীন বর্ণনা","description":"$book_name$ $hadith_number$ - $chapter_name$. মুমিনের উচ্ছিষ্টে আরোগ্য আছে—এটি হাদিস নয়; অন্য দুর্বল বর্ণনা দিয়েও এই দাবির স্পষ্ট সমর্থন পাওয়া যায় না।"},"heading":{"title":"মুমিনের উচ্ছিষ্ট ও আরোগ্য: ভিত্তিহীন হাদিসের সতর্কতা","description":"এই বর্ণনায় বলা হয়েছে, মুমিনের উচ্ছিষ্টে আরোগ্য আছে। প্রদত্ত তাহকীক অনুযায়ী এর কোনো ভিত্তি নেই। আহমাদ আল-গাযাযী বলেছেন, এটি হাদিস নয়; আজলূনীও তা সমর্থন করেছেন। আলী আল-কারী অর্থের দিক দিয়ে একটি বর্ণনার কথা উল্লেখ করলেও আলবানী ব্যাখ্যা করেছেন, ইবনু আব্বাস রা.-এর সেই মারফূ বর্ণনাও সহীহ নয়। আরও বলা হয়েছে, সেখানে “উচ্ছিষ্টে আরোগ্য” কথাটি স্পষ্ট বা পরোক্ষভাবেও নেই। তাই কারো উচ্ছিষ্ট পান করা, বিনয় বা সম্পর্কের কথা আলাদা হতে পারে; কিন্তু “আরোগ্য” দাবি করা এই পাঠের আলোকে প্রমাণিত নয়। স্বাস্থ্য, রোগমুক্তি ও বরকত নিয়ে কথা বলার সময় জাল বা ভিত্তিহীন হাদিস থেকে দূরে থাকা দরকার।"},"teachings":["কোনো বস্তুকে আরোগ্যের কারণ বলতে প্রমাণ দরকার।","অন্য দুর্বল বর্ণনা দিয়ে ভিত্তিহীন দাবিকে শক্ত করা যায় না।","হাদিস নয় এমন বাক্যকে নবীজির নামে বলা উচিত নয়।","বিনয় ও আরোগ্য—দুইটি আলাদা দাবি; গুলিয়ে ফেলা ঠিক নয়।"],"related_hadiths":[{"id":"2659","book_id":"5","label":"Jami at-Tirmidhi"},{"id":"7400","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মুমিনের উচ্ছিষ্টে আরোগ্য—ভিত্তিহীন বর্ণনা","description":"$book_name$ $hadith_number$ - $chapter_name$. মুমিনের উচ্ছিষ্টে আরোগ্য আছে—এটি হাদিস নয়; অন্য দুর্বল বর্ণনা দিয়েও এই দাবির স্পষ্ট সমর্থন পাওয়া যায় না।"},"heading":{"title":"মুমিনের উচ্ছিষ্ট ও আরোগ্য: ভিত্তিহীন হাদিসের সতর্কতা","description":"এই বর্ণনায় বলা হয়েছে, মুমিনের উচ্ছিষ্টে আরোগ্য আছে। প্রদত্ত তাহকীক অনুযায়ী এর কোনো ভিত্তি নেই। আহমাদ আল-গাযাযী বলেছেন, এটি হাদিস নয়; আজলূনীও তা সমর্থন করেছেন। আলী আল-কারী অর্থের দিক দিয়ে একটি বর্ণনার কথা উল্লেখ করলেও আলবানী ব্যাখ্যা করেছেন, ইবনু আব্বাস রা.-এর সেই মারফূ বর্ণনাও সহীহ নয়। আরও বলা হয়েছে, সেখানে “উচ্ছিষ্টে আরোগ্য” কথাটি স্পষ্ট বা পরোক্ষভাবেও নেই। তাই কারো উচ্ছিষ্ট পান করা, বিনয় বা সম্পর্কের কথা আলাদা হতে পারে; কিন্তু “আরোগ্য” দাবি করা এই পাঠের আলোকে প্রমাণিত নয়। স্বাস্থ্য, রোগমুক্তি ও বরকত নিয়ে কথা বলার সময় জাল বা ভিত্তিহীন হাদিস থেকে দূরে থাকা দরকার।"},"teachings":["কোনো বস্তুকে আরোগ্যের কারণ বলতে প্রমাণ দরকার।","অন্য দুর্বল বর্ণনা দিয়ে ভিত্তিহীন দাবিকে শক্ত করা যায় না।","হাদিস নয় এমন বাক্যকে নবীজির নামে বলা উচিত নয়।","বিনয় ও আরোগ্য—দুইটি আলাদা দাবি; গুলিয়ে ফেলা ঠিক নয়।"],"related_hadiths":[{"id":"2659","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"7400","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E37" s="4" t="n"/>
@@ -1320,7 +1324,7 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ভাইয়ের উচ্ছিষ্ট পান ও সত্তর মর্যাদা—জাল","description":"$book_name$ $hadith_number$ - $chapter_name$. ভাইয়ের উচ্ছিষ্ট পান করলে সত্তর মর্যাদা ও গুনাহ মোচনের বর্ণনা জাল; নম্রতার কথা প্রমাণহীন ফজিলতে বাড়ানো যাবে না।"},"heading":{"title":"উচ্ছিষ্ট পান করার ফজিলত: জাল বর্ণনার বিশ্লেষণ","description":"এই বর্ণনায় বলা হয়েছে, ভাইয়ের উচ্ছিষ্ট পান করা নম্রতার অন্তর্ভুক্ত এবং আল্লাহর সন্তুষ্টির জন্য তা করলে সত্তর গুণ মর্যাদা, সত্তর গুনাহ মোচন ও সত্তর মর্যাদা লেখা হবে। প্রদত্ত তাহকীক অনুযায়ী হাদিসটি জাল। সনদে নূহ ইবনু মারইয়াম আছেন, যিনি হাদিস বর্ণনায় মিথ্যার দোষে দোষী হিসেবে আলোচিত। সুয়ূতী যে মুতাবাআতের কথা বলেছেন, আলবানী সেটিও গ্রহণযোগ্য নয় বলে দেখিয়েছেন; কারণ সেখানে অপরিচিত ও মুনকার বর্ণনাকারী আছে। তাই নম্রতা শেখাতে গিয়ে সত্তর সংখ্যার আকর্ষণীয় প্রতিশ্রুতি প্রচার করা ঠিক নয়। এমন ফজিলত শুনলে আগে উৎস ও হুকুম দেখা উচিত।"},"teachings":["সত্তর মর্যাদা বা গুনাহ মোচনের দাবি প্রমাণ ছাড়া বলা যাবে না।","মুতাবাআত থাকলেই বর্ণনা সহীহ হয়ে যায় না।","মিথ্যার দোষে অভিযুক্ত বর্ণনাকারীর হাদিস গ্রহণযোগ্য নয়।","নম্রতা শেখাতে সহীহ ভাষা ব্যবহার করা দরকার।"],"related_hadiths":[{"id":"2659","book_id":"5","label":"Jami at-Tirmidhi"},{"id":"7400","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ভাইয়ের উচ্ছিষ্ট পান ও সত্তর মর্যাদা—জাল","description":"$book_name$ $hadith_number$ - $chapter_name$. ভাইয়ের উচ্ছিষ্ট পান করলে সত্তর মর্যাদা ও গুনাহ মোচনের বর্ণনা জাল; নম্রতার কথা প্রমাণহীন ফজিলতে বাড়ানো যাবে না।"},"heading":{"title":"উচ্ছিষ্ট পান করার ফজিলত: জাল বর্ণনার বিশ্লেষণ","description":"এই বর্ণনায় বলা হয়েছে, ভাইয়ের উচ্ছিষ্ট পান করা নম্রতার অন্তর্ভুক্ত এবং আল্লাহর সন্তুষ্টির জন্য তা করলে সত্তর গুণ মর্যাদা, সত্তর গুনাহ মোচন ও সত্তর মর্যাদা লেখা হবে। প্রদত্ত তাহকীক অনুযায়ী হাদিসটি জাল। সনদে নূহ ইবনু মারইয়াম আছেন, যিনি হাদিস বর্ণনায় মিথ্যার দোষে দোষী হিসেবে আলোচিত। সুয়ূতী যে মুতাবাআতের কথা বলেছেন, আলবানী সেটিও গ্রহণযোগ্য নয় বলে দেখিয়েছেন; কারণ সেখানে অপরিচিত ও মুনকার বর্ণনাকারী আছে। তাই নম্রতা শেখাতে গিয়ে সত্তর সংখ্যার আকর্ষণীয় প্রতিশ্রুতি প্রচার করা ঠিক নয়। এমন ফজিলত শুনলে আগে উৎস ও হুকুম দেখা উচিত।"},"teachings":["সত্তর মর্যাদা বা গুনাহ মোচনের দাবি প্রমাণ ছাড়া বলা যাবে না।","মুতাবাআত থাকলেই বর্ণনা সহীহ হয়ে যায় না।","মিথ্যার দোষে অভিযুক্ত বর্ণনাকারীর হাদিস গ্রহণযোগ্য নয়।","নম্রতা শেখাতে সহীহ ভাষা ব্যবহার করা দরকার।"],"related_hadiths":[{"id":"2659","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"7400","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E38" s="4" t="n"/>
@@ -1343,7 +1347,7 @@
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | দুনিয়া-আখেরাত নিয়ে ভিত্তিহীন বর্ণনা","description":"$book_name$ $hadith_number$ - $chapter_name$. দুনিয়া ও আখেরাত নিয়ে প্রচলিত এই বাক্যটি মারফূ হাদিস হিসেবে ভিত্তিহীন বলা হয়েছে।"},"heading":{"title":"দুনিয়া ও আখেরাত নিয়ে প্রচলিত বাণী: মারফূ হাদিস নয়","description":"এই বর্ণনায় বলা হয়েছে, “দুনিয়ার জন্য এমনভাবে কাজ কর, যেন তুমি চিরকাল বাঁচবে; আর আখেরাতের জন্য এমনভাবে আমল কর, যেন কালই মারা যাবে।” কথাটি খুব পরিচিত। কিন্তু প্রদত্ত আলোচনায় বলা হয়েছে, মারফূ হিসেবে এর কোনো ভিত্তি নেই। অর্থাৎ রাসূল صلى الله عليه وسلم-এর বাণী হিসেবে এটি সাব্যস্ত নয়। লেখায় মাওকূফভাবে কিছু ভিত্তির কথা এসেছে, কিন্তু সনদে বিচ্ছিন্নতা ও দুর্বলতার কথা বলা হয়েছে। তাই “দুনিয়ার জন্য কাজ কর আখেরাতের জন্য আমল কর” বাক্যটি জনপ্রিয় হলেও সহীহ হাদিস হিসেবে বলা ঠিক নয়। এর মধ্যে মানুষকে দুনিয়া ও আখেরাতের ভারসাম্যের কথা মনে করানো হতে পারে, কিন্তু নবী صلى الله عليه وسلم-এর নামে বলতে হলে সহীহ প্রমাণ দরকার। ইসলামে আখেরাতের প্রস্তুতি ও হালাল দুনিয়াবি কাজ—দুটিই গুরুত্বপূর্ণ, তবে দলিলের ভাষা ঠিক রাখতে হবে।"},"teachings":["প্রচলিত বাণী সব সময় সহীহ হাদিস নয়।","মারফূ হাদিস হিসেবে দাবি করতে শক্ত দলিল দরকার।","দুনিয়া ও আখেরাতের ভারসাম্য বোঝাতে সহীহ দলিল ব্যবহার করা উচিত।","জনপ্রিয় বাক্য শেয়ার করার আগে তার উৎস দেখা দরকার।"],"related_hadiths":[{"id":"6416","book_id":"1","label":"Sahih Bukhari"},{"id":"2346","book_id":"5","label":"Jami at-Tirmidhi"},{"id":"4105","book_id":"6","label":"Sunan Ibn Majah"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | দুনিয়া-আখেরাত নিয়ে ভিত্তিহীন বর্ণনা","description":"$book_name$ $hadith_number$ - $chapter_name$. দুনিয়া ও আখেরাত নিয়ে প্রচলিত এই বাক্যটি মারফূ হাদিস হিসেবে ভিত্তিহীন বলা হয়েছে।"},"heading":{"title":"দুনিয়া ও আখেরাত নিয়ে প্রচলিত বাণী: মারফূ হাদিস নয়","description":"এই বর্ণনায় বলা হয়েছে, “দুনিয়ার জন্য এমনভাবে কাজ কর, যেন তুমি চিরকাল বাঁচবে; আর আখেরাতের জন্য এমনভাবে আমল কর, যেন কালই মারা যাবে।” কথাটি খুব পরিচিত। কিন্তু প্রদত্ত আলোচনায় বলা হয়েছে, মারফূ হিসেবে এর কোনো ভিত্তি নেই। অর্থাৎ রাসূল صلى الله عليه وسلم-এর বাণী হিসেবে এটি সাব্যস্ত নয়। লেখায় মাওকূফভাবে কিছু ভিত্তির কথা এসেছে, কিন্তু সনদে বিচ্ছিন্নতা ও দুর্বলতার কথা বলা হয়েছে। তাই “দুনিয়ার জন্য কাজ কর আখেরাতের জন্য আমল কর” বাক্যটি জনপ্রিয় হলেও সহীহ হাদিস হিসেবে বলা ঠিক নয়। এর মধ্যে মানুষকে দুনিয়া ও আখেরাতের ভারসাম্যের কথা মনে করানো হতে পারে, কিন্তু নবী صلى الله عليه وسلم-এর নামে বলতে হলে সহীহ প্রমাণ দরকার। ইসলামে আখেরাতের প্রস্তুতি ও হালাল দুনিয়াবি কাজ—দুটিই গুরুত্বপূর্ণ, তবে দলিলের ভাষা ঠিক রাখতে হবে।"},"teachings":["প্রচলিত বাণী সব সময় সহীহ হাদিস নয়।","মারফূ হাদিস হিসেবে দাবি করতে শক্ত দলিল দরকার।","দুনিয়া ও আখেরাতের ভারসাম্য বোঝাতে সহীহ দলিল ব্যবহার করা উচিত।","জনপ্রিয় বাক্য শেয়ার করার আগে তার উৎস দেখা দরকার।"],"related_hadiths":[{"id":"6416","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2346","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"4105","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
         </is>
       </c>
       <c r="E39" s="4" t="n"/>
@@ -1366,7 +1370,7 @@
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মাহদী আব্বাসের সন্তান—জাল বর্ণনা","description":"$book_name$ $hadith_number$ - $chapter_name$. মাহদী আব্বাস রা.-এর সন্তানদের থেকে হবে—এই বর্ণনা জাল; প্রদত্ত পাঠে একে অন্য বর্ণনার বিরোধীও বলা হয়েছে।"},"heading":{"title":"মাহদী আব্বাসের সন্তান? জাল বর্ণনার সতর্কতা","description":"এই বর্ণনায় বলা হয়েছে, মাহদী হবে নবী সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম-এর চাচা আব্বাস রা.-এর সন্তানদের মধ্য থেকে। প্রদত্ত তাহকীক অনুযায়ী হাদিসটি জাল। দারাকুতনী এটিকে গারীব বলেছেন এবং মুহাম্মাদ ইবনুল ওয়ালীদ এককভাবে বর্ণনা করেছেন। আলবানী বলেছেন, তিনি মিথ্যার দোষে দোষী; ইবনু আদী তাঁর সম্পর্কে হাদিস জাল করার কথা বলেছেন, আবূ আরূবাহ তাঁকে মিথ্যুক বলেছেন। পাঠে আরও বলা হয়েছে, এই বর্ণনা সেই কথার বিরোধী যেখানে মাহদীকে ফাতিমা রা.-এর সন্তানদের মধ্য থেকে বলা হয়েছে। তাই মাহদীর বংশ, পরিচয় ও শেষ যুগের কথা নিয়ে নিশ্চিত দাবি করতে হলে সহীহ বা গ্রহণযোগ্য দলীল দরকার। জাল বর্ণনা বিশ্বাসের বিষয়কে ঘোলাটে করে।"},"teachings":["মাহদীর বংশ নিয়ে জাল বর্ণনা প্রচার করা উচিত নয়।","একজন মিথ্যুক বর্ণনাকারীর একক বর্ণনা গ্রহণযোগ্য নয়।","শেষ যুগের বিষয়ে আবেগ নয়, দলীল প্রয়োজন।","প্রচলিত দাবি অন্য বর্ণনার বিরোধী হলে আরও সতর্ক হতে হয়।"],"related_hadiths":[{"id":"2230","book_id":"5","label":"Jami at-Tirmidhi"},{"id":"2659","book_id":"5","label":"Jami at-Tirmidhi"},{"id":"7400","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মাহদী আব্বাসের সন্তান—জাল বর্ণনা","description":"$book_name$ $hadith_number$ - $chapter_name$. মাহদী আব্বাস রা.-এর সন্তানদের থেকে হবে—এই বর্ণনা জাল; প্রদত্ত পাঠে একে অন্য বর্ণনার বিরোধীও বলা হয়েছে।"},"heading":{"title":"মাহদী আব্বাসের সন্তান? জাল বর্ণনার সতর্কতা","description":"এই বর্ণনায় বলা হয়েছে, মাহদী হবে নবী সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম-এর চাচা আব্বাস রা.-এর সন্তানদের মধ্য থেকে। প্রদত্ত তাহকীক অনুযায়ী হাদিসটি জাল। দারাকুতনী এটিকে গারীব বলেছেন এবং মুহাম্মাদ ইবনুল ওয়ালীদ এককভাবে বর্ণনা করেছেন। আলবানী বলেছেন, তিনি মিথ্যার দোষে দোষী; ইবনু আদী তাঁর সম্পর্কে হাদিস জাল করার কথা বলেছেন, আবূ আরূবাহ তাঁকে মিথ্যুক বলেছেন। পাঠে আরও বলা হয়েছে, এই বর্ণনা সেই কথার বিরোধী যেখানে মাহদীকে ফাতিমা রা.-এর সন্তানদের মধ্য থেকে বলা হয়েছে। তাই মাহদীর বংশ, পরিচয় ও শেষ যুগের কথা নিয়ে নিশ্চিত দাবি করতে হলে সহীহ বা গ্রহণযোগ্য দলীল দরকার। জাল বর্ণনা বিশ্বাসের বিষয়কে ঘোলাটে করে।"},"teachings":["মাহদীর বংশ নিয়ে জাল বর্ণনা প্রচার করা উচিত নয়।","একজন মিথ্যুক বর্ণনাকারীর একক বর্ণনা গ্রহণযোগ্য নয়।","শেষ যুগের বিষয়ে আবেগ নয়, দলীল প্রয়োজন।","প্রচলিত দাবি অন্য বর্ণনার বিরোধী হলে আরও সতর্ক হতে হয়।"],"related_hadiths":[{"id":"2230","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"2659","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"7400","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E40" s="4" t="n"/>
@@ -1389,7 +1393,7 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আব্বাস বংশের মাহদী বিষয়ক জাল হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. আব্বাস বংশের এক যুবক নিয়ে বর্ণিত মাহদী সংক্রান্ত কথাটি জাল; সনদের দুর্বলতা ও মিথ্যার অভিযোগ স্পষ্ট করা হয়েছে।"},"heading":{"title":"আব্বাস বংশের মাহদী বিষয়ক জাল হাদিস: সনদ যাচাইয়ের শিক্ষা","description":"এই বর্ণনায় বলা হয়েছে, আল্লাহ রাসূলের মাধ্যমে একটি কাজ শুরু করেছেন এবং আব্বাস (রাঃ)-এর সন্তানদের মধ্য থেকে এক যুবকের মাধ্যমে তা শেষ করবেন। আরও বলা হয়েছে, তিনি পৃথিবীকে ইনসাফে পূর্ণ করবেন এবং ঈসা (আঃ)-এর সঙ্গে সালাত কায়েম করবেন। কিন্তু প্রদত্ত তাহকীক অনুযায়ী হাদিসটি জাল। এখানে মূল বিষয় হলো মাহদী বিষয়ক বর্ণনা যাচাই এবং জাল হাদিস চেনা। সনদে আহমাদ ইবনু হাজ্জাজ নামে একজন বর্ণনাকারী আছেন, যাকে যাহাবী এ হাদিসের ব্যাপারে মিথ্যার দোষে অভিযুক্ত করেছেন। ইবনু হাজারও এ কথার সঙ্গে একমত হয়েছেন। অন্য সনদেও আব্দুস সামাদ ইবনু আলী এবং মুহাম্মদ ইবনু নূহ সম্পর্কে সমস্যা বলা হয়েছে। তাই আকর্ষণীয় কথা হলেও হাদিস গ্রহণের আগে সনদ দেখা জরুরি।"},"teachings":["মাহদী বিষয়ক বর্ণনা শুনলেই তা গ্রহণ করা ঠিক নয়; সনদ যাচাই দরকার।","কোনো বর্ণনাকারীর ওপর মিথ্যার অভিযোগ থাকলে সেই বর্ণনা গ্রহণযোগ্য থাকে না।","ধর্মীয় বিষয়ে আবেগ নয়, যাচাই করা জ্ঞানকে গুরুত্ব দিতে হয়।","জাল হাদিস প্রচার করা থেকে সতর্ক থাকা উচিত।"],"related_hadiths":[{"id":"107","book_id":"1","label":"Sahih Bukhari"},{"id":"5","book_id":"2","label":"Sahih Muslim"},{"id":"4282","book_id":"4","label":"Sunan Abu Dawud"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আব্বাস বংশের মাহদী বিষয়ক জাল হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. আব্বাস বংশের এক যুবক নিয়ে বর্ণিত মাহদী সংক্রান্ত কথাটি জাল; সনদের দুর্বলতা ও মিথ্যার অভিযোগ স্পষ্ট করা হয়েছে।"},"heading":{"title":"আব্বাস বংশের মাহদী বিষয়ক জাল হাদিস: সনদ যাচাইয়ের শিক্ষা","description":"এই বর্ণনায় বলা হয়েছে, আল্লাহ রাসূলের মাধ্যমে একটি কাজ শুরু করেছেন এবং আব্বাস (রাঃ)-এর সন্তানদের মধ্য থেকে এক যুবকের মাধ্যমে তা শেষ করবেন। আরও বলা হয়েছে, তিনি পৃথিবীকে ইনসাফে পূর্ণ করবেন এবং ঈসা (আঃ)-এর সঙ্গে সালাত কায়েম করবেন। কিন্তু প্রদত্ত তাহকীক অনুযায়ী হাদিসটি জাল। এখানে মূল বিষয় হলো মাহদী বিষয়ক বর্ণনা যাচাই এবং জাল হাদিস চেনা। সনদে আহমাদ ইবনু হাজ্জাজ নামে একজন বর্ণনাকারী আছেন, যাকে যাহাবী এ হাদিসের ব্যাপারে মিথ্যার দোষে অভিযুক্ত করেছেন। ইবনু হাজারও এ কথার সঙ্গে একমত হয়েছেন। অন্য সনদেও আব্দুস সামাদ ইবনু আলী এবং মুহাম্মদ ইবনু নূহ সম্পর্কে সমস্যা বলা হয়েছে। তাই আকর্ষণীয় কথা হলেও হাদিস গ্রহণের আগে সনদ দেখা জরুরি।"},"teachings":["মাহদী বিষয়ক বর্ণনা শুনলেই তা গ্রহণ করা ঠিক নয়; সনদ যাচাই দরকার।","কোনো বর্ণনাকারীর ওপর মিথ্যার অভিযোগ থাকলে সেই বর্ণনা গ্রহণযোগ্য থাকে না।","ধর্মীয় বিষয়ে আবেগ নয়, যাচাই করা জ্ঞানকে গুরুত্ব দিতে হয়।","জাল হাদিস প্রচার করা থেকে সতর্ক থাকা উচিত।"],"related_hadiths":[{"id":"107","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"5","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"4282","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"}]}</t>
         </is>
       </c>
       <c r="E41" s="4" t="n"/>
@@ -1412,7 +1416,7 @@
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আবুল ফযলকে সুসংবাদ বিষয়ক জাল হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. আবুল ফযলকে দেওয়া সুসংবাদ হিসেবে প্রচলিত বর্ণনাটি জাল; লাহিয নামক বর্ণনাকারীর মিথ্যার অভিযোগ উল্লেখ করা হয়েছে।"},"heading":{"title":"আবুল ফযলকে সুসংবাদ বিষয়ক জাল হাদিস ও বর্ণনাকারী যাচাই","description":"এই বর্ণনায় আবুল ফযলকে উদ্দেশ করে বলা হয়েছে, আল্লাহ রাসূলের মাধ্যমে একটি কাজ শুরু করেছেন এবং তা তাঁর সন্তান দ্বারা শেষ করবেন। কথাটি শুনতে বিশেষ মর্যাদার মতো মনে হলেও প্রদত্ত তাহকীক অনুযায়ী হাদিসটি জাল। এখানে প্রধান শিক্ষা হলো ফযীলত বিষয়ক বর্ণনা যাচাই করা। আবূ নু‘য়াইম হিলইয়্যাহ গ্রন্থে এটি উল্লেখ করেছেন, কিন্তু সনদে লাহিয ইবনু জা‘ফার আত-তাইমী আছেন। আলবানীর বক্তব্য অনুযায়ী, লাহিয মিথ্যার দোষে দোষী ব্যক্তি। ইবনু আদী তাকে বাগদাদী মাজহূল বলেছেন এবং নির্ভরযোগ্যদের নামে মুনকার হাদিস বর্ণনা করতেন বলে উল্লেখ করেছেন। তাই কারও মর্যাদা বা বংশ নিয়ে কোনো কথা প্রচার হলে শুধু সুন্দর শোনার কারণে তা গ্রহণ করা নিরাপদ নয়।"},"teachings":["ফযীলত বিষয়ক হাদিসও সনদ ছাড়া গ্রহণ করা যায় না।","মাজহূল বা মিথ্যার দোষে অভিযুক্ত বর্ণনাকারীর বর্ণনা থেকে সতর্ক থাকতে হয়।","কারও বংশ বা মর্যাদা নিয়ে অতিরঞ্জিত কথা যাচাই ছাড়া প্রচার করা উচিত নয়।","জাল হাদিস চেনার জন্য মুহাদ্দিসদের সমালোচনা গুরুত্বপূর্ণ।"],"related_hadiths":[{"id":"107","book_id":"1","label":"Sahih Bukhari"},{"id":"5","book_id":"2","label":"Sahih Muslim"},{"id":"200","book_id":"14","label":"Mishkat al-Masabih"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আবুল ফযলকে সুসংবাদ বিষয়ক জাল হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. আবুল ফযলকে দেওয়া সুসংবাদ হিসেবে প্রচলিত বর্ণনাটি জাল; লাহিয নামক বর্ণনাকারীর মিথ্যার অভিযোগ উল্লেখ করা হয়েছে।"},"heading":{"title":"আবুল ফযলকে সুসংবাদ বিষয়ক জাল হাদিস ও বর্ণনাকারী যাচাই","description":"এই বর্ণনায় আবুল ফযলকে উদ্দেশ করে বলা হয়েছে, আল্লাহ রাসূলের মাধ্যমে একটি কাজ শুরু করেছেন এবং তা তাঁর সন্তান দ্বারা শেষ করবেন। কথাটি শুনতে বিশেষ মর্যাদার মতো মনে হলেও প্রদত্ত তাহকীক অনুযায়ী হাদিসটি জাল। এখানে প্রধান শিক্ষা হলো ফযীলত বিষয়ক বর্ণনা যাচাই করা। আবূ নু‘য়াইম হিলইয়্যাহ গ্রন্থে এটি উল্লেখ করেছেন, কিন্তু সনদে লাহিয ইবনু জা‘ফার আত-তাইমী আছেন। আলবানীর বক্তব্য অনুযায়ী, লাহিয মিথ্যার দোষে দোষী ব্যক্তি। ইবনু আদী তাকে বাগদাদী মাজহূল বলেছেন এবং নির্ভরযোগ্যদের নামে মুনকার হাদিস বর্ণনা করতেন বলে উল্লেখ করেছেন। তাই কারও মর্যাদা বা বংশ নিয়ে কোনো কথা প্রচার হলে শুধু সুন্দর শোনার কারণে তা গ্রহণ করা নিরাপদ নয়।"},"teachings":["ফযীলত বিষয়ক হাদিসও সনদ ছাড়া গ্রহণ করা যায় না।","মাজহূল বা মিথ্যার দোষে অভিযুক্ত বর্ণনাকারীর বর্ণনা থেকে সতর্ক থাকতে হয়।","কারও বংশ বা মর্যাদা নিয়ে অতিরঞ্জিত কথা যাচাই ছাড়া প্রচার করা উচিত নয়।","জাল হাদিস চেনার জন্য মুহাদ্দিসদের সমালোচনা গুরুত্বপূর্ণ।"],"related_hadiths":[{"id":"107","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"5","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"200","book_id":"14","slug":"mishkatul-masabih","label":"মিশকাতুল মাসাবীহ"}]}</t>
         </is>
       </c>
       <c r="E42" s="4" t="n"/>
@@ -1435,7 +1439,7 @@
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | তাসবীহ দানা নিয়ে জাল হাদিসের তাহকীক","description":"$book_name$ $hadith_number$ - $chapter_name$. তাসবীহ দানা দিয়ে জিকিরের প্রশংসা করা বর্ণনাটি জাল; সনদের মাজহূল ও মিথ্যুক বর্ণনাকারীদের কথা এসেছে।"},"heading":{"title":"তাসবীহ দানা নিয়ে জাল হাদিস: জিকিরে সুন্নাহ অনুসরণের শিক্ষা","description":"এই বর্ণনায় তাসবীহ পাঠের যন্ত্র বা দানা ব্যবহারকারীকে ভালো বলা হয়েছে। কিন্তু প্রদত্ত তাহকীক অনুযায়ী হাদিসটি জাল। দাইলামী এটি বর্ণনা করেছেন, পরে সুয়ূতী ও শাওকানী উল্লেখ করলেও তারা হুকুম দেননি। আলবানীর বিশ্লেষণে সনদে বহু অন্ধকার দিক আছে। অনেক বর্ণনাকারী মাজহূল, আবার কেউ কেউ মিথ্যার দোষে অভিযুক্ত। বিশেষ করে মুহাম্মদ ইবনু হারুন ইবনে ঈসা আল-হাশেমী সম্পর্কে বলা হয়েছে, তিনি হাদিস জাল করতেন। এখানে তাসবীহ দানা, তাসবীহ পাঠ ও জিকিরের পদ্ধতি নিয়ে সতর্কতা দেখা যায়। প্রদত্ত লেখায় আরও বলা হয়েছে, রাসূল (সা.)-এর দিকনির্দেশনা ছিল ডান হাতে বা অঙ্গুলিতে তাসবীহ গণনা করা। তাই জিকিরের মতো ভালো আমলেও সহিহ দলীলকে গুরুত্ব দেওয়া দরকার।"},"teachings":["তাসবীহ ও জিকিরের পদ্ধতিতে সহিহ দলীলকে অগ্রাধিকার দিতে হয়।","কোনো আমল জনপ্রিয় হলেই তা হাদিস দ্বারা প্রমাণিত ধরে নেওয়া ঠিক নয়।","সনদে মাজহূল বা জালকারী থাকলে বর্ণনা গ্রহণযোগ্য থাকে না।","সুন্নাহর পদ্ধতি জানার জন্য নির্ভরযোগ্য বর্ণনা অনুসরণ করা জরুরি।"],"related_hadiths":[{"id":"1502","book_id":"4","label":"Sunan Abu Dawud"},{"id":"3411","book_id":"5","label":"Jami at-Tirmidhi"},{"id":"2726","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | তাসবীহ দানা নিয়ে জাল হাদিসের তাহকীক","description":"$book_name$ $hadith_number$ - $chapter_name$. তাসবীহ দানা দিয়ে জিকিরের প্রশংসা করা বর্ণনাটি জাল; সনদের মাজহূল ও মিথ্যুক বর্ণনাকারীদের কথা এসেছে।"},"heading":{"title":"তাসবীহ দানা নিয়ে জাল হাদিস: জিকিরে সুন্নাহ অনুসরণের শিক্ষা","description":"এই বর্ণনায় তাসবীহ পাঠের যন্ত্র বা দানা ব্যবহারকারীকে ভালো বলা হয়েছে। কিন্তু প্রদত্ত তাহকীক অনুযায়ী হাদিসটি জাল। দাইলামী এটি বর্ণনা করেছেন, পরে সুয়ূতী ও শাওকানী উল্লেখ করলেও তারা হুকুম দেননি। আলবানীর বিশ্লেষণে সনদে বহু অন্ধকার দিক আছে। অনেক বর্ণনাকারী মাজহূল, আবার কেউ কেউ মিথ্যার দোষে অভিযুক্ত। বিশেষ করে মুহাম্মদ ইবনু হারুন ইবনে ঈসা আল-হাশেমী সম্পর্কে বলা হয়েছে, তিনি হাদিস জাল করতেন। এখানে তাসবীহ দানা, তাসবীহ পাঠ ও জিকিরের পদ্ধতি নিয়ে সতর্কতা দেখা যায়। প্রদত্ত লেখায় আরও বলা হয়েছে, রাসূল (সা.)-এর দিকনির্দেশনা ছিল ডান হাতে বা অঙ্গুলিতে তাসবীহ গণনা করা। তাই জিকিরের মতো ভালো আমলেও সহিহ দলীলকে গুরুত্ব দেওয়া দরকার।"},"teachings":["তাসবীহ ও জিকিরের পদ্ধতিতে সহিহ দলীলকে অগ্রাধিকার দিতে হয়।","কোনো আমল জনপ্রিয় হলেই তা হাদিস দ্বারা প্রমাণিত ধরে নেওয়া ঠিক নয়।","সনদে মাজহূল বা জালকারী থাকলে বর্ণনা গ্রহণযোগ্য থাকে না।","সুন্নাহর পদ্ধতি জানার জন্য নির্ভরযোগ্য বর্ণনা অনুসরণ করা জরুরি।"],"related_hadiths":[{"id":"1502","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"3411","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"2726","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E43" s="4" t="n"/>
@@ -1458,7 +1462,7 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কালো পতাকা ও মাহদী বিষয়ক মুনকার হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. খুরাসানের কালো পতাকা ও মাহদীর বাইআত নিয়ে বর্ণনাটি মুনকার; বিশেষ অংশের বিশুদ্ধ সূত্র নেই বলা হয়েছে।"},"heading":{"title":"কালো পতাকা ও মাহদী বিষয়ক মুনকার হাদিস: যাচাই ছাড়া প্রচার নয়","description":"এই বর্ণনায় সংরক্ষিত সম্পদের কাছে তিন খলীফার পুত্র নিহত হওয়া, প্রাচ্য থেকে ঝাণ্ডা বের হওয়া এবং বরফের ওপর হামাগুড়ি দিয়ে হলেও মাহদীর কাছে যাওয়ার কথা এসেছে। অন্য বর্ণনায় খুরাসানের দিক থেকে বড় দলের ঝাণ্ডার কথাও আছে। প্রদত্ত তাহকীক অনুযায়ী হাদিসটি মুনকার। সনদে ‘আলী ইবনু যায়েদ দুর্বল বলা হয়েছে। আরও বলা হয়েছে, আবূ কিলাবা আনআন সূত্রে বর্ণনা করেছেন এবং তিনি মুদাল্লিসদের অন্তর্ভুক্ত। সবচেয়ে গুরুত্বপূর্ণ বিষয় হলো, ‘আল্লাহর প্রতিনিধি মাহদী’ অংশটির বিশুদ্ধ সূত্র নেই। তাই মাহদী, কালো পতাকা, খুরাসান—এ ধরনের সংবেদনশীল বিষয়ে আবেগী প্রচার নয়; বরং নির্ভরযোগ্য সনদ দেখা প্রয়োজন।"},"teachings":["মাহদী ও ফিতনা বিষয়ক বর্ণনা প্রচারের আগে সনদ যাচাই জরুরি।","মুনকার হাদিসকে সহিহের মতো ব্যবহার করা ঠিক নয়।","কোনো বর্ণনার একটি অংশও আলাদা করে দুর্বল বা অপ্রমাণিত হতে পারে।","ধর্মীয় ভাষায় ‘আল্লাহর প্রতিনিধি’ ধরনের শব্দ ব্যবহারে সতর্কতা দরকার।"],"related_hadiths":[{"id":"4282","book_id":"4","label":"Sunan Abu Dawud"},{"id":"4284","book_id":"4","label":"Sunan Abu Dawud"},{"id":"107","book_id":"1","label":"Sahih Bukhari"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কালো পতাকা ও মাহদী বিষয়ক মুনকার হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. খুরাসানের কালো পতাকা ও মাহদীর বাইআত নিয়ে বর্ণনাটি মুনকার; বিশেষ অংশের বিশুদ্ধ সূত্র নেই বলা হয়েছে।"},"heading":{"title":"কালো পতাকা ও মাহদী বিষয়ক মুনকার হাদিস: যাচাই ছাড়া প্রচার নয়","description":"এই বর্ণনায় সংরক্ষিত সম্পদের কাছে তিন খলীফার পুত্র নিহত হওয়া, প্রাচ্য থেকে ঝাণ্ডা বের হওয়া এবং বরফের ওপর হামাগুড়ি দিয়ে হলেও মাহদীর কাছে যাওয়ার কথা এসেছে। অন্য বর্ণনায় খুরাসানের দিক থেকে বড় দলের ঝাণ্ডার কথাও আছে। প্রদত্ত তাহকীক অনুযায়ী হাদিসটি মুনকার। সনদে ‘আলী ইবনু যায়েদ দুর্বল বলা হয়েছে। আরও বলা হয়েছে, আবূ কিলাবা আনআন সূত্রে বর্ণনা করেছেন এবং তিনি মুদাল্লিসদের অন্তর্ভুক্ত। সবচেয়ে গুরুত্বপূর্ণ বিষয় হলো, ‘আল্লাহর প্রতিনিধি মাহদী’ অংশটির বিশুদ্ধ সূত্র নেই। তাই মাহদী, কালো পতাকা, খুরাসান—এ ধরনের সংবেদনশীল বিষয়ে আবেগী প্রচার নয়; বরং নির্ভরযোগ্য সনদ দেখা প্রয়োজন।"},"teachings":["মাহদী ও ফিতনা বিষয়ক বর্ণনা প্রচারের আগে সনদ যাচাই জরুরি।","মুনকার হাদিসকে সহিহের মতো ব্যবহার করা ঠিক নয়।","কোনো বর্ণনার একটি অংশও আলাদা করে দুর্বল বা অপ্রমাণিত হতে পারে।","ধর্মীয় ভাষায় ‘আল্লাহর প্রতিনিধি’ ধরনের শব্দ ব্যবহারে সতর্কতা দরকার।"],"related_hadiths":[{"id":"4282","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"4284","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"107","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
         </is>
       </c>
       <c r="E44" s="4" t="n"/>
@@ -1481,7 +1485,7 @@
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মালিকের বস্তু বহন বিষয়ক জাল হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. নিজের বস্তু নিজে বহনের অধিকার ও দুর্বলকে সাহায্য বিষয়ক বর্ণনাটি জাল; সনদে নিতান্ত দুর্বল রাবী আছে।"},"heading":{"title":"মালিকের বস্তু বহন ও সাহায্য: সুন্দর অর্থ হলেও জাল হাদিস","description":"এই বর্ণনায় বলা হয়েছে, বস্তুর মালিকই তার বস্তু বহন করার অধিক হকদার; তবে সে দুর্বল হলে তার মুসলিম ভাই তাকে সাহায্য করবে। কথাটি আচরণের দিক থেকে ভালো মনে হতে পারে, কিন্তু প্রদত্ত তাহকীক অনুযায়ী হাদিসটি জাল। সনদে ইউসুফ ইবনু যিয়াদ আল-বাসরী আছেন। ইমাম বুখারী তাকে মুনকারুল হাদিস বলেছেন। দারাকুতনী বলেছেন, তিনি বাতিল হাদিস বর্ণনার ক্ষেত্রে প্রসিদ্ধ। ইবনু হিব্বান বলেছেন, তিনি নির্ভরযোগ্যদের উদ্ধৃতিতে জাল হাদিস বর্ণনা করতেন। আরও আছে আব্দুর রহমান আল-ইফরীকী, যিনি নিতান্ত দুর্বল। তাই হাদিস যাচাইয়ের বড় শিক্ষা হলো: কোনো কথা সুন্দর নৈতিকতা শেখালেও, রাসূল (সা.)-এর নামে বলতে হলে সনদ সহিহ হতে হবে।"},"teachings":["ভালো অর্থের কথা হলেও তা জাল হাদিস হতে পারে।","রাসূলের নামে কথা বলার আগে সনদ যাচাই জরুরি।","দুর্বলকে সাহায্য করা ভালো কাজ, তবে এই নির্দিষ্ট বর্ণনা দলীল নয়।","মিথ্যার দোষে অভিযুক্ত বর্ণনাকারী থাকলে হাদিস গ্রহণযোগ্য থাকে না।"],"related_hadiths":[{"id":"107","book_id":"1","label":"Sahih Bukhari"},{"id":"5","book_id":"2","label":"Sahih Muslim"},{"id":"2442","book_id":"1","label":"Sahih Bukhari"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মালিকের বস্তু বহন বিষয়ক জাল হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. নিজের বস্তু নিজে বহনের অধিকার ও দুর্বলকে সাহায্য বিষয়ক বর্ণনাটি জাল; সনদে নিতান্ত দুর্বল রাবী আছে।"},"heading":{"title":"মালিকের বস্তু বহন ও সাহায্য: সুন্দর অর্থ হলেও জাল হাদিস","description":"এই বর্ণনায় বলা হয়েছে, বস্তুর মালিকই তার বস্তু বহন করার অধিক হকদার; তবে সে দুর্বল হলে তার মুসলিম ভাই তাকে সাহায্য করবে। কথাটি আচরণের দিক থেকে ভালো মনে হতে পারে, কিন্তু প্রদত্ত তাহকীক অনুযায়ী হাদিসটি জাল। সনদে ইউসুফ ইবনু যিয়াদ আল-বাসরী আছেন। ইমাম বুখারী তাকে মুনকারুল হাদিস বলেছেন। দারাকুতনী বলেছেন, তিনি বাতিল হাদিস বর্ণনার ক্ষেত্রে প্রসিদ্ধ। ইবনু হিব্বান বলেছেন, তিনি নির্ভরযোগ্যদের উদ্ধৃতিতে জাল হাদিস বর্ণনা করতেন। আরও আছে আব্দুর রহমান আল-ইফরীকী, যিনি নিতান্ত দুর্বল। তাই হাদিস যাচাইয়ের বড় শিক্ষা হলো: কোনো কথা সুন্দর নৈতিকতা শেখালেও, রাসূল (সা.)-এর নামে বলতে হলে সনদ সহিহ হতে হবে।"},"teachings":["ভালো অর্থের কথা হলেও তা জাল হাদিস হতে পারে।","রাসূলের নামে কথা বলার আগে সনদ যাচাই জরুরি।","দুর্বলকে সাহায্য করা ভালো কাজ, তবে এই নির্দিষ্ট বর্ণনা দলীল নয়।","মিথ্যার দোষে অভিযুক্ত বর্ণনাকারী থাকলে হাদিস গ্রহণযোগ্য থাকে না।"],"related_hadiths":[{"id":"107","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"5","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"2442","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
         </is>
       </c>
       <c r="E45" s="4" t="n"/>
@@ -1504,7 +1508,7 @@
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | পরহেজগার নিয়ে ভিত্তিহীন হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. আমি প্রত্যেক পরহেজগারের দাদা—এই কথাটির কোনো ভিত্তি নেই বলে সুয়ূতীর বক্তব্যে এসেছে।"},"heading":{"title":"পরহেজগার নিয়ে ভিত্তিহীন হাদিস: “আমি দাদা” কথার হুকুম","description":"এই বর্ণনায় বলা হয়েছে, “আমি প্রত্যেক পরহেজগার ব্যক্তির দাদা।” প্রদত্ত আলোচনায় বলা হয়েছে, হাদিসটির কোনো ভিত্তি নেই। হাফিয সুয়ূতীকে এ বিষয়ে জিজ্ঞাসা করা হলে তিনি বলেন, তিনি এ হাদিসটি চেনেন না। তাই এই বাক্যটি রাসূল صلى الله عليه وسلم-এর হাদিস হিসেবে বলা বা ছড়ানো ঠিক নয়। এখানে মূল শিক্ষা হলো—তাকওয়া বা পরহেজগারি নিয়ে কথা বলতে গিয়ে উৎসহীন বর্ণনা ব্যবহার করা উচিত নয়। তাকওয়া ইসলামের বড় বিষয়, কিন্তু তাকওয়ার মর্যাদা বোঝাতে সহীহ আয়াত ও হাদিস যথেষ্ট আছে। কোনো অচেনা বা ভিত্তিহীন কথা নবী صلى الله عليه وسلم-এর নামে বললে মানুষ ভুল ধারণা পেতে পারে। “পরহেজগার সম্পর্কে হাদিস” খোঁজার সময় নির্ভরযোগ্য বই ও যাচাই করা সূত্র দেখা দরকার।"},"teachings":["অচেনা বর্ণনা রাসূল صلى الله عليه وسلم-এর নামে বলা যাবে না।","তাকওয়ার গুরুত্ব বোঝাতে সহীহ দলিল ব্যবহার করা উচিত।","কোনো আলেম হাদিসটি না চিনলে আরও সতর্ক হওয়া দরকার।","ভিত্তিহীন কথা ছড়ালে হাদিস সম্পর্কে ভুল ধারণা তৈরি হতে পারে।"],"related_hadiths":[{"id":"13","book_id":"1","label":"Sahih Bukhari"},{"id":"2564","book_id":"2","label":"Sahih Muslim"},{"id":"1987","book_id":"5","label":"Jami at-Tirmidhi"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | পরহেজগার নিয়ে ভিত্তিহীন হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. আমি প্রত্যেক পরহেজগারের দাদা—এই কথাটির কোনো ভিত্তি নেই বলে সুয়ূতীর বক্তব্যে এসেছে।"},"heading":{"title":"পরহেজগার নিয়ে ভিত্তিহীন হাদিস: “আমি দাদা” কথার হুকুম","description":"এই বর্ণনায় বলা হয়েছে, “আমি প্রত্যেক পরহেজগার ব্যক্তির দাদা।” প্রদত্ত আলোচনায় বলা হয়েছে, হাদিসটির কোনো ভিত্তি নেই। হাফিয সুয়ূতীকে এ বিষয়ে জিজ্ঞাসা করা হলে তিনি বলেন, তিনি এ হাদিসটি চেনেন না। তাই এই বাক্যটি রাসূল صلى الله عليه وسلم-এর হাদিস হিসেবে বলা বা ছড়ানো ঠিক নয়। এখানে মূল শিক্ষা হলো—তাকওয়া বা পরহেজগারি নিয়ে কথা বলতে গিয়ে উৎসহীন বর্ণনা ব্যবহার করা উচিত নয়। তাকওয়া ইসলামের বড় বিষয়, কিন্তু তাকওয়ার মর্যাদা বোঝাতে সহীহ আয়াত ও হাদিস যথেষ্ট আছে। কোনো অচেনা বা ভিত্তিহীন কথা নবী صلى الله عليه وسلم-এর নামে বললে মানুষ ভুল ধারণা পেতে পারে। “পরহেজগার সম্পর্কে হাদিস” খোঁজার সময় নির্ভরযোগ্য বই ও যাচাই করা সূত্র দেখা দরকার।"},"teachings":["অচেনা বর্ণনা রাসূল صلى الله عليه وسلم-এর নামে বলা যাবে না।","তাকওয়ার গুরুত্ব বোঝাতে সহীহ দলিল ব্যবহার করা উচিত।","কোনো আলেম হাদিসটি না চিনলে আরও সতর্ক হওয়া দরকার।","ভিত্তিহীন কথা ছড়ালে হাদিস সম্পর্কে ভুল ধারণা তৈরি হতে পারে।"],"related_hadiths":[{"id":"13","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2564","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"1987","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"}]}</t>
         </is>
       </c>
       <c r="E46" s="4" t="n"/>
@@ -1527,7 +1531,7 @@
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | পশমী পোশাকের ফযিলত বিষয়ক জাল হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. পশমী পোশাক গ্রহণে ঈমানের মধুরতা ও আখেরাতে পরিচয়ের কথাটি জাল; সনদে জালকারী রাবীর কথা আছে।"},"heading":{"title":"পশমী পোশাকের ফযিলত নিয়ে জাল হাদিস: বাহ্যিক পোশাক নয়, দলীল জরুরি","description":"এই দীর্ঘ বর্ণনায় পশমী পোশাক গ্রহণ করলে হৃদয়ে ঈমানের মধুরতা পাওয়া, কম খাদ্য পাওয়া, আখেরাতে চেনা যাওয়া এবং অন্তর নরম হওয়া ইত্যাদি কথা বলা হয়েছে। প্রদত্ত তাহকীক অনুযায়ী এটি জাল। ইবনুল জাওযী বলেছেন, হাদিসটি সহিহ নয়; কুদায়মী হাদিস জাল করতেন এবং তার শাইখ দ্বারা দলীল নেওয়া যায় না। সুয়ূতী কিছু অংশকে মারফূ হিসেবে আলাদা করার কথা উল্লেখ করলেও, আলোচনায় বলা হয়েছে সেই সূত্রেও জালকারী মুহাম্মদ ইবনু ইউনুস আছেন। তার সম্পর্কে ইবনু হিব্বান বলেছেন, তিনি বহু হাদিস জাল করেছেন। তাই পোশাক, যুহদ, কম খাওয়া, অন্তরের অবস্থা—এসব বিষয়ে অতিরঞ্জিত কথা শুনলে সতর্ক হতে হবে। ইসলামে পোশাকের মূল্য আছে, কিন্তু কোনো নির্দিষ্ট পোশাকের নামে বানানো ফযিলত প্রচার করা ঠিক নয়।"},"teachings":["নির্দিষ্ট পোশাকের নামে অতিরঞ্জিত ফযিলত প্রচার করা থেকে সতর্ক থাকা উচিত।","সনদে জালকারী থাকলে বর্ণনা গ্রহণযোগ্য নয়।","অন্তরের নরমতা বা ঈমানের মধুরতা নিয়ে দাবি করতে সহিহ দলীল দরকার।","যুহদ বা সরল জীবন নিয়ে কথা বললেও জাল হাদিস ব্যবহার করা ঠিক নয়।"],"related_hadiths":[{"id":"107","book_id":"1","label":"Sahih Bukhari"},{"id":"5","book_id":"2","label":"Sahih Muslim"},{"id":"5789","book_id":"1","label":"Sahih Bukhari"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | পশমী পোশাকের ফযিলত বিষয়ক জাল হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. পশমী পোশাক গ্রহণে ঈমানের মধুরতা ও আখেরাতে পরিচয়ের কথাটি জাল; সনদে জালকারী রাবীর কথা আছে।"},"heading":{"title":"পশমী পোশাকের ফযিলত নিয়ে জাল হাদিস: বাহ্যিক পোশাক নয়, দলীল জরুরি","description":"এই দীর্ঘ বর্ণনায় পশমী পোশাক গ্রহণ করলে হৃদয়ে ঈমানের মধুরতা পাওয়া, কম খাদ্য পাওয়া, আখেরাতে চেনা যাওয়া এবং অন্তর নরম হওয়া ইত্যাদি কথা বলা হয়েছে। প্রদত্ত তাহকীক অনুযায়ী এটি জাল। ইবনুল জাওযী বলেছেন, হাদিসটি সহিহ নয়; কুদায়মী হাদিস জাল করতেন এবং তার শাইখ দ্বারা দলীল নেওয়া যায় না। সুয়ূতী কিছু অংশকে মারফূ হিসেবে আলাদা করার কথা উল্লেখ করলেও, আলোচনায় বলা হয়েছে সেই সূত্রেও জালকারী মুহাম্মদ ইবনু ইউনুস আছেন। তার সম্পর্কে ইবনু হিব্বান বলেছেন, তিনি বহু হাদিস জাল করেছেন। তাই পোশাক, যুহদ, কম খাওয়া, অন্তরের অবস্থা—এসব বিষয়ে অতিরঞ্জিত কথা শুনলে সতর্ক হতে হবে। ইসলামে পোশাকের মূল্য আছে, কিন্তু কোনো নির্দিষ্ট পোশাকের নামে বানানো ফযিলত প্রচার করা ঠিক নয়।"},"teachings":["নির্দিষ্ট পোশাকের নামে অতিরঞ্জিত ফযিলত প্রচার করা থেকে সতর্ক থাকা উচিত।","সনদে জালকারী থাকলে বর্ণনা গ্রহণযোগ্য নয়।","অন্তরের নরমতা বা ঈমানের মধুরতা নিয়ে দাবি করতে সহিহ দলীল দরকার।","যুহদ বা সরল জীবন নিয়ে কথা বললেও জাল হাদিস ব্যবহার করা ঠিক নয়।"],"related_hadiths":[{"id":"107","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"5","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"5789","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
         </is>
       </c>
       <c r="E47" s="4" t="n"/>
@@ -1550,7 +1554,7 @@
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | দুর্বল, পিতা-মাতা ও অধীনস্তদের ইহসান বিষয়ক জাল হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. দুর্বলকে দয়া, পিতা-মাতার প্রতি নম্রতা ও অধীনস্তদের ইহসান নিয়ে বর্ণনাটি জাল; সনদে জালকারী আছে।"},"heading":{"title":"দুর্বলকে দয়া ও পিতা-মাতার নম্রতা: ভালো শিক্ষা, কিন্তু জাল বর্ণনা","description":"এই বর্ণনায় তিনটি গুণের কথা এসেছে: দুর্বলকে দয়া করা, পিতা-মাতার প্রতি নম্র ব্যবহার করা এবং অধীনস্তদের প্রতি ইহসান করা। বলা হয়েছে, এগুলো যার মাঝে থাকবে আল্লাহ তার বক্ষ প্রশস্ত করবেন এবং জান্নাতে প্রবেশ করাবেন। কিন্তু প্রদত্ত তাহকীক অনুযায়ী হাদিসটি জাল। তিরমিযী এটি গারীব বলেছেন। আলবানী উল্লেখ করেছেন, সনদে আব্দুল্লাহ ইবনু ইবরাহীম আল-গিফারী আছেন, যার সম্পর্কে ইবনু হিব্বান বলেছেন তিনি হাদিস জাল করতেন। তার পিতাও মাজহূল। তাই দুর্বলদের প্রতি দয়া, পিতা-মাতার সঙ্গে নম্রতা ও অধীনস্তদের ভালো ব্যবহার অবশ্যই ভালো চরিত্রের বিষয়, কিন্তু এই নির্দিষ্ট প্রতিশ্রুতি রাসূলের নামে প্রমাণিত নয়। ধর্মীয় ভাষায় সঠিক উৎস জানা খুব জরুরি।"},"teachings":["ভালো চরিত্রের কথা থাকলেও নির্দিষ্ট বর্ণনা জাল হতে পারে।","জান্নাতের প্রতিশ্রুতি ধরনের কথা সহিহ দলীল ছাড়া বলা উচিত নয়।","জালকারী ও মাজহূল রাবী থাকলে বর্ণনা দলীল হয় না।","দুর্বল, পিতা-মাতা ও অধীনস্তদের অধিকার নিয়ে কথা বললেও সতর্কতা দরকার।"],"related_hadiths":[{"id":"5971","book_id":"1","label":"Sahih Bukhari"},{"id":"2548","book_id":"2","label":"Sahih Muslim"},{"id":"6011","book_id":"1","label":"Sahih Bukhari"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | দুর্বল, পিতা-মাতা ও অধীনস্তদের ইহসান বিষয়ক জাল হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. দুর্বলকে দয়া, পিতা-মাতার প্রতি নম্রতা ও অধীনস্তদের ইহসান নিয়ে বর্ণনাটি জাল; সনদে জালকারী আছে।"},"heading":{"title":"দুর্বলকে দয়া ও পিতা-মাতার নম্রতা: ভালো শিক্ষা, কিন্তু জাল বর্ণনা","description":"এই বর্ণনায় তিনটি গুণের কথা এসেছে: দুর্বলকে দয়া করা, পিতা-মাতার প্রতি নম্র ব্যবহার করা এবং অধীনস্তদের প্রতি ইহসান করা। বলা হয়েছে, এগুলো যার মাঝে থাকবে আল্লাহ তার বক্ষ প্রশস্ত করবেন এবং জান্নাতে প্রবেশ করাবেন। কিন্তু প্রদত্ত তাহকীক অনুযায়ী হাদিসটি জাল। তিরমিযী এটি গারীব বলেছেন। আলবানী উল্লেখ করেছেন, সনদে আব্দুল্লাহ ইবনু ইবরাহীম আল-গিফারী আছেন, যার সম্পর্কে ইবনু হিব্বান বলেছেন তিনি হাদিস জাল করতেন। তার পিতাও মাজহূল। তাই দুর্বলদের প্রতি দয়া, পিতা-মাতার সঙ্গে নম্রতা ও অধীনস্তদের ভালো ব্যবহার অবশ্যই ভালো চরিত্রের বিষয়, কিন্তু এই নির্দিষ্ট প্রতিশ্রুতি রাসূলের নামে প্রমাণিত নয়। ধর্মীয় ভাষায় সঠিক উৎস জানা খুব জরুরি।"},"teachings":["ভালো চরিত্রের কথা থাকলেও নির্দিষ্ট বর্ণনা জাল হতে পারে।","জান্নাতের প্রতিশ্রুতি ধরনের কথা সহিহ দলীল ছাড়া বলা উচিত নয়।","জালকারী ও মাজহূল রাবী থাকলে বর্ণনা দলীল হয় না।","দুর্বল, পিতা-মাতা ও অধীনস্তদের অধিকার নিয়ে কথা বললেও সতর্কতা দরকার।"],"related_hadiths":[{"id":"5971","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2548","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"6011","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
         </is>
       </c>
       <c r="E48" s="4" t="n"/>
@@ -1573,7 +1577,7 @@
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | পানি পান করানো ও সুপারিশ বিষয়ক দুর্বল হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. কিয়ামতে পানি পান করানো বা কাজে সাহায্যের বিনিময়ে সুপারিশের বর্ণনাটি দুর্বল; ইয়াযীদ রুকাশী দুর্বল রাবী।"},"heading":{"title":"পানি পান করানো ও কিয়ামতের সুপারিশ: দুর্বল বর্ণনার তাহকীক","description":"এই বর্ণনায় কিয়ামতের দিন মানুষের কাতার, জাহান্নামের এক ব্যক্তির স্মরণ করানো এবং একবার পানি পান করানো বা পবিত্রতার জন্য পানি দেওয়ার কারণে সুপারিশের কথা এসেছে। আরও একজনের প্রয়োজনীয় কাজে যাওয়ার কথাও উল্লেখ আছে। কিন্তু প্রদত্ত তাহকীক অনুযায়ী হাদিসটি দুর্বল। ইবনু মাজাহ এটি ইয়াযীদ রুকাশী সূত্রে আনাস (রাঃ) থেকে বর্ণনা করেছেন। ইয়াযীদ ইবনু আবান রুকাশী সম্পর্কে বলা হয়েছে, তিনি দুর্বল। অন্য সূত্রেও আনাস (রাঃ) থেকে এমন বর্ণনা এসেছে, কিন্তু কোনোটি সহিহ নয়। এখানে পানি পান করানো, ছোট সাহায্য, সুপারিশ—এসব বিষয় আবেগপূর্ণ হলেও এই নির্দিষ্ট কিয়ামতের দৃশ্যকে সহিহ হাদিস হিসেবে বলা ঠিক নয়। হাদিসের মান জানা থাকলে ধর্মীয় বক্তব্য নিরাপদ থাকে।"},"teachings":["আবেগপূর্ণ কিয়ামতের বর্ণনা হলেও সনদ যাচাই করা দরকার।","দুর্বল রাবীর বর্ণনা দিয়ে নিশ্চিত প্রতিশ্রুতি দেওয়া ঠিক নয়।","মানুষকে পানি দেওয়া ও সাহায্য করা ভালো কাজ, তবে এই বর্ণনা সহিহ নয়।","সুপারিশ বিষয়ক কথা বলার সময় সহিহ দলীল দরকার।"],"related_hadiths":[{"id":"2363","book_id":"1","label":"Sahih Bukhari"},{"id":"2699","book_id":"2","label":"Sahih Muslim"},{"id":"3684","book_id":"6","label":"Sunan Ibn Majah"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | পানি পান করানো ও সুপারিশ বিষয়ক দুর্বল হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. কিয়ামতে পানি পান করানো বা কাজে সাহায্যের বিনিময়ে সুপারিশের বর্ণনাটি দুর্বল; ইয়াযীদ রুকাশী দুর্বল রাবী।"},"heading":{"title":"পানি পান করানো ও কিয়ামতের সুপারিশ: দুর্বল বর্ণনার তাহকীক","description":"এই বর্ণনায় কিয়ামতের দিন মানুষের কাতার, জাহান্নামের এক ব্যক্তির স্মরণ করানো এবং একবার পানি পান করানো বা পবিত্রতার জন্য পানি দেওয়ার কারণে সুপারিশের কথা এসেছে। আরও একজনের প্রয়োজনীয় কাজে যাওয়ার কথাও উল্লেখ আছে। কিন্তু প্রদত্ত তাহকীক অনুযায়ী হাদিসটি দুর্বল। ইবনু মাজাহ এটি ইয়াযীদ রুকাশী সূত্রে আনাস (রাঃ) থেকে বর্ণনা করেছেন। ইয়াযীদ ইবনু আবান রুকাশী সম্পর্কে বলা হয়েছে, তিনি দুর্বল। অন্য সূত্রেও আনাস (রাঃ) থেকে এমন বর্ণনা এসেছে, কিন্তু কোনোটি সহিহ নয়। এখানে পানি পান করানো, ছোট সাহায্য, সুপারিশ—এসব বিষয় আবেগপূর্ণ হলেও এই নির্দিষ্ট কিয়ামতের দৃশ্যকে সহিহ হাদিস হিসেবে বলা ঠিক নয়। হাদিসের মান জানা থাকলে ধর্মীয় বক্তব্য নিরাপদ থাকে।"},"teachings":["আবেগপূর্ণ কিয়ামতের বর্ণনা হলেও সনদ যাচাই করা দরকার।","দুর্বল রাবীর বর্ণনা দিয়ে নিশ্চিত প্রতিশ্রুতি দেওয়া ঠিক নয়।","মানুষকে পানি দেওয়া ও সাহায্য করা ভালো কাজ, তবে এই বর্ণনা সহিহ নয়।","সুপারিশ বিষয়ক কথা বলার সময় সহিহ দলীল দরকার।"],"related_hadiths":[{"id":"2363","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2699","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"3684","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
         </is>
       </c>
       <c r="E49" s="4" t="n"/>
@@ -1596,7 +1600,7 @@
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ইসলামের তিন স্তম্ভ বলা দুর্বল হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. ইসলামের ভিত্তি তিনটি বলে সালাত বা সওম ছাড়লে কুফর বলা বর্ণনাটি দুর্বল; সহিহ হাদিসে ইসলামের পাঁচ স্তম্ভ আছে।"},"heading":{"title":"ইসলামের তিন স্তম্ভ বলা দুর্বল হাদিস: পাঁচ স্তম্ভের সহিহ বর্ণনার বিপরীত","description":"এই বর্ণনায় বলা হয়েছে, ইসলামের হাতল ও দ্বীনের স্তম্ভ তিনটি: শাহাদাত, ফরয সালাত ও রমাযানের সওম। আরও বলা হয়েছে, এগুলোর কোনো একটি ছেড়ে দিলে সে কুফরকারী হবে এবং তার রক্ত হালাল। প্রদত্ত তাহকীক অনুযায়ী হাদিসটি দুর্বল। সনদে আম্র ইবনু মালেক আন-নুকারী আছেন, যাকে ইবনু হিব্বান ছাড়া অন্য কেউ নির্ভরযোগ্য বলেননি বলে উল্লেখ করা হয়েছে। মুয়াম্মিল ইবনু ইসমাঈল সত্যবাদী হলেও বহু ভুল করতেন। সবচেয়ে বড় কথা, এটি ইসলামের স্তম্ভ পাঁচটি উল্লেখকারী সহিহ হাদিসের বিপরীত। তাই ইসলাম, ঈমান, সালাত, রমাযানের সওম ও কুফর বিষয়ে খুব সতর্ক ভাষা দরকার। কারও রক্ত হালাল বা কুফরের মতো গুরুতর কথা দুর্বল বর্ণনার ওপর বলা যায় না।"},"teachings":["ইসলামের স্তম্ভ সম্পর্কে সহিহ বর্ণনা অনুসরণ করতে হয়।","কুফর বা রক্ত হালালের মতো গুরুতর কথা দুর্বল হাদিসে বলা যায় না।","সনদের দুর্বলতা থাকলে আকীদা ও আহকামের দলীল হয় না।","সহিহ হাদিসের বিপরীত বর্ণনা গ্রহণে সতর্কতা জরুরি।"],"related_hadiths":[{"id":"8","book_id":"1","label":"Sahih Bukhari"},{"id":"16","book_id":"2","label":"Sahih Muslim"},{"id":"2616","book_id":"5","label":"Jami at-Tirmidhi"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ইসলামের তিন স্তম্ভ বলা দুর্বল হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. ইসলামের ভিত্তি তিনটি বলে সালাত বা সওম ছাড়লে কুফর বলা বর্ণনাটি দুর্বল; সহিহ হাদিসে ইসলামের পাঁচ স্তম্ভ আছে।"},"heading":{"title":"ইসলামের তিন স্তম্ভ বলা দুর্বল হাদিস: পাঁচ স্তম্ভের সহিহ বর্ণনার বিপরীত","description":"এই বর্ণনায় বলা হয়েছে, ইসলামের হাতল ও দ্বীনের স্তম্ভ তিনটি: শাহাদাত, ফরয সালাত ও রমাযানের সওম। আরও বলা হয়েছে, এগুলোর কোনো একটি ছেড়ে দিলে সে কুফরকারী হবে এবং তার রক্ত হালাল। প্রদত্ত তাহকীক অনুযায়ী হাদিসটি দুর্বল। সনদে আম্র ইবনু মালেক আন-নুকারী আছেন, যাকে ইবনু হিব্বান ছাড়া অন্য কেউ নির্ভরযোগ্য বলেননি বলে উল্লেখ করা হয়েছে। মুয়াম্মিল ইবনু ইসমাঈল সত্যবাদী হলেও বহু ভুল করতেন। সবচেয়ে বড় কথা, এটি ইসলামের স্তম্ভ পাঁচটি উল্লেখকারী সহিহ হাদিসের বিপরীত। তাই ইসলাম, ঈমান, সালাত, রমাযানের সওম ও কুফর বিষয়ে খুব সতর্ক ভাষা দরকার। কারও রক্ত হালাল বা কুফরের মতো গুরুতর কথা দুর্বল বর্ণনার ওপর বলা যায় না।"},"teachings":["ইসলামের স্তম্ভ সম্পর্কে সহিহ বর্ণনা অনুসরণ করতে হয়।","কুফর বা রক্ত হালালের মতো গুরুতর কথা দুর্বল হাদিসে বলা যায় না।","সনদের দুর্বলতা থাকলে আকীদা ও আহকামের দলীল হয় না।","সহিহ হাদিসের বিপরীত বর্ণনা গ্রহণে সতর্কতা জরুরি।"],"related_hadiths":[{"id":"8","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"16","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"2616","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"}]}</t>
         </is>
       </c>
       <c r="E50" s="4" t="n"/>
@@ -1619,7 +1623,7 @@
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | পথভ্রষ্ট তওবাকারী মুমিন বিষয়ক জাল হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. আল্লাহ পথভ্রষ্ট তওবাকারী মুমিনকে ভালবাসেন—এ বর্ণনাটি জাল; সনদে জালকারী ও মাজহূল রাবী আছে।"},"heading":{"title":"পথভ্রষ্ট তওবাকারী মুমিনকে ভালবাসা: জাল হাদিসের সনদ বিশ্লেষণ","description":"এই বর্ণনায় বলা হয়েছে, আল্লাহ পথভ্রষ্ট তওবাকারী মুমিন বান্দাকে ভালবাসেন। কিন্তু প্রদত্ত তাহকীক অনুযায়ী হাদিসটি জাল। সনদে আবু আব্দিল্লাহ মাসলামা আর-রাযী আছেন, যার জীবনী পাওয়া যায়নি বলে উল্লেখ করা হয়েছে। আবূ আম্র আল-বাজালী সম্পর্কে ইবনু হিব্বান বলেছেন, তার মাধ্যমে দলীল গ্রহণ করা হালাল নয়। হাফিয ইবনু হাজারের উদ্ধৃতিতে তাকে আবীদা ইবনু আব্দির রহমান বলা হয়েছে এবং তার সম্পর্কে বলা হয়েছে, তিনি নির্ভরযোগ্যদের নামে জাল হাদিস বর্ণনা করতেন। আব্দুল মালেক ইবনু সুফিয়ান আস-সাকাফীও মাজহূল। তাই তওবা, আল্লাহর ভালোবাসা ও মুমিনের ফিরে আসার কথা বললেও এই নির্দিষ্ট বাক্য প্রমাণিত নয়।"},"teachings":["আল্লাহর ভালোবাসা নিয়ে নির্দিষ্ট দাবি করতে সহিহ দলীল দরকার।","মাজহূল ও জালকারী রাবী থাকলে বর্ণনা গ্রহণযোগ্য নয়।","তওবা বিষয়ে সুন্দর বাক্য হলেও তা হাদিস হতে নাও পারে।","ধর্মীয় আশা দেওয়ার সময় জাল বর্ণনা ব্যবহার করা উচিত নয়।"],"related_hadiths":[{"id":"6309","book_id":"1","label":"Sahih Bukhari"},{"id":"2747","book_id":"2","label":"Sahih Muslim"},{"id":"3537","book_id":"5","label":"Jami at-Tirmidhi"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | পথভ্রষ্ট তওবাকারী মুমিন বিষয়ক জাল হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. আল্লাহ পথভ্রষ্ট তওবাকারী মুমিনকে ভালবাসেন—এ বর্ণনাটি জাল; সনদে জালকারী ও মাজহূল রাবী আছে।"},"heading":{"title":"পথভ্রষ্ট তওবাকারী মুমিনকে ভালবাসা: জাল হাদিসের সনদ বিশ্লেষণ","description":"এই বর্ণনায় বলা হয়েছে, আল্লাহ পথভ্রষ্ট তওবাকারী মুমিন বান্দাকে ভালবাসেন। কিন্তু প্রদত্ত তাহকীক অনুযায়ী হাদিসটি জাল। সনদে আবু আব্দিল্লাহ মাসলামা আর-রাযী আছেন, যার জীবনী পাওয়া যায়নি বলে উল্লেখ করা হয়েছে। আবূ আম্র আল-বাজালী সম্পর্কে ইবনু হিব্বান বলেছেন, তার মাধ্যমে দলীল গ্রহণ করা হালাল নয়। হাফিয ইবনু হাজারের উদ্ধৃতিতে তাকে আবীদা ইবনু আব্দির রহমান বলা হয়েছে এবং তার সম্পর্কে বলা হয়েছে, তিনি নির্ভরযোগ্যদের নামে জাল হাদিস বর্ণনা করতেন। আব্দুল মালেক ইবনু সুফিয়ান আস-সাকাফীও মাজহূল। তাই তওবা, আল্লাহর ভালোবাসা ও মুমিনের ফিরে আসার কথা বললেও এই নির্দিষ্ট বাক্য প্রমাণিত নয়।"},"teachings":["আল্লাহর ভালোবাসা নিয়ে নির্দিষ্ট দাবি করতে সহিহ দলীল দরকার।","মাজহূল ও জালকারী রাবী থাকলে বর্ণনা গ্রহণযোগ্য নয়।","তওবা বিষয়ে সুন্দর বাক্য হলেও তা হাদিস হতে নাও পারে।","ধর্মীয় আশা দেওয়ার সময় জাল বর্ণনা ব্যবহার করা উচিত নয়।"],"related_hadiths":[{"id":"6309","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2747","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"3537","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"}]}</t>
         </is>
       </c>
       <c r="E51" s="4" t="n"/>
@@ -1642,7 +1646,7 @@
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | তওবাকারী যুবক বিষয়ক দুর্বল হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. আল্লাহ তওবাকারী যুবককে ভালবাসেন—এ বর্ণনা দুর্বল; ইবনু আবিদ দুনিয়া ও আবূশ শাইখ দুর্বল সনদে এনেছেন।"},"heading":{"title":"তওবাকারী যুবককে আল্লাহ ভালবাসেন: দুর্বল হাদিসের তাহকীক","description":"এই বর্ণনায় বলা হয়েছে, আল্লাহ তওবাকারী যুবককে ভালবাসেন। কথা হিসেবে এটি তওবা ও যুবকদের আল্লাহর পথে ফিরে আসার প্রতি উৎসাহ দেয়। কিন্তু প্রদত্ত তাহকীক অনুযায়ী হাদিসটি দুর্বল। হাফিয ইরাকী বলেছেন, ইবনু আবিদ দুনিয়া আত-তাওবাহ গ্রন্থে এবং আবূশ শাইখ কিতাবুস সাওয়াব গ্রন্থে আনাস (রাঃ)-এর হাদিস হিসেবে দুর্বল সনদে এটি উল্লেখ করেছেন। তাই তওবাকারী যুবক, যৌবনে তওবা, আল্লাহর ভালোবাসা—এসব বিষয়ে আলোচনা করা যায়, তবে এই নির্দিষ্ট বাক্যকে সহিহ হাদিস হিসেবে বলা ঠিক নয়। তওবা সম্পর্কে সহিহ দলীল অনেক আছে; তাই দুর্বল বর্ণনার ওপর নির্ভর না করে নির্ভরযোগ্য বর্ণনা ব্যবহার করাই ভালো।"},"teachings":["যুবকদের তওবার কথা বলা ভালো, তবে দুর্বল বর্ণনাকে সহিহ বলা যাবে না।","আল্লাহর ভালোবাসা নিয়ে নির্দিষ্ট বাক্য প্রচারের আগে সনদ দেখা দরকার।","দুর্বল সনদ মানে বর্ণনাটি প্রমাণের স্তরে শক্ত নয়।","তওবা বিষয়ে সহিহ দলীল ব্যবহার করা বেশি নিরাপদ।"],"related_hadiths":[{"id":"6309","book_id":"1","label":"Sahih Bukhari"},{"id":"2749","book_id":"2","label":"Sahih Muslim"},{"id":"6479","book_id":"1","label":"Sahih Bukhari"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | তওবাকারী যুবক বিষয়ক দুর্বল হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. আল্লাহ তওবাকারী যুবককে ভালবাসেন—এ বর্ণনা দুর্বল; ইবনু আবিদ দুনিয়া ও আবূশ শাইখ দুর্বল সনদে এনেছেন।"},"heading":{"title":"তওবাকারী যুবককে আল্লাহ ভালবাসেন: দুর্বল হাদিসের তাহকীক","description":"এই বর্ণনায় বলা হয়েছে, আল্লাহ তওবাকারী যুবককে ভালবাসেন। কথা হিসেবে এটি তওবা ও যুবকদের আল্লাহর পথে ফিরে আসার প্রতি উৎসাহ দেয়। কিন্তু প্রদত্ত তাহকীক অনুযায়ী হাদিসটি দুর্বল। হাফিয ইরাকী বলেছেন, ইবনু আবিদ দুনিয়া আত-তাওবাহ গ্রন্থে এবং আবূশ শাইখ কিতাবুস সাওয়াব গ্রন্থে আনাস (রাঃ)-এর হাদিস হিসেবে দুর্বল সনদে এটি উল্লেখ করেছেন। তাই তওবাকারী যুবক, যৌবনে তওবা, আল্লাহর ভালোবাসা—এসব বিষয়ে আলোচনা করা যায়, তবে এই নির্দিষ্ট বাক্যকে সহিহ হাদিস হিসেবে বলা ঠিক নয়। তওবা সম্পর্কে সহিহ দলীল অনেক আছে; তাই দুর্বল বর্ণনার ওপর নির্ভর না করে নির্ভরযোগ্য বর্ণনা ব্যবহার করাই ভালো।"},"teachings":["যুবকদের তওবার কথা বলা ভালো, তবে দুর্বল বর্ণনাকে সহিহ বলা যাবে না।","আল্লাহর ভালোবাসা নিয়ে নির্দিষ্ট বাক্য প্রচারের আগে সনদ দেখা দরকার।","দুর্বল সনদ মানে বর্ণনাটি প্রমাণের স্তরে শক্ত নয়।","তওবা বিষয়ে সহিহ দলীল ব্যবহার করা বেশি নিরাপদ।"],"related_hadiths":[{"id":"6309","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2749","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"6479","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
         </is>
       </c>
       <c r="E52" s="4" t="n"/>
@@ -1665,7 +1669,7 @@
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | যৌবন আল্লাহর আনুগত্যে কাটানো বিষয়ক জাল হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. যৌবন আল্লাহর আনুগত্যে কাটানো যুবককে আল্লাহ ভালবাসেন—এ বর্ণনাটি জাল; সনদে মিথ্যুক রাবী আছে।"},"heading":{"title":"যৌবন আল্লাহর আনুগত্যে কাটানো: ভালো অর্থ, কিন্তু এই বর্ণনা জাল","description":"এই বর্ণনায় বলা হয়েছে, আল্লাহ সেই যুবককে ভালবাসেন, যে তার যৌবনকাল আল্লাহর আনুগত্যে কাটায়। অর্থের দিক থেকে এটি যুবকদের জন্য সুন্দর উপদেশ মনে হতে পারে। কিন্তু প্রদত্ত তাহকীক অনুযায়ী হাদিসটি জাল। আবূ নু‘য়াইম ও দাইলামী এটি মুহাম্মাদ ইবনুল ফযল ইবনু আতিয়া সূত্রে বর্ণনা করেছেন। আলবানী বলেছেন, এ সনদ জাল; কারণ মুহাম্মাদ ইবনুল ফযল মিথ্যুক। আরও বলা হয়েছে, উমার ইবনু আব্দিল আযীয ও ইবনু উমার (রাঃ)-এর মধ্যে সনদ বিচ্ছিন্নতার আশঙ্কা আছে। তাই যুবক, আনুগত্য, ইবাদত ও আল্লাহর ভালোবাসা বিষয়ে কথা বললেও এই নির্দিষ্ট ভাষা রাসূলের নামে বলা যাবে না। সহিহ বর্ণনায় যুবকের ইবাদতের মর্যাদা আছে, সেটিই ব্যবহার করা উচিত।"},"teachings":["সুন্দর অর্থের বর্ণনাও সনদে মিথ্যুক থাকলে জাল হয়।","যুবকদের আনুগত্যে উৎসাহ দিতে সহিহ দলীল ব্যবহার করা দরকার।","সনদে বিচ্ছিন্নতা থাকলে বর্ণনার মান দুর্বল হয়।","রাসূলের নামে কোনো বাক্য বলার আগে উৎস যাচাই করা জরুরি।"],"related_hadiths":[{"id":"660","book_id":"1","label":"Sahih Bukhari"},{"id":"1031","book_id":"2","label":"Sahih Muslim"},{"id":"6479","book_id":"1","label":"Sahih Bukhari"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | যৌবন আল্লাহর আনুগত্যে কাটানো বিষয়ক জাল হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. যৌবন আল্লাহর আনুগত্যে কাটানো যুবককে আল্লাহ ভালবাসেন—এ বর্ণনাটি জাল; সনদে মিথ্যুক রাবী আছে।"},"heading":{"title":"যৌবন আল্লাহর আনুগত্যে কাটানো: ভালো অর্থ, কিন্তু এই বর্ণনা জাল","description":"এই বর্ণনায় বলা হয়েছে, আল্লাহ সেই যুবককে ভালবাসেন, যে তার যৌবনকাল আল্লাহর আনুগত্যে কাটায়। অর্থের দিক থেকে এটি যুবকদের জন্য সুন্দর উপদেশ মনে হতে পারে। কিন্তু প্রদত্ত তাহকীক অনুযায়ী হাদিসটি জাল। আবূ নু‘য়াইম ও দাইলামী এটি মুহাম্মাদ ইবনুল ফযল ইবনু আতিয়া সূত্রে বর্ণনা করেছেন। আলবানী বলেছেন, এ সনদ জাল; কারণ মুহাম্মাদ ইবনুল ফযল মিথ্যুক। আরও বলা হয়েছে, উমার ইবনু আব্দিল আযীয ও ইবনু উমার (রাঃ)-এর মধ্যে সনদ বিচ্ছিন্নতার আশঙ্কা আছে। তাই যুবক, আনুগত্য, ইবাদত ও আল্লাহর ভালোবাসা বিষয়ে কথা বললেও এই নির্দিষ্ট ভাষা রাসূলের নামে বলা যাবে না। সহিহ বর্ণনায় যুবকের ইবাদতের মর্যাদা আছে, সেটিই ব্যবহার করা উচিত।"},"teachings":["সুন্দর অর্থের বর্ণনাও সনদে মিথ্যুক থাকলে জাল হয়।","যুবকদের আনুগত্যে উৎসাহ দিতে সহিহ দলীল ব্যবহার করা দরকার।","সনদে বিচ্ছিন্নতা থাকলে বর্ণনার মান দুর্বল হয়।","রাসূলের নামে কোনো বাক্য বলার আগে উৎস যাচাই করা জরুরি।"],"related_hadiths":[{"id":"660","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"1031","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"6479","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
         </is>
       </c>
       <c r="E53" s="4" t="n"/>
@@ -1688,7 +1692,7 @@
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | পরিষ্কার-পরিচ্ছন্ন ইবাদতকারী বিষয়ক জাল হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. পরিষ্কার-পরিচ্ছন্নতার সঙ্গে ইবাদতকারীকে আল্লাহ ভালবাসেন—এ বর্ণনাটি জাল; গিফারী রাবীর জাল করার দোষ আছে।"},"heading":{"title":"পরিষ্কার-পরিচ্ছন্নতার সঙ্গে ইবাদত: এই নির্দিষ্ট বর্ণনা জাল","description":"এই বর্ণনায় বলা হয়েছে, আল্লাহ পরিষ্কার-পরিচ্ছন্নতার সঙ্গে ইবাদতকারীকে ভালবাসেন। পরিষ্কার-পরিচ্ছন্নতা ইসলামে গুরুত্বপূর্ণ হলেও প্রদত্ত তাহকীক অনুযায়ী এই নির্দিষ্ট হাদিসটি জাল। খাতীব বাগদাদী এটি আব্দুল্লাহ ইবনু ইবরাহীম আল-গিফারী সূত্রে বর্ণনা করেছেন। আলবানী বলেছেন, এ সনদ জাল; কারণ গিফারী জাল করার দোষে দোষী। তার শাইখ মুনকাদির ইবনু মুহাম্মাদও হাদিসের ক্ষেত্রে দুর্বল বলে উল্লেখ করা হয়েছে। তাই তাহারাত, পরিচ্ছন্নতা ও ইবাদত বিষয়ে বক্তব্য দিতে গেলে সহিহ দলীল ব্যবহার করা দরকার। কোনো কথা ইসলামের সাধারণ শিক্ষার সঙ্গে মিললেও, সেটি রাসূলের নামে নির্দিষ্ট হাদিস হিসেবে প্রমাণিত হতে হবে। এই সতর্কতাই হাদিস যাচাইয়ের মূল শিক্ষা।"},"teachings":["পরিষ্কার-পরিচ্ছন্নতা গুরুত্বপূর্ণ, কিন্তু এই নির্দিষ্ট বর্ণনা জাল।","সনদে জালকারী থাকলে হাদিস গ্রহণযোগ্য নয়।","সাধারণ ইসলামি শিক্ষার সঙ্গে মিল থাকলেই কোনো বাক্য হাদিস হয় না।","ইবাদত ও তাহারাত বিষয়ে নির্ভরযোগ্য দলীল ব্যবহার করা উচিত।"],"related_hadiths":[{"id":"223","book_id":"2","label":"Sahih Muslim"},{"id":"1","book_id":"1","label":"Sahih Bukhari"},{"id":"61","book_id":"4","label":"Sunan Abu Dawud"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | পরিষ্কার-পরিচ্ছন্ন ইবাদতকারী বিষয়ক জাল হাদিস","description":"$book_name$ $hadith_number$ - $chapter_name$. পরিষ্কার-পরিচ্ছন্নতার সঙ্গে ইবাদতকারীকে আল্লাহ ভালবাসেন—এ বর্ণনাটি জাল; গিফারী রাবীর জাল করার দোষ আছে।"},"heading":{"title":"পরিষ্কার-পরিচ্ছন্নতার সঙ্গে ইবাদত: এই নির্দিষ্ট বর্ণনা জাল","description":"এই বর্ণনায় বলা হয়েছে, আল্লাহ পরিষ্কার-পরিচ্ছন্নতার সঙ্গে ইবাদতকারীকে ভালবাসেন। পরিষ্কার-পরিচ্ছন্নতা ইসলামে গুরুত্বপূর্ণ হলেও প্রদত্ত তাহকীক অনুযায়ী এই নির্দিষ্ট হাদিসটি জাল। খাতীব বাগদাদী এটি আব্দুল্লাহ ইবনু ইবরাহীম আল-গিফারী সূত্রে বর্ণনা করেছেন। আলবানী বলেছেন, এ সনদ জাল; কারণ গিফারী জাল করার দোষে দোষী। তার শাইখ মুনকাদির ইবনু মুহাম্মাদও হাদিসের ক্ষেত্রে দুর্বল বলে উল্লেখ করা হয়েছে। তাই তাহারাত, পরিচ্ছন্নতা ও ইবাদত বিষয়ে বক্তব্য দিতে গেলে সহিহ দলীল ব্যবহার করা দরকার। কোনো কথা ইসলামের সাধারণ শিক্ষার সঙ্গে মিললেও, সেটি রাসূলের নামে নির্দিষ্ট হাদিস হিসেবে প্রমাণিত হতে হবে। এই সতর্কতাই হাদিস যাচাইয়ের মূল শিক্ষা।"},"teachings":["পরিষ্কার-পরিচ্ছন্নতা গুরুত্বপূর্ণ, কিন্তু এই নির্দিষ্ট বর্ণনা জাল।","সনদে জালকারী থাকলে হাদিস গ্রহণযোগ্য নয়।","সাধারণ ইসলামি শিক্ষার সঙ্গে মিল থাকলেই কোনো বাক্য হাদিস হয় না।","ইবাদত ও তাহারাত বিষয়ে নির্ভরযোগ্য দলীল ব্যবহার করা উচিত।"],"related_hadiths":[{"id":"223","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"1","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"61","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"}]}</t>
         </is>
       </c>
       <c r="E54" s="4" t="n"/>

</xml_diff>